<commit_message>
Added README.md File for Project
</commit_message>
<xml_diff>
--- a/Excels/Customers.xlsx
+++ b/Excels/Customers.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="X12" s="0" t="inlineStr">
         <is>
-          <t>101694200.00</t>
+          <t>101890200.00</t>
         </is>
       </c>
       <c r="Z12" s="0" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="X22" s="0" t="inlineStr">
         <is>
-          <t>13081200.00</t>
+          <t>13237600.00</t>
         </is>
       </c>
       <c r="Z22" s="0" t="inlineStr">
@@ -5775,12 +5775,7 @@
     <row r="176" spans="1:29">
       <c r="A176" s="0" t="inlineStr">
         <is>
-          <t>HASIYA</t>
-        </is>
-      </c>
-      <c r="B176" s="0" t="inlineStr">
-        <is>
-          <t> TURAKI - ABK</t>
+          <t>HAJ SUMAYYA</t>
         </is>
       </c>
       <c r="R176" s="0" t="inlineStr">
@@ -5805,19 +5800,14 @@
       </c>
       <c r="AC176" s="0" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>324</t>
         </is>
       </c>
     </row>
     <row r="177" spans="1:29">
       <c r="A177" s="0" t="inlineStr">
         <is>
-          <t>HAJ SAMIRA</t>
-        </is>
-      </c>
-      <c r="B177" s="0" t="inlineStr">
-        <is>
-          <t>- ABK</t>
+          <t>ZAHRA LATEST</t>
         </is>
       </c>
       <c r="R177" s="0" t="inlineStr">
@@ -5827,7 +5817,7 @@
       </c>
       <c r="X177" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>180000.00</t>
         </is>
       </c>
       <c r="Z177" s="0" t="inlineStr">
@@ -5842,19 +5832,19 @@
       </c>
       <c r="AC177" s="0" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>325</t>
         </is>
       </c>
     </row>
     <row r="178" spans="1:29">
       <c r="A178" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>HASIYA</t>
         </is>
       </c>
       <c r="B178" s="0" t="inlineStr">
         <is>
-          <t>ABANA</t>
+          <t> TURAKI - ABK</t>
         </is>
       </c>
       <c r="R178" s="0" t="inlineStr">
@@ -5864,7 +5854,7 @@
       </c>
       <c r="X178" s="0" t="inlineStr">
         <is>
-          <t>251500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z178" s="0" t="inlineStr">
@@ -5879,19 +5869,19 @@
       </c>
       <c r="AC178" s="0" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>222</t>
         </is>
       </c>
     </row>
     <row r="179" spans="1:29">
       <c r="A179" s="0" t="inlineStr">
         <is>
-          <t>KHADIJA</t>
+          <t>HAJ SAMIRA</t>
         </is>
       </c>
       <c r="B179" s="0" t="inlineStr">
         <is>
-          <t>ABDULQADIR</t>
+          <t>- ABK</t>
         </is>
       </c>
       <c r="R179" s="0" t="inlineStr">
@@ -5916,19 +5906,19 @@
       </c>
       <c r="AC179" s="0" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="180" spans="1:29">
       <c r="A180" s="0" t="inlineStr">
         <is>
-          <t>NURIYYAH</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B180" s="0" t="inlineStr">
         <is>
-          <t>AHMAD</t>
+          <t>ABANA</t>
         </is>
       </c>
       <c r="R180" s="0" t="inlineStr">
@@ -5938,7 +5928,7 @@
       </c>
       <c r="X180" s="0" t="inlineStr">
         <is>
-          <t>283000.00</t>
+          <t>251500.00</t>
         </is>
       </c>
       <c r="Z180" s="0" t="inlineStr">
@@ -5953,19 +5943,19 @@
       </c>
       <c r="AC180" s="0" t="inlineStr">
         <is>
-          <t>112</t>
+          <t>281</t>
         </is>
       </c>
     </row>
     <row r="181" spans="1:29">
       <c r="A181" s="0" t="inlineStr">
         <is>
-          <t>HAJ MAIMUNA</t>
+          <t>KHADIJA</t>
         </is>
       </c>
       <c r="B181" s="0" t="inlineStr">
         <is>
-          <t>AHMAD</t>
+          <t>ABDULQADIR</t>
         </is>
       </c>
       <c r="R181" s="0" t="inlineStr">
@@ -5990,19 +5980,19 @@
       </c>
       <c r="AC181" s="0" t="inlineStr">
         <is>
-          <t>279</t>
+          <t>191</t>
         </is>
       </c>
     </row>
     <row r="182" spans="1:29">
       <c r="A182" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>NURIYYAH</t>
         </is>
       </c>
       <c r="B182" s="0" t="inlineStr">
         <is>
-          <t>AIRFORCE</t>
+          <t>AHMAD</t>
         </is>
       </c>
       <c r="R182" s="0" t="inlineStr">
@@ -6012,7 +6002,7 @@
       </c>
       <c r="X182" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>283000.00</t>
         </is>
       </c>
       <c r="Z182" s="0" t="inlineStr">
@@ -6027,19 +6017,19 @@
       </c>
       <c r="AC182" s="0" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>112</t>
         </is>
       </c>
     </row>
     <row r="183" spans="1:29">
       <c r="A183" s="0" t="inlineStr">
         <is>
-          <t>SADIYA</t>
+          <t>HAJ MAIMUNA</t>
         </is>
       </c>
       <c r="B183" s="0" t="inlineStr">
         <is>
-          <t>ALA</t>
+          <t>AHMAD</t>
         </is>
       </c>
       <c r="R183" s="0" t="inlineStr">
@@ -6064,19 +6054,19 @@
       </c>
       <c r="AC183" s="0" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>279</t>
         </is>
       </c>
     </row>
     <row r="184" spans="1:29">
       <c r="A184" s="0" t="inlineStr">
         <is>
-          <t>HAJ ZALIHATU</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B184" s="0" t="inlineStr">
         <is>
-          <t>ALERU</t>
+          <t>AIRFORCE</t>
         </is>
       </c>
       <c r="R184" s="0" t="inlineStr">
@@ -6101,19 +6091,19 @@
       </c>
       <c r="AC184" s="0" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>111</t>
         </is>
       </c>
     </row>
     <row r="185" spans="1:29">
       <c r="A185" s="0" t="inlineStr">
         <is>
-          <t>MA'U</t>
+          <t>SADIYA</t>
         </is>
       </c>
       <c r="B185" s="0" t="inlineStr">
         <is>
-          <t>ALHASSAN</t>
+          <t>ALA</t>
         </is>
       </c>
       <c r="R185" s="0" t="inlineStr">
@@ -6123,7 +6113,7 @@
       </c>
       <c r="X185" s="0" t="inlineStr">
         <is>
-          <t>48000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z185" s="0" t="inlineStr">
@@ -6138,19 +6128,19 @@
       </c>
       <c r="AC185" s="0" t="inlineStr">
         <is>
-          <t>183</t>
+          <t>126</t>
         </is>
       </c>
     </row>
     <row r="186" spans="1:29">
       <c r="A186" s="0" t="inlineStr">
         <is>
-          <t>BILKISU</t>
+          <t>HAJ ZALIHATU</t>
         </is>
       </c>
       <c r="B186" s="0" t="inlineStr">
         <is>
-          <t>ALI BALA</t>
+          <t>ALERU</t>
         </is>
       </c>
       <c r="R186" s="0" t="inlineStr">
@@ -6160,7 +6150,7 @@
       </c>
       <c r="X186" s="0" t="inlineStr">
         <is>
-          <t>842000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z186" s="0" t="inlineStr">
@@ -6175,19 +6165,19 @@
       </c>
       <c r="AC186" s="0" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>287</t>
         </is>
       </c>
     </row>
     <row r="187" spans="1:29">
       <c r="A187" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>MA'U</t>
         </is>
       </c>
       <c r="B187" s="0" t="inlineStr">
         <is>
-          <t>AMATU</t>
+          <t>ALHASSAN</t>
         </is>
       </c>
       <c r="R187" s="0" t="inlineStr">
@@ -6197,7 +6187,7 @@
       </c>
       <c r="X187" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>48000.00</t>
         </is>
       </c>
       <c r="Z187" s="0" t="inlineStr">
@@ -6212,7 +6202,7 @@
       </c>
       <c r="AC187" s="0" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>183</t>
         </is>
       </c>
     </row>
@@ -6224,7 +6214,7 @@
       </c>
       <c r="B188" s="0" t="inlineStr">
         <is>
-          <t>AMMANI</t>
+          <t>ALI BALA</t>
         </is>
       </c>
       <c r="R188" s="0" t="inlineStr">
@@ -6234,7 +6224,7 @@
       </c>
       <c r="X188" s="0" t="inlineStr">
         <is>
-          <t>65000.00</t>
+          <t>842000.00</t>
         </is>
       </c>
       <c r="Z188" s="0" t="inlineStr">
@@ -6249,19 +6239,19 @@
       </c>
       <c r="AC188" s="0" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>79</t>
         </is>
       </c>
     </row>
     <row r="189" spans="1:29">
       <c r="A189" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B189" s="0" t="inlineStr">
         <is>
-          <t>AMMI</t>
+          <t>AMATU</t>
         </is>
       </c>
       <c r="R189" s="0" t="inlineStr">
@@ -6271,7 +6261,7 @@
       </c>
       <c r="X189" s="0" t="inlineStr">
         <is>
-          <t>128000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z189" s="0" t="inlineStr">
@@ -6286,19 +6276,19 @@
       </c>
       <c r="AC189" s="0" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>134</t>
         </is>
       </c>
     </row>
     <row r="190" spans="1:29">
       <c r="A190" s="0" t="inlineStr">
         <is>
-          <t>SAMIRA</t>
+          <t>BILKISU</t>
         </is>
       </c>
       <c r="B190" s="0" t="inlineStr">
         <is>
-          <t>ARC</t>
+          <t>AMMANI</t>
         </is>
       </c>
       <c r="R190" s="0" t="inlineStr">
@@ -6308,7 +6298,7 @@
       </c>
       <c r="X190" s="0" t="inlineStr">
         <is>
-          <t>166500.00</t>
+          <t>65000.00</t>
         </is>
       </c>
       <c r="Z190" s="0" t="inlineStr">
@@ -6323,19 +6313,19 @@
       </c>
       <c r="AC190" s="0" t="inlineStr">
         <is>
-          <t>187</t>
+          <t>189</t>
         </is>
       </c>
     </row>
     <row r="191" spans="1:29">
       <c r="A191" s="0" t="inlineStr">
         <is>
-          <t>HAJ HAUWA</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B191" s="0" t="inlineStr">
         <is>
-          <t>AWAISU</t>
+          <t>AMMI</t>
         </is>
       </c>
       <c r="R191" s="0" t="inlineStr">
@@ -6345,7 +6335,7 @@
       </c>
       <c r="X191" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>128000.00</t>
         </is>
       </c>
       <c r="Z191" s="0" t="inlineStr">
@@ -6360,19 +6350,19 @@
       </c>
       <c r="AC191" s="0" t="inlineStr">
         <is>
-          <t>284</t>
+          <t>130</t>
         </is>
       </c>
     </row>
     <row r="192" spans="1:29">
       <c r="A192" s="0" t="inlineStr">
         <is>
-          <t>ZAINAB</t>
+          <t>SAMIRA</t>
         </is>
       </c>
       <c r="B192" s="0" t="inlineStr">
         <is>
-          <t>AZARE</t>
+          <t>ARC</t>
         </is>
       </c>
       <c r="R192" s="0" t="inlineStr">
@@ -6382,7 +6372,7 @@
       </c>
       <c r="X192" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>166500.00</t>
         </is>
       </c>
       <c r="Z192" s="0" t="inlineStr">
@@ -6397,19 +6387,19 @@
       </c>
       <c r="AC192" s="0" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>187</t>
         </is>
       </c>
     </row>
     <row r="193" spans="1:29">
       <c r="A193" s="0" t="inlineStr">
         <is>
-          <t>RAHAMA</t>
+          <t>HAJ HAUWA</t>
         </is>
       </c>
       <c r="B193" s="0" t="inlineStr">
         <is>
-          <t>BAMALLI</t>
+          <t>AWAISU</t>
         </is>
       </c>
       <c r="R193" s="0" t="inlineStr">
@@ -6434,19 +6424,19 @@
       </c>
       <c r="AC193" s="0" t="inlineStr">
         <is>
-          <t>265</t>
+          <t>284</t>
         </is>
       </c>
     </row>
     <row r="194" spans="1:29">
       <c r="A194" s="0" t="inlineStr">
         <is>
-          <t>NAFISA</t>
+          <t>ZAINAB</t>
         </is>
       </c>
       <c r="B194" s="0" t="inlineStr">
         <is>
-          <t>BARAU</t>
+          <t>AZARE</t>
         </is>
       </c>
       <c r="R194" s="0" t="inlineStr">
@@ -6471,19 +6461,19 @@
       </c>
       <c r="AC194" s="0" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>144</t>
         </is>
       </c>
     </row>
     <row r="195" spans="1:29">
       <c r="A195" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>RAHAMA</t>
         </is>
       </c>
       <c r="B195" s="0" t="inlineStr">
         <is>
-          <t>BAUCHI</t>
+          <t>BAMALLI</t>
         </is>
       </c>
       <c r="R195" s="0" t="inlineStr">
@@ -6493,7 +6483,7 @@
       </c>
       <c r="X195" s="0" t="inlineStr">
         <is>
-          <t>162000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z195" s="0" t="inlineStr">
@@ -6508,19 +6498,19 @@
       </c>
       <c r="AC195" s="0" t="inlineStr">
         <is>
-          <t>314</t>
+          <t>265</t>
         </is>
       </c>
     </row>
     <row r="196" spans="1:29">
       <c r="A196" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>NAFISA</t>
         </is>
       </c>
       <c r="B196" s="0" t="inlineStr">
         <is>
-          <t>BAWA ROAD</t>
+          <t>BARAU</t>
         </is>
       </c>
       <c r="R196" s="0" t="inlineStr">
@@ -6530,7 +6520,7 @@
       </c>
       <c r="X196" s="0" t="inlineStr">
         <is>
-          <t>853000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z196" s="0" t="inlineStr">
@@ -6545,19 +6535,19 @@
       </c>
       <c r="AC196" s="0" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>148</t>
         </is>
       </c>
     </row>
     <row r="197" spans="1:29">
       <c r="A197" s="0" t="inlineStr">
         <is>
-          <t>HAUWA</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B197" s="0" t="inlineStr">
         <is>
-          <t>BELLO</t>
+          <t>BAUCHI</t>
         </is>
       </c>
       <c r="R197" s="0" t="inlineStr">
@@ -6567,7 +6557,7 @@
       </c>
       <c r="X197" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>162000.00</t>
         </is>
       </c>
       <c r="Z197" s="0" t="inlineStr">
@@ -6582,19 +6572,19 @@
       </c>
       <c r="AC197" s="0" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>314</t>
         </is>
       </c>
     </row>
     <row r="198" spans="1:29">
       <c r="A198" s="0" t="inlineStr">
         <is>
-          <t>FARIDA</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B198" s="0" t="inlineStr">
         <is>
-          <t>BINDAWA</t>
+          <t>BAWA ROAD</t>
         </is>
       </c>
       <c r="R198" s="0" t="inlineStr">
@@ -6604,7 +6594,7 @@
       </c>
       <c r="X198" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1258000.00</t>
         </is>
       </c>
       <c r="Z198" s="0" t="inlineStr">
@@ -6619,19 +6609,19 @@
       </c>
       <c r="AC198" s="0" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>113</t>
         </is>
       </c>
     </row>
     <row r="199" spans="1:29">
       <c r="A199" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>HAUWA</t>
         </is>
       </c>
       <c r="B199" s="0" t="inlineStr">
         <is>
-          <t>BINDAWA</t>
+          <t>BELLO</t>
         </is>
       </c>
       <c r="R199" s="0" t="inlineStr">
@@ -6641,7 +6631,7 @@
       </c>
       <c r="X199" s="0" t="inlineStr">
         <is>
-          <t>937000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z199" s="0" t="inlineStr">
@@ -6656,19 +6646,19 @@
       </c>
       <c r="AC199" s="0" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>125</t>
         </is>
       </c>
     </row>
     <row r="200" spans="1:29">
       <c r="A200" s="0" t="inlineStr">
         <is>
-          <t>MARIA</t>
+          <t>FARIDA</t>
         </is>
       </c>
       <c r="B200" s="0" t="inlineStr">
         <is>
-          <t>BOSE</t>
+          <t>BINDAWA</t>
         </is>
       </c>
       <c r="R200" s="0" t="inlineStr">
@@ -6693,19 +6683,19 @@
       </c>
       <c r="AC200" s="0" t="inlineStr">
         <is>
-          <t>295</t>
+          <t>93</t>
         </is>
       </c>
     </row>
     <row r="201" spans="1:29">
       <c r="A201" s="0" t="inlineStr">
         <is>
-          <t>HAJ MARYAM</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B201" s="0" t="inlineStr">
         <is>
-          <t>BUHARI</t>
+          <t>BINDAWA</t>
         </is>
       </c>
       <c r="R201" s="0" t="inlineStr">
@@ -6715,7 +6705,7 @@
       </c>
       <c r="X201" s="0" t="inlineStr">
         <is>
-          <t>115000.00</t>
+          <t>937000.00</t>
         </is>
       </c>
       <c r="Z201" s="0" t="inlineStr">
@@ -6730,19 +6720,19 @@
       </c>
       <c r="AC201" s="0" t="inlineStr">
         <is>
-          <t>312</t>
+          <t>123</t>
         </is>
       </c>
     </row>
     <row r="202" spans="1:29">
       <c r="A202" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>MARIA</t>
         </is>
       </c>
       <c r="B202" s="0" t="inlineStr">
         <is>
-          <t>BULAMA</t>
+          <t>BOSE</t>
         </is>
       </c>
       <c r="R202" s="0" t="inlineStr">
@@ -6767,19 +6757,19 @@
       </c>
       <c r="AC202" s="0" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>295</t>
         </is>
       </c>
     </row>
     <row r="203" spans="1:29">
       <c r="A203" s="0" t="inlineStr">
         <is>
-          <t>KHADIJA</t>
+          <t>HAJ MARYAM</t>
         </is>
       </c>
       <c r="B203" s="0" t="inlineStr">
         <is>
-          <t>CHIROMA</t>
+          <t>BUHARI</t>
         </is>
       </c>
       <c r="R203" s="0" t="inlineStr">
@@ -6789,7 +6779,7 @@
       </c>
       <c r="X203" s="0" t="inlineStr">
         <is>
-          <t>8500.00</t>
+          <t>115000.00</t>
         </is>
       </c>
       <c r="Z203" s="0" t="inlineStr">
@@ -6804,19 +6794,19 @@
       </c>
       <c r="AC203" s="0" t="inlineStr">
         <is>
-          <t>184</t>
+          <t>312</t>
         </is>
       </c>
     </row>
     <row r="204" spans="1:29">
       <c r="A204" s="0" t="inlineStr">
         <is>
-          <t>ZAHRA</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B204" s="0" t="inlineStr">
         <is>
-          <t>COLLECTION</t>
+          <t>BULAMA</t>
         </is>
       </c>
       <c r="R204" s="0" t="inlineStr">
@@ -6826,7 +6816,7 @@
       </c>
       <c r="X204" s="0" t="inlineStr">
         <is>
-          <t>171000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z204" s="0" t="inlineStr">
@@ -6841,19 +6831,19 @@
       </c>
       <c r="AC204" s="0" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>253</t>
         </is>
       </c>
     </row>
     <row r="205" spans="1:29">
       <c r="A205" s="0" t="inlineStr">
         <is>
-          <t>MAIMUNA</t>
+          <t>KHADIJA</t>
         </is>
       </c>
       <c r="B205" s="0" t="inlineStr">
         <is>
-          <t>CUSTOM</t>
+          <t>CHIROMA</t>
         </is>
       </c>
       <c r="R205" s="0" t="inlineStr">
@@ -6863,7 +6853,7 @@
       </c>
       <c r="X205" s="0" t="inlineStr">
         <is>
-          <t>20000.00</t>
+          <t>8500.00</t>
         </is>
       </c>
       <c r="Z205" s="0" t="inlineStr">
@@ -6878,19 +6868,19 @@
       </c>
       <c r="AC205" s="0" t="inlineStr">
         <is>
-          <t>227</t>
+          <t>184</t>
         </is>
       </c>
     </row>
     <row r="206" spans="1:29">
       <c r="A206" s="0" t="inlineStr">
         <is>
-          <t>MAMAN AISHA</t>
+          <t>ZAHRA</t>
         </is>
       </c>
       <c r="B206" s="0" t="inlineStr">
         <is>
-          <t>DAHIRU</t>
+          <t>COLLECTION</t>
         </is>
       </c>
       <c r="R206" s="0" t="inlineStr">
@@ -6900,7 +6890,7 @@
       </c>
       <c r="X206" s="0" t="inlineStr">
         <is>
-          <t>75000.00</t>
+          <t>171000.00</t>
         </is>
       </c>
       <c r="Z206" s="0" t="inlineStr">
@@ -6915,7 +6905,7 @@
       </c>
       <c r="AC206" s="0" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>136</t>
         </is>
       </c>
     </row>
@@ -6927,7 +6917,7 @@
       </c>
       <c r="B207" s="0" t="inlineStr">
         <is>
-          <t>DAN ASABE</t>
+          <t>CUSTOM</t>
         </is>
       </c>
       <c r="R207" s="0" t="inlineStr">
@@ -6937,7 +6927,7 @@
       </c>
       <c r="X207" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>20000.00</t>
         </is>
       </c>
       <c r="Z207" s="0" t="inlineStr">
@@ -6952,19 +6942,19 @@
       </c>
       <c r="AC207" s="0" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>227</t>
         </is>
       </c>
     </row>
     <row r="208" spans="1:29">
       <c r="A208" s="0" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>MAMAN AISHA</t>
         </is>
       </c>
       <c r="B208" s="0" t="inlineStr">
         <is>
-          <t>DORAYI</t>
+          <t>DAHIRU</t>
         </is>
       </c>
       <c r="R208" s="0" t="inlineStr">
@@ -6974,7 +6964,7 @@
       </c>
       <c r="X208" s="0" t="inlineStr">
         <is>
-          <t>3667000.00</t>
+          <t>75000.00</t>
         </is>
       </c>
       <c r="Z208" s="0" t="inlineStr">
@@ -6989,19 +6979,19 @@
       </c>
       <c r="AC208" s="0" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>194</t>
         </is>
       </c>
     </row>
     <row r="209" spans="1:29">
       <c r="A209" s="0" t="inlineStr">
         <is>
-          <t>UMMI</t>
+          <t>MAIMUNA</t>
         </is>
       </c>
       <c r="B209" s="0" t="inlineStr">
         <is>
-          <t>FAB SHOP</t>
+          <t>DAN ASABE</t>
         </is>
       </c>
       <c r="R209" s="0" t="inlineStr">
@@ -7011,7 +7001,7 @@
       </c>
       <c r="X209" s="0" t="inlineStr">
         <is>
-          <t>790000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z209" s="0" t="inlineStr">
@@ -7026,19 +7016,19 @@
       </c>
       <c r="AC209" s="0" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>169</t>
         </is>
       </c>
     </row>
     <row r="210" spans="1:29">
       <c r="A210" s="0" t="inlineStr">
         <is>
-          <t>JAMI</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="B210" s="0" t="inlineStr">
         <is>
-          <t>FABRICS</t>
+          <t>DORAYI</t>
         </is>
       </c>
       <c r="R210" s="0" t="inlineStr">
@@ -7048,7 +7038,7 @@
       </c>
       <c r="X210" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>3667000.00</t>
         </is>
       </c>
       <c r="Z210" s="0" t="inlineStr">
@@ -7063,19 +7053,19 @@
       </c>
       <c r="AC210" s="0" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>172</t>
         </is>
       </c>
     </row>
     <row r="211" spans="1:29">
       <c r="A211" s="0" t="inlineStr">
         <is>
-          <t>SAMIRA</t>
+          <t>UMMI</t>
         </is>
       </c>
       <c r="B211" s="0" t="inlineStr">
         <is>
-          <t>FAGGE</t>
+          <t>FAB SHOP</t>
         </is>
       </c>
       <c r="R211" s="0" t="inlineStr">
@@ -7085,7 +7075,7 @@
       </c>
       <c r="X211" s="0" t="inlineStr">
         <is>
-          <t>119000.00</t>
+          <t>790000.00</t>
         </is>
       </c>
       <c r="Z211" s="0" t="inlineStr">
@@ -7100,19 +7090,19 @@
       </c>
       <c r="AC211" s="0" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>100</t>
         </is>
       </c>
     </row>
     <row r="212" spans="1:29">
       <c r="A212" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>JAMI</t>
         </is>
       </c>
       <c r="B212" s="0" t="inlineStr">
         <is>
-          <t>FAGGO</t>
+          <t>FABRICS</t>
         </is>
       </c>
       <c r="R212" s="0" t="inlineStr">
@@ -7122,7 +7112,7 @@
       </c>
       <c r="X212" s="0" t="inlineStr">
         <is>
-          <t>45000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z212" s="0" t="inlineStr">
@@ -7137,19 +7127,19 @@
       </c>
       <c r="AC212" s="0" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>142</t>
         </is>
       </c>
     </row>
     <row r="213" spans="1:29">
       <c r="A213" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>SAMIRA</t>
         </is>
       </c>
       <c r="B213" s="0" t="inlineStr">
         <is>
-          <t>FAROUQ</t>
+          <t>FAGGE</t>
         </is>
       </c>
       <c r="R213" s="0" t="inlineStr">
@@ -7159,7 +7149,7 @@
       </c>
       <c r="X213" s="0" t="inlineStr">
         <is>
-          <t>290000.00</t>
+          <t>119000.00</t>
         </is>
       </c>
       <c r="Z213" s="0" t="inlineStr">
@@ -7174,19 +7164,19 @@
       </c>
       <c r="AC213" s="0" t="inlineStr">
         <is>
-          <t>212</t>
+          <t>89</t>
         </is>
       </c>
     </row>
     <row r="214" spans="1:29">
       <c r="A214" s="0" t="inlineStr">
         <is>
-          <t>MUSA</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B214" s="0" t="inlineStr">
         <is>
-          <t>GARBA</t>
+          <t>FAGGO</t>
         </is>
       </c>
       <c r="R214" s="0" t="inlineStr">
@@ -7196,7 +7186,7 @@
       </c>
       <c r="X214" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>45000.00</t>
         </is>
       </c>
       <c r="Z214" s="0" t="inlineStr">
@@ -7211,19 +7201,19 @@
       </c>
       <c r="AC214" s="0" t="inlineStr">
         <is>
-          <t>214</t>
+          <t>204</t>
         </is>
       </c>
     </row>
     <row r="215" spans="1:29">
       <c r="A215" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B215" s="0" t="inlineStr">
         <is>
-          <t>GOMBE</t>
+          <t>FAROUQ</t>
         </is>
       </c>
       <c r="R215" s="0" t="inlineStr">
@@ -7233,7 +7223,7 @@
       </c>
       <c r="X215" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>290000.00</t>
         </is>
       </c>
       <c r="Z215" s="0" t="inlineStr">
@@ -7248,19 +7238,19 @@
       </c>
       <c r="AC215" s="0" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>212</t>
         </is>
       </c>
     </row>
     <row r="216" spans="1:29">
       <c r="A216" s="0" t="inlineStr">
         <is>
-          <t>MOMY</t>
+          <t>MUSA</t>
         </is>
       </c>
       <c r="B216" s="0" t="inlineStr">
         <is>
-          <t>GOMBE</t>
+          <t>GARBA</t>
         </is>
       </c>
       <c r="R216" s="0" t="inlineStr">
@@ -7270,7 +7260,7 @@
       </c>
       <c r="X216" s="0" t="inlineStr">
         <is>
-          <t>245000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z216" s="0" t="inlineStr">
@@ -7285,14 +7275,14 @@
       </c>
       <c r="AC216" s="0" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>214</t>
         </is>
       </c>
     </row>
     <row r="217" spans="1:29">
       <c r="A217" s="0" t="inlineStr">
         <is>
-          <t>HAJ HAJARA</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B217" s="0" t="inlineStr">
@@ -7322,19 +7312,19 @@
       </c>
       <c r="AC217" s="0" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>103</t>
         </is>
       </c>
     </row>
     <row r="218" spans="1:29">
       <c r="A218" s="0" t="inlineStr">
         <is>
-          <t>SAMIRA</t>
+          <t>MOMY</t>
         </is>
       </c>
       <c r="B218" s="0" t="inlineStr">
         <is>
-          <t>GUNU</t>
+          <t>GOMBE</t>
         </is>
       </c>
       <c r="R218" s="0" t="inlineStr">
@@ -7344,7 +7334,7 @@
       </c>
       <c r="X218" s="0" t="inlineStr">
         <is>
-          <t>24000.00</t>
+          <t>245000.00</t>
         </is>
       </c>
       <c r="Z218" s="0" t="inlineStr">
@@ -7359,19 +7349,19 @@
       </c>
       <c r="AC218" s="0" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>143</t>
         </is>
       </c>
     </row>
     <row r="219" spans="1:29">
       <c r="A219" s="0" t="inlineStr">
         <is>
-          <t>BILKISU</t>
+          <t>HAJ HAJARA</t>
         </is>
       </c>
       <c r="B219" s="0" t="inlineStr">
         <is>
-          <t>GWALABE</t>
+          <t>GOMBE</t>
         </is>
       </c>
       <c r="R219" s="0" t="inlineStr">
@@ -7396,19 +7386,19 @@
       </c>
       <c r="AC219" s="0" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>209</t>
         </is>
       </c>
     </row>
     <row r="220" spans="1:29">
       <c r="A220" s="0" t="inlineStr">
         <is>
-          <t>HAUWA</t>
+          <t>SAMIRA</t>
         </is>
       </c>
       <c r="B220" s="0" t="inlineStr">
         <is>
-          <t>GWALABE</t>
+          <t>GUNU</t>
         </is>
       </c>
       <c r="R220" s="0" t="inlineStr">
@@ -7418,7 +7408,7 @@
       </c>
       <c r="X220" s="0" t="inlineStr">
         <is>
-          <t>60000.00</t>
+          <t>24000.00</t>
         </is>
       </c>
       <c r="Z220" s="0" t="inlineStr">
@@ -7433,19 +7423,19 @@
       </c>
       <c r="AC220" s="0" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>159</t>
         </is>
       </c>
     </row>
     <row r="221" spans="1:29">
       <c r="A221" s="0" t="inlineStr">
         <is>
-          <t>MAMA</t>
+          <t>BILKISU</t>
         </is>
       </c>
       <c r="B221" s="0" t="inlineStr">
         <is>
-          <t>H &amp; M</t>
+          <t>GWALABE</t>
         </is>
       </c>
       <c r="R221" s="0" t="inlineStr">
@@ -7470,19 +7460,19 @@
       </c>
       <c r="AC221" s="0" t="inlineStr">
         <is>
-          <t>163</t>
+          <t>101</t>
         </is>
       </c>
     </row>
     <row r="222" spans="1:29">
       <c r="A222" s="0" t="inlineStr">
         <is>
-          <t>HAJ HAUWA</t>
+          <t>HAUWA</t>
         </is>
       </c>
       <c r="B222" s="0" t="inlineStr">
         <is>
-          <t>HABIB</t>
+          <t>GWALABE</t>
         </is>
       </c>
       <c r="R222" s="0" t="inlineStr">
@@ -7492,7 +7482,7 @@
       </c>
       <c r="X222" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>60000.00</t>
         </is>
       </c>
       <c r="Z222" s="0" t="inlineStr">
@@ -7507,24 +7497,19 @@
       </c>
       <c r="AC222" s="0" t="inlineStr">
         <is>
-          <t>264</t>
+          <t>321</t>
         </is>
       </c>
     </row>
     <row r="223" spans="1:29">
       <c r="A223" s="0" t="inlineStr">
         <is>
-          <t>KAMILA</t>
+          <t>MAMA</t>
         </is>
       </c>
       <c r="B223" s="0" t="inlineStr">
         <is>
-          <t>HADEJA</t>
-        </is>
-      </c>
-      <c r="D223" s="0" t="inlineStr">
-        <is>
-          <t>+2347054680033</t>
+          <t>H &amp; M</t>
         </is>
       </c>
       <c r="R223" s="0" t="inlineStr">
@@ -7549,19 +7534,19 @@
       </c>
       <c r="AC223" s="0" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>163</t>
         </is>
       </c>
     </row>
     <row r="224" spans="1:29">
       <c r="A224" s="0" t="inlineStr">
         <is>
-          <t>HAJ RAKIYA</t>
+          <t>HAJ HAUWA</t>
         </is>
       </c>
       <c r="B224" s="0" t="inlineStr">
         <is>
-          <t>HAMZA</t>
+          <t>HABIB</t>
         </is>
       </c>
       <c r="R224" s="0" t="inlineStr">
@@ -7586,19 +7571,24 @@
       </c>
       <c r="AC224" s="0" t="inlineStr">
         <is>
-          <t>291</t>
+          <t>264</t>
         </is>
       </c>
     </row>
     <row r="225" spans="1:29">
       <c r="A225" s="0" t="inlineStr">
         <is>
-          <t>HAJ HAFSAT</t>
+          <t>KAMILA</t>
         </is>
       </c>
       <c r="B225" s="0" t="inlineStr">
         <is>
-          <t>HAMZA</t>
+          <t>HADEJA</t>
+        </is>
+      </c>
+      <c r="D225" s="0" t="inlineStr">
+        <is>
+          <t>+2347054680033</t>
         </is>
       </c>
       <c r="R225" s="0" t="inlineStr">
@@ -7623,19 +7613,19 @@
       </c>
       <c r="AC225" s="0" t="inlineStr">
         <is>
-          <t>306</t>
+          <t>199</t>
         </is>
       </c>
     </row>
     <row r="226" spans="1:29">
       <c r="A226" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>HAJ RAKIYA</t>
         </is>
       </c>
       <c r="B226" s="0" t="inlineStr">
         <is>
-          <t>HANIFA GOMBE</t>
+          <t>HAMZA</t>
         </is>
       </c>
       <c r="R226" s="0" t="inlineStr">
@@ -7645,7 +7635,7 @@
       </c>
       <c r="X226" s="0" t="inlineStr">
         <is>
-          <t>279000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z226" s="0" t="inlineStr">
@@ -7660,19 +7650,19 @@
       </c>
       <c r="AC226" s="0" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>291</t>
         </is>
       </c>
     </row>
     <row r="227" spans="1:29">
       <c r="A227" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>HAJ HAFSAT</t>
         </is>
       </c>
       <c r="B227" s="0" t="inlineStr">
         <is>
-          <t>HISHAM - ABK</t>
+          <t>HAMZA</t>
         </is>
       </c>
       <c r="R227" s="0" t="inlineStr">
@@ -7697,19 +7687,19 @@
       </c>
       <c r="AC227" s="0" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>306</t>
         </is>
       </c>
     </row>
     <row r="228" spans="1:29">
       <c r="A228" s="0" t="inlineStr">
         <is>
-          <t>MALAMA</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B228" s="0" t="inlineStr">
         <is>
-          <t>HUSSAINA</t>
+          <t>HANIFA GOMBE</t>
         </is>
       </c>
       <c r="R228" s="0" t="inlineStr">
@@ -7719,7 +7709,7 @@
       </c>
       <c r="X228" s="0" t="inlineStr">
         <is>
-          <t>590000.00</t>
+          <t>279000.00</t>
         </is>
       </c>
       <c r="Z228" s="0" t="inlineStr">
@@ -7734,19 +7724,19 @@
       </c>
       <c r="AC228" s="0" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>120</t>
         </is>
       </c>
     </row>
     <row r="229" spans="1:29">
       <c r="A229" s="0" t="inlineStr">
         <is>
-          <t>SA'ADATU </t>
+          <t>MAIMUNA</t>
         </is>
       </c>
       <c r="B229" s="0" t="inlineStr">
         <is>
-          <t>HUSSAINI</t>
+          <t>HASSAN</t>
         </is>
       </c>
       <c r="R229" s="0" t="inlineStr">
@@ -7771,19 +7761,19 @@
       </c>
       <c r="AC229" s="0" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>323</t>
         </is>
       </c>
     </row>
     <row r="230" spans="1:29">
       <c r="A230" s="0" t="inlineStr">
         <is>
-          <t>UMRATU</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B230" s="0" t="inlineStr">
         <is>
-          <t>HUSSAINI</t>
+          <t>HISHAM - ABK</t>
         </is>
       </c>
       <c r="R230" s="0" t="inlineStr">
@@ -7808,19 +7798,19 @@
       </c>
       <c r="AC230" s="0" t="inlineStr">
         <is>
-          <t>322</t>
+          <t>215</t>
         </is>
       </c>
     </row>
     <row r="231" spans="1:29">
       <c r="A231" s="0" t="inlineStr">
         <is>
-          <t>FARIDA </t>
+          <t>MALAMA</t>
         </is>
       </c>
       <c r="B231" s="0" t="inlineStr">
         <is>
-          <t>IBRAHIM</t>
+          <t>HUSSAINA</t>
         </is>
       </c>
       <c r="R231" s="0" t="inlineStr">
@@ -7830,7 +7820,7 @@
       </c>
       <c r="X231" s="0" t="inlineStr">
         <is>
-          <t>8500.00</t>
+          <t>590000.00</t>
         </is>
       </c>
       <c r="Z231" s="0" t="inlineStr">
@@ -7845,19 +7835,19 @@
       </c>
       <c r="AC231" s="0" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>141</t>
         </is>
       </c>
     </row>
     <row r="232" spans="1:29">
       <c r="A232" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>SA'ADATU </t>
         </is>
       </c>
       <c r="B232" s="0" t="inlineStr">
         <is>
-          <t>IBRAHIM</t>
+          <t>HUSSAINI</t>
         </is>
       </c>
       <c r="R232" s="0" t="inlineStr">
@@ -7867,7 +7857,7 @@
       </c>
       <c r="X232" s="0" t="inlineStr">
         <is>
-          <t>35000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z232" s="0" t="inlineStr">
@@ -7882,24 +7872,19 @@
       </c>
       <c r="AC232" s="0" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>131</t>
         </is>
       </c>
     </row>
     <row r="233" spans="1:29">
       <c r="A233" s="0" t="inlineStr">
         <is>
-          <t>SALISU</t>
+          <t>UMRATU</t>
         </is>
       </c>
       <c r="B233" s="0" t="inlineStr">
         <is>
-          <t>IDRIS</t>
-        </is>
-      </c>
-      <c r="D233" s="0" t="inlineStr">
-        <is>
-          <t>08184133063</t>
+          <t>HUSSAINI</t>
         </is>
       </c>
       <c r="R233" s="0" t="inlineStr">
@@ -7924,54 +7909,19 @@
       </c>
       <c r="AC233" s="0" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>322</t>
         </is>
       </c>
     </row>
     <row r="234" spans="1:29">
       <c r="A234" s="0" t="inlineStr">
         <is>
-          <t>Ibrahim BB</t>
+          <t>FARIDA </t>
         </is>
       </c>
       <c r="B234" s="0" t="inlineStr">
         <is>
-          <t>Jafar</t>
-        </is>
-      </c>
-      <c r="D234" s="0" t="inlineStr">
-        <is>
-          <t>08146595795</t>
-        </is>
-      </c>
-      <c r="J234" s="0" t="inlineStr">
-        <is>
-          <t>No 393 Rangi Quaters, Tudun Murtala, Nassarawa Kano</t>
-        </is>
-      </c>
-      <c r="L234" s="0" t="inlineStr">
-        <is>
-          <t>Kano</t>
-        </is>
-      </c>
-      <c r="M234" s="0" t="inlineStr">
-        <is>
-          <t>Kano</t>
-        </is>
-      </c>
-      <c r="N234" s="0" t="inlineStr">
-        <is>
-          <t>700281</t>
-        </is>
-      </c>
-      <c r="O234" s="0" t="inlineStr">
-        <is>
-          <t>Nigeria</t>
-        </is>
-      </c>
-      <c r="Q234" s="0" t="inlineStr">
-        <is>
-          <t>1522263645</t>
+          <t>IBRAHIM</t>
         </is>
       </c>
       <c r="R234" s="0" t="inlineStr">
@@ -7979,29 +7929,9 @@
           <t>y</t>
         </is>
       </c>
-      <c r="T234" s="0" t="inlineStr">
-        <is>
-          <t>Tahir General Merchant</t>
-        </is>
-      </c>
-      <c r="V234" s="0" t="inlineStr">
-        <is>
-          <t>High-value returning customer. Frequently purchases in bulk during seasonal periods. Offer priority support and notify early about new stock arrivals or discounts.</t>
-        </is>
-      </c>
-      <c r="W234" s="0" t="inlineStr">
-        <is>
-          <t>REGULAR customer, with less than 5% discounts on sales.</t>
-        </is>
-      </c>
       <c r="X234" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="Y234" s="0" t="inlineStr">
-        <is>
-          <t>50000000.00</t>
+          <t>8500.00</t>
         </is>
       </c>
       <c r="Z234" s="0" t="inlineStr">
@@ -8016,19 +7946,19 @@
       </c>
       <c r="AC234" s="0" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>224</t>
         </is>
       </c>
     </row>
     <row r="235" spans="1:29">
       <c r="A235" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B235" s="0" t="inlineStr">
         <is>
-          <t>JARMA</t>
+          <t>IBRAHIM</t>
         </is>
       </c>
       <c r="R235" s="0" t="inlineStr">
@@ -8038,7 +7968,7 @@
       </c>
       <c r="X235" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>35000.00</t>
         </is>
       </c>
       <c r="Z235" s="0" t="inlineStr">
@@ -8053,19 +7983,24 @@
       </c>
       <c r="AC235" s="0" t="inlineStr">
         <is>
-          <t>274</t>
+          <t>225</t>
         </is>
       </c>
     </row>
     <row r="236" spans="1:29">
       <c r="A236" s="0" t="inlineStr">
         <is>
-          <t>SUMAYYA</t>
+          <t>SALISU</t>
         </is>
       </c>
       <c r="B236" s="0" t="inlineStr">
         <is>
-          <t>JEGA</t>
+          <t>IDRIS</t>
+        </is>
+      </c>
+      <c r="D236" s="0" t="inlineStr">
+        <is>
+          <t>08184133063</t>
         </is>
       </c>
       <c r="R236" s="0" t="inlineStr">
@@ -8090,19 +8025,54 @@
       </c>
       <c r="AC236" s="0" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>17</t>
         </is>
       </c>
     </row>
     <row r="237" spans="1:29">
       <c r="A237" s="0" t="inlineStr">
         <is>
-          <t>PHIL</t>
+          <t>Ibrahim BB</t>
         </is>
       </c>
       <c r="B237" s="0" t="inlineStr">
         <is>
-          <t>JULIUS</t>
+          <t>Jafar</t>
+        </is>
+      </c>
+      <c r="D237" s="0" t="inlineStr">
+        <is>
+          <t>08146595795</t>
+        </is>
+      </c>
+      <c r="J237" s="0" t="inlineStr">
+        <is>
+          <t>No 393 Rangi Quaters, Tudun Murtala, Nassarawa Kano</t>
+        </is>
+      </c>
+      <c r="L237" s="0" t="inlineStr">
+        <is>
+          <t>Kano</t>
+        </is>
+      </c>
+      <c r="M237" s="0" t="inlineStr">
+        <is>
+          <t>Kano</t>
+        </is>
+      </c>
+      <c r="N237" s="0" t="inlineStr">
+        <is>
+          <t>700281</t>
+        </is>
+      </c>
+      <c r="O237" s="0" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="Q237" s="0" t="inlineStr">
+        <is>
+          <t>1522263645</t>
         </is>
       </c>
       <c r="R237" s="0" t="inlineStr">
@@ -8110,11 +8080,31 @@
           <t>y</t>
         </is>
       </c>
+      <c r="T237" s="0" t="inlineStr">
+        <is>
+          <t>Tahir General Merchant</t>
+        </is>
+      </c>
+      <c r="V237" s="0" t="inlineStr">
+        <is>
+          <t>High-value returning customer. Frequently purchases in bulk during seasonal periods. Offer priority support and notify early about new stock arrivals or discounts.</t>
+        </is>
+      </c>
+      <c r="W237" s="0" t="inlineStr">
+        <is>
+          <t>REGULAR customer, with less than 5% discounts on sales.</t>
+        </is>
+      </c>
       <c r="X237" s="0" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>
       </c>
+      <c r="Y237" s="0" t="inlineStr">
+        <is>
+          <t>50000000.00</t>
+        </is>
+      </c>
       <c r="Z237" s="0" t="inlineStr">
         <is>
           <t>n</t>
@@ -8127,19 +8117,19 @@
       </c>
       <c r="AC237" s="0" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>31</t>
         </is>
       </c>
     </row>
     <row r="238" spans="1:29">
       <c r="A238" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B238" s="0" t="inlineStr">
         <is>
-          <t>JUMARE</t>
+          <t>JARMA</t>
         </is>
       </c>
       <c r="R238" s="0" t="inlineStr">
@@ -8149,7 +8139,7 @@
       </c>
       <c r="X238" s="0" t="inlineStr">
         <is>
-          <t>269000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z238" s="0" t="inlineStr">
@@ -8164,29 +8154,19 @@
       </c>
       <c r="AC238" s="0" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>274</t>
         </is>
       </c>
     </row>
     <row r="239" spans="1:29">
       <c r="A239" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>SUMAYYA</t>
         </is>
       </c>
       <c r="B239" s="0" t="inlineStr">
         <is>
-          <t>KADUNA</t>
-        </is>
-      </c>
-      <c r="L239" s="0" t="inlineStr">
-        <is>
-          <t>KADUNA</t>
-        </is>
-      </c>
-      <c r="M239" s="0" t="inlineStr">
-        <is>
-          <t>KADUNA</t>
+          <t>JEGA</t>
         </is>
       </c>
       <c r="R239" s="0" t="inlineStr">
@@ -8196,7 +8176,7 @@
       </c>
       <c r="X239" s="0" t="inlineStr">
         <is>
-          <t>151500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z239" s="0" t="inlineStr">
@@ -8211,19 +8191,19 @@
       </c>
       <c r="AC239" s="0" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>114</t>
         </is>
       </c>
     </row>
     <row r="240" spans="1:29">
       <c r="A240" s="0" t="inlineStr">
         <is>
-          <t>HAJ FATIMA</t>
+          <t>PHIL</t>
         </is>
       </c>
       <c r="B240" s="0" t="inlineStr">
         <is>
-          <t>KADUNA</t>
+          <t>JULIUS</t>
         </is>
       </c>
       <c r="R240" s="0" t="inlineStr">
@@ -8233,7 +8213,7 @@
       </c>
       <c r="X240" s="0" t="inlineStr">
         <is>
-          <t>582000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z240" s="0" t="inlineStr">
@@ -8248,7 +8228,7 @@
       </c>
       <c r="AC240" s="0" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>255</t>
         </is>
       </c>
     </row>
@@ -8260,7 +8240,7 @@
       </c>
       <c r="B241" s="0" t="inlineStr">
         <is>
-          <t>KADUNA</t>
+          <t>JUMARE</t>
         </is>
       </c>
       <c r="R241" s="0" t="inlineStr">
@@ -8270,7 +8250,7 @@
       </c>
       <c r="X241" s="0" t="inlineStr">
         <is>
-          <t>127500.00</t>
+          <t>269000.00</t>
         </is>
       </c>
       <c r="Z241" s="0" t="inlineStr">
@@ -8285,19 +8265,29 @@
       </c>
       <c r="AC241" s="0" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>129</t>
         </is>
       </c>
     </row>
     <row r="242" spans="1:29">
       <c r="A242" s="0" t="inlineStr">
         <is>
-          <t>SA'ADATU</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B242" s="0" t="inlineStr">
         <is>
-          <t>KANGIWA</t>
+          <t>KADUNA</t>
+        </is>
+      </c>
+      <c r="L242" s="0" t="inlineStr">
+        <is>
+          <t>KADUNA</t>
+        </is>
+      </c>
+      <c r="M242" s="0" t="inlineStr">
+        <is>
+          <t>KADUNA</t>
         </is>
       </c>
       <c r="R242" s="0" t="inlineStr">
@@ -8307,7 +8297,7 @@
       </c>
       <c r="X242" s="0" t="inlineStr">
         <is>
-          <t>200000.00</t>
+          <t>151500.00</t>
         </is>
       </c>
       <c r="Z242" s="0" t="inlineStr">
@@ -8322,19 +8312,19 @@
       </c>
       <c r="AC242" s="0" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>82</t>
         </is>
       </c>
     </row>
     <row r="243" spans="1:29">
       <c r="A243" s="0" t="inlineStr">
         <is>
-          <t>MOMY</t>
+          <t>HAJ FATIMA</t>
         </is>
       </c>
       <c r="B243" s="0" t="inlineStr">
         <is>
-          <t>KARETO</t>
+          <t>KADUNA</t>
         </is>
       </c>
       <c r="R243" s="0" t="inlineStr">
@@ -8344,7 +8334,7 @@
       </c>
       <c r="X243" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>582000.00</t>
         </is>
       </c>
       <c r="Z243" s="0" t="inlineStr">
@@ -8359,19 +8349,19 @@
       </c>
       <c r="AC243" s="0" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>91</t>
         </is>
       </c>
     </row>
     <row r="244" spans="1:29">
       <c r="A244" s="0" t="inlineStr">
         <is>
-          <t>JIDDAH</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B244" s="0" t="inlineStr">
         <is>
-          <t>KATSINA</t>
+          <t>KADUNA</t>
         </is>
       </c>
       <c r="R244" s="0" t="inlineStr">
@@ -8381,7 +8371,7 @@
       </c>
       <c r="X244" s="0" t="inlineStr">
         <is>
-          <t>45000.00</t>
+          <t>127500.00</t>
         </is>
       </c>
       <c r="Z244" s="0" t="inlineStr">
@@ -8396,19 +8386,19 @@
       </c>
       <c r="AC244" s="0" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>95</t>
         </is>
       </c>
     </row>
     <row r="245" spans="1:29">
       <c r="A245" s="0" t="inlineStr">
         <is>
-          <t>ANTY FATIMA</t>
+          <t>SA'ADATU</t>
         </is>
       </c>
       <c r="B245" s="0" t="inlineStr">
         <is>
-          <t>KATSINA</t>
+          <t>KANGIWA</t>
         </is>
       </c>
       <c r="R245" s="0" t="inlineStr">
@@ -8418,7 +8408,7 @@
       </c>
       <c r="X245" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>200000.00</t>
         </is>
       </c>
       <c r="Z245" s="0" t="inlineStr">
@@ -8433,19 +8423,19 @@
       </c>
       <c r="AC245" s="0" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>109</t>
         </is>
       </c>
     </row>
     <row r="246" spans="1:29">
       <c r="A246" s="0" t="inlineStr">
         <is>
-          <t>HAJ ZAINAB</t>
+          <t>MOMY</t>
         </is>
       </c>
       <c r="B246" s="0" t="inlineStr">
         <is>
-          <t>KATSINA</t>
+          <t>KARETO</t>
         </is>
       </c>
       <c r="R246" s="0" t="inlineStr">
@@ -8470,14 +8460,14 @@
       </c>
       <c r="AC246" s="0" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>157</t>
         </is>
       </c>
     </row>
     <row r="247" spans="1:29">
       <c r="A247" s="0" t="inlineStr">
         <is>
-          <t>HAJ HADIZA</t>
+          <t>JIDDAH</t>
         </is>
       </c>
       <c r="B247" s="0" t="inlineStr">
@@ -8492,7 +8482,7 @@
       </c>
       <c r="X247" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>45000.00</t>
         </is>
       </c>
       <c r="Z247" s="0" t="inlineStr">
@@ -8507,14 +8497,14 @@
       </c>
       <c r="AC247" s="0" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>77</t>
         </is>
       </c>
     </row>
     <row r="248" spans="1:29">
       <c r="A248" s="0" t="inlineStr">
         <is>
-          <t>SUMAYYA</t>
+          <t>ANTY FATIMA</t>
         </is>
       </c>
       <c r="B248" s="0" t="inlineStr">
@@ -8544,14 +8534,14 @@
       </c>
       <c r="AC248" s="0" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="249" spans="1:29">
       <c r="A249" s="0" t="inlineStr">
         <is>
-          <t>HADIZA</t>
+          <t>HAJ ZAINAB</t>
         </is>
       </c>
       <c r="B249" s="0" t="inlineStr">
@@ -8566,7 +8556,7 @@
       </c>
       <c r="X249" s="0" t="inlineStr">
         <is>
-          <t>12000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z249" s="0" t="inlineStr">
@@ -8581,19 +8571,19 @@
       </c>
       <c r="AC249" s="0" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>92</t>
         </is>
       </c>
     </row>
     <row r="250" spans="1:29">
       <c r="A250" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>HAJ HADIZA</t>
         </is>
       </c>
       <c r="B250" s="0" t="inlineStr">
         <is>
-          <t>KAUSAR</t>
+          <t>KATSINA</t>
         </is>
       </c>
       <c r="R250" s="0" t="inlineStr">
@@ -8618,19 +8608,19 @@
       </c>
       <c r="AC250" s="0" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>108</t>
         </is>
       </c>
     </row>
     <row r="251" spans="1:29">
       <c r="A251" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>SUMAYYA</t>
         </is>
       </c>
       <c r="B251" s="0" t="inlineStr">
         <is>
-          <t>KHALIFA KATSINA</t>
+          <t>KATSINA</t>
         </is>
       </c>
       <c r="R251" s="0" t="inlineStr">
@@ -8640,7 +8630,7 @@
       </c>
       <c r="X251" s="0" t="inlineStr">
         <is>
-          <t>170500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z251" s="0" t="inlineStr">
@@ -8655,19 +8645,19 @@
       </c>
       <c r="AC251" s="0" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>186</t>
         </is>
       </c>
     </row>
     <row r="252" spans="1:29">
       <c r="A252" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>HADIZA</t>
         </is>
       </c>
       <c r="B252" s="0" t="inlineStr">
         <is>
-          <t>KOLMANI</t>
+          <t>KATSINA</t>
         </is>
       </c>
       <c r="R252" s="0" t="inlineStr">
@@ -8677,7 +8667,7 @@
       </c>
       <c r="X252" s="0" t="inlineStr">
         <is>
-          <t>40000.00</t>
+          <t>12000.00</t>
         </is>
       </c>
       <c r="Z252" s="0" t="inlineStr">
@@ -8692,19 +8682,19 @@
       </c>
       <c r="AC252" s="0" t="inlineStr">
         <is>
-          <t>205</t>
+          <t>213</t>
         </is>
       </c>
     </row>
     <row r="253" spans="1:29">
       <c r="A253" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B253" s="0" t="inlineStr">
         <is>
-          <t>KWAIRANGA</t>
+          <t>KAUSAR</t>
         </is>
       </c>
       <c r="R253" s="0" t="inlineStr">
@@ -8714,7 +8704,7 @@
       </c>
       <c r="X253" s="0" t="inlineStr">
         <is>
-          <t>480000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z253" s="0" t="inlineStr">
@@ -8729,19 +8719,19 @@
       </c>
       <c r="AC253" s="0" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>160</t>
         </is>
       </c>
     </row>
     <row r="254" spans="1:29">
       <c r="A254" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B254" s="0" t="inlineStr">
         <is>
-          <t>KYARI</t>
+          <t>KHALIFA KATSINA</t>
         </is>
       </c>
       <c r="R254" s="0" t="inlineStr">
@@ -8751,7 +8741,7 @@
       </c>
       <c r="X254" s="0" t="inlineStr">
         <is>
-          <t>40000.00</t>
+          <t>170500.00</t>
         </is>
       </c>
       <c r="Z254" s="0" t="inlineStr">
@@ -8766,19 +8756,19 @@
       </c>
       <c r="AC254" s="0" t="inlineStr">
         <is>
-          <t>292</t>
+          <t>106</t>
         </is>
       </c>
     </row>
     <row r="255" spans="1:29">
       <c r="A255" s="0" t="inlineStr">
         <is>
-          <t>HADIZA</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B255" s="0" t="inlineStr">
         <is>
-          <t>LABO</t>
+          <t>KOLMANI</t>
         </is>
       </c>
       <c r="R255" s="0" t="inlineStr">
@@ -8788,7 +8778,7 @@
       </c>
       <c r="X255" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>40000.00</t>
         </is>
       </c>
       <c r="Z255" s="0" t="inlineStr">
@@ -8803,19 +8793,19 @@
       </c>
       <c r="AC255" s="0" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>205</t>
         </is>
       </c>
     </row>
     <row r="256" spans="1:29">
       <c r="A256" s="0" t="inlineStr">
         <is>
-          <t>UMMI</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B256" s="0" t="inlineStr">
         <is>
-          <t>LABO</t>
+          <t>KWAIRANGA</t>
         </is>
       </c>
       <c r="R256" s="0" t="inlineStr">
@@ -8825,7 +8815,7 @@
       </c>
       <c r="X256" s="0" t="inlineStr">
         <is>
-          <t>1678300.00</t>
+          <t>480000.00</t>
         </is>
       </c>
       <c r="Z256" s="0" t="inlineStr">
@@ -8840,19 +8830,19 @@
       </c>
       <c r="AC256" s="0" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>104</t>
         </is>
       </c>
     </row>
     <row r="257" spans="1:29">
       <c r="A257" s="0" t="inlineStr">
         <is>
-          <t>INNAN</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B257" s="0" t="inlineStr">
         <is>
-          <t>LARAI</t>
+          <t>KYARI</t>
         </is>
       </c>
       <c r="R257" s="0" t="inlineStr">
@@ -8862,7 +8852,7 @@
       </c>
       <c r="X257" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>40000.00</t>
         </is>
       </c>
       <c r="Z257" s="0" t="inlineStr">
@@ -8877,19 +8867,19 @@
       </c>
       <c r="AC257" s="0" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>292</t>
         </is>
       </c>
     </row>
     <row r="258" spans="1:29">
       <c r="A258" s="0" t="inlineStr">
         <is>
-          <t>RAHAMA</t>
+          <t>HADIZA</t>
         </is>
       </c>
       <c r="B258" s="0" t="inlineStr">
         <is>
-          <t>LAWAL</t>
+          <t>LABO</t>
         </is>
       </c>
       <c r="R258" s="0" t="inlineStr">
@@ -8899,7 +8889,7 @@
       </c>
       <c r="X258" s="0" t="inlineStr">
         <is>
-          <t>35000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z258" s="0" t="inlineStr">
@@ -8914,19 +8904,19 @@
       </c>
       <c r="AC258" s="0" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>88</t>
         </is>
       </c>
     </row>
     <row r="259" spans="1:29">
       <c r="A259" s="0" t="inlineStr">
         <is>
-          <t>HAJ HADIZA</t>
+          <t>UMMI</t>
         </is>
       </c>
       <c r="B259" s="0" t="inlineStr">
         <is>
-          <t>LAWAL</t>
+          <t>LABO</t>
         </is>
       </c>
       <c r="R259" s="0" t="inlineStr">
@@ -8936,7 +8926,7 @@
       </c>
       <c r="X259" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1678300.00</t>
         </is>
       </c>
       <c r="Z259" s="0" t="inlineStr">
@@ -8951,19 +8941,19 @@
       </c>
       <c r="AC259" s="0" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>119</t>
         </is>
       </c>
     </row>
     <row r="260" spans="1:29">
       <c r="A260" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>INNAN</t>
         </is>
       </c>
       <c r="B260" s="0" t="inlineStr">
         <is>
-          <t>MACHINA</t>
+          <t>LARAI</t>
         </is>
       </c>
       <c r="R260" s="0" t="inlineStr">
@@ -8973,7 +8963,7 @@
       </c>
       <c r="X260" s="0" t="inlineStr">
         <is>
-          <t>116000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z260" s="0" t="inlineStr">
@@ -8988,19 +8978,19 @@
       </c>
       <c r="AC260" s="0" t="inlineStr">
         <is>
-          <t>296</t>
+          <t>84</t>
         </is>
       </c>
     </row>
     <row r="261" spans="1:29">
       <c r="A261" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>RAHAMA</t>
         </is>
       </c>
       <c r="B261" s="0" t="inlineStr">
         <is>
-          <t>MADU</t>
+          <t>LAWAL</t>
         </is>
       </c>
       <c r="R261" s="0" t="inlineStr">
@@ -9010,7 +9000,7 @@
       </c>
       <c r="X261" s="0" t="inlineStr">
         <is>
-          <t>48000.00</t>
+          <t>35000.00</t>
         </is>
       </c>
       <c r="Z261" s="0" t="inlineStr">
@@ -9025,19 +9015,19 @@
       </c>
       <c r="AC261" s="0" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>80</t>
         </is>
       </c>
     </row>
     <row r="262" spans="1:29">
       <c r="A262" s="0" t="inlineStr">
         <is>
-          <t>RAHAMA</t>
+          <t>HAJ HADIZA</t>
         </is>
       </c>
       <c r="B262" s="0" t="inlineStr">
         <is>
-          <t>MAHMUD</t>
+          <t>LAWAL</t>
         </is>
       </c>
       <c r="R262" s="0" t="inlineStr">
@@ -9062,19 +9052,19 @@
       </c>
       <c r="AC262" s="0" t="inlineStr">
         <is>
-          <t>311</t>
+          <t>310</t>
         </is>
       </c>
     </row>
     <row r="263" spans="1:29">
       <c r="A263" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B263" s="0" t="inlineStr">
         <is>
-          <t>MAIGARI</t>
+          <t>MACHINA</t>
         </is>
       </c>
       <c r="R263" s="0" t="inlineStr">
@@ -9084,7 +9074,7 @@
       </c>
       <c r="X263" s="0" t="inlineStr">
         <is>
-          <t>1978300.00</t>
+          <t>116000.00</t>
         </is>
       </c>
       <c r="Z263" s="0" t="inlineStr">
@@ -9099,19 +9089,19 @@
       </c>
       <c r="AC263" s="0" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>296</t>
         </is>
       </c>
     </row>
     <row r="264" spans="1:29">
       <c r="A264" s="0" t="inlineStr">
         <is>
-          <t>ZUWAIRA</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B264" s="0" t="inlineStr">
         <is>
-          <t>MAJIDADI</t>
+          <t>MADU</t>
         </is>
       </c>
       <c r="R264" s="0" t="inlineStr">
@@ -9121,7 +9111,7 @@
       </c>
       <c r="X264" s="0" t="inlineStr">
         <is>
-          <t>71800.00</t>
+          <t>48000.00</t>
         </is>
       </c>
       <c r="Z264" s="0" t="inlineStr">
@@ -9136,19 +9126,19 @@
       </c>
       <c r="AC264" s="0" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>151</t>
         </is>
       </c>
     </row>
     <row r="265" spans="1:29">
       <c r="A265" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>RAHAMA</t>
         </is>
       </c>
       <c r="B265" s="0" t="inlineStr">
         <is>
-          <t>MALAM</t>
+          <t>MAHMUD</t>
         </is>
       </c>
       <c r="R265" s="0" t="inlineStr">
@@ -9158,7 +9148,7 @@
       </c>
       <c r="X265" s="0" t="inlineStr">
         <is>
-          <t>26500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z265" s="0" t="inlineStr">
@@ -9173,19 +9163,19 @@
       </c>
       <c r="AC265" s="0" t="inlineStr">
         <is>
-          <t>316</t>
+          <t>311</t>
         </is>
       </c>
     </row>
     <row r="266" spans="1:29">
       <c r="A266" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B266" s="0" t="inlineStr">
         <is>
-          <t>MALUMFASHI</t>
+          <t>MAIGARI</t>
         </is>
       </c>
       <c r="R266" s="0" t="inlineStr">
@@ -9195,7 +9185,7 @@
       </c>
       <c r="X266" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1978300.00</t>
         </is>
       </c>
       <c r="Z266" s="0" t="inlineStr">
@@ -9210,19 +9200,19 @@
       </c>
       <c r="AC266" s="0" t="inlineStr">
         <is>
-          <t>124</t>
+          <t>162</t>
         </is>
       </c>
     </row>
     <row r="267" spans="1:29">
       <c r="A267" s="0" t="inlineStr">
         <is>
-          <t>DJA</t>
+          <t>ZUWAIRA</t>
         </is>
       </c>
       <c r="B267" s="0" t="inlineStr">
         <is>
-          <t>MAMAN ABDALLAH</t>
+          <t>MAJIDADI</t>
         </is>
       </c>
       <c r="R267" s="0" t="inlineStr">
@@ -9232,7 +9222,7 @@
       </c>
       <c r="X267" s="0" t="inlineStr">
         <is>
-          <t>120000.00</t>
+          <t>71800.00</t>
         </is>
       </c>
       <c r="Z267" s="0" t="inlineStr">
@@ -9247,19 +9237,19 @@
       </c>
       <c r="AC267" s="0" t="inlineStr">
         <is>
-          <t>178</t>
+          <t>207</t>
         </is>
       </c>
     </row>
     <row r="268" spans="1:29">
       <c r="A268" s="0" t="inlineStr">
         <is>
-          <t>UMMU</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B268" s="0" t="inlineStr">
         <is>
-          <t>MAMAN UWAIS</t>
+          <t>MALAM</t>
         </is>
       </c>
       <c r="R268" s="0" t="inlineStr">
@@ -9269,7 +9259,7 @@
       </c>
       <c r="X268" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>26500.00</t>
         </is>
       </c>
       <c r="Z268" s="0" t="inlineStr">
@@ -9284,19 +9274,19 @@
       </c>
       <c r="AC268" s="0" t="inlineStr">
         <is>
-          <t>271</t>
+          <t>316</t>
         </is>
       </c>
     </row>
     <row r="269" spans="1:29">
       <c r="A269" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B269" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>MALUMFASHI</t>
         </is>
       </c>
       <c r="R269" s="0" t="inlineStr">
@@ -9321,19 +9311,19 @@
       </c>
       <c r="AC269" s="0" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>124</t>
         </is>
       </c>
     </row>
     <row r="270" spans="1:29">
       <c r="A270" s="0" t="inlineStr">
         <is>
-          <t>HAJ FATIMA</t>
+          <t>DJA</t>
         </is>
       </c>
       <c r="B270" s="0" t="inlineStr">
         <is>
-          <t>MUHD</t>
+          <t>MAMAN ABDALLAH</t>
         </is>
       </c>
       <c r="R270" s="0" t="inlineStr">
@@ -9343,7 +9333,7 @@
       </c>
       <c r="X270" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>120000.00</t>
         </is>
       </c>
       <c r="Z270" s="0" t="inlineStr">
@@ -9358,19 +9348,19 @@
       </c>
       <c r="AC270" s="0" t="inlineStr">
         <is>
-          <t>247</t>
+          <t>178</t>
         </is>
       </c>
     </row>
     <row r="271" spans="1:29">
       <c r="A271" s="0" t="inlineStr">
         <is>
-          <t>SHAMSIYYAH</t>
+          <t>UMMU</t>
         </is>
       </c>
       <c r="B271" s="0" t="inlineStr">
         <is>
-          <t>MUHD</t>
+          <t>MAMAN UWAIS</t>
         </is>
       </c>
       <c r="R271" s="0" t="inlineStr">
@@ -9395,19 +9385,19 @@
       </c>
       <c r="AC271" s="0" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>271</t>
         </is>
       </c>
     </row>
     <row r="272" spans="1:29">
       <c r="A272" s="0" t="inlineStr">
         <is>
-          <t>BILKISU</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B272" s="0" t="inlineStr">
         <is>
-          <t>MUKHTAR</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="R272" s="0" t="inlineStr">
@@ -9417,7 +9407,7 @@
       </c>
       <c r="X272" s="0" t="inlineStr">
         <is>
-          <t>108000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z272" s="0" t="inlineStr">
@@ -9432,19 +9422,19 @@
       </c>
       <c r="AC272" s="0" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>94</t>
         </is>
       </c>
     </row>
     <row r="273" spans="1:29">
       <c r="A273" s="0" t="inlineStr">
         <is>
-          <t>UMMI</t>
+          <t>HAJ FATIMA</t>
         </is>
       </c>
       <c r="B273" s="0" t="inlineStr">
         <is>
-          <t>MUMTAZ</t>
+          <t>MUHD</t>
         </is>
       </c>
       <c r="R273" s="0" t="inlineStr">
@@ -9454,7 +9444,7 @@
       </c>
       <c r="X273" s="0" t="inlineStr">
         <is>
-          <t>2507000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z273" s="0" t="inlineStr">
@@ -9469,19 +9459,19 @@
       </c>
       <c r="AC273" s="0" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>247</t>
         </is>
       </c>
     </row>
     <row r="274" spans="1:29">
       <c r="A274" s="0" t="inlineStr">
         <is>
-          <t>MAMAN </t>
+          <t>SHAMSIYYAH</t>
         </is>
       </c>
       <c r="B274" s="0" t="inlineStr">
         <is>
-          <t>NABILA</t>
+          <t>MUHD</t>
         </is>
       </c>
       <c r="R274" s="0" t="inlineStr">
@@ -9506,19 +9496,19 @@
       </c>
       <c r="AC274" s="0" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>257</t>
         </is>
       </c>
     </row>
     <row r="275" spans="1:29">
       <c r="A275" s="0" t="inlineStr">
         <is>
-          <t>ANTY</t>
+          <t>BILKISU</t>
         </is>
       </c>
       <c r="B275" s="0" t="inlineStr">
         <is>
-          <t>NAS</t>
+          <t>MUKHTAR</t>
         </is>
       </c>
       <c r="R275" s="0" t="inlineStr">
@@ -9528,7 +9518,7 @@
       </c>
       <c r="X275" s="0" t="inlineStr">
         <is>
-          <t>1579000.00</t>
+          <t>108000.00</t>
         </is>
       </c>
       <c r="Z275" s="0" t="inlineStr">
@@ -9543,19 +9533,19 @@
       </c>
       <c r="AC275" s="0" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>138</t>
         </is>
       </c>
     </row>
     <row r="276" spans="1:29">
       <c r="A276" s="0" t="inlineStr">
         <is>
-          <t>RUKAYYA</t>
+          <t>UMMI</t>
         </is>
       </c>
       <c r="B276" s="0" t="inlineStr">
         <is>
-          <t>NASIR</t>
+          <t>MUMTAZ</t>
         </is>
       </c>
       <c r="R276" s="0" t="inlineStr">
@@ -9565,7 +9555,7 @@
       </c>
       <c r="X276" s="0" t="inlineStr">
         <is>
-          <t>402000.00</t>
+          <t>2507000.00</t>
         </is>
       </c>
       <c r="Z276" s="0" t="inlineStr">
@@ -9580,19 +9570,19 @@
       </c>
       <c r="AC276" s="0" t="inlineStr">
         <is>
-          <t>188</t>
+          <t>140</t>
         </is>
       </c>
     </row>
     <row r="277" spans="1:29">
       <c r="A277" s="0" t="inlineStr">
         <is>
-          <t>HAFSAT</t>
+          <t>MAMAN </t>
         </is>
       </c>
       <c r="B277" s="0" t="inlineStr">
         <is>
-          <t>NASIR</t>
+          <t>NABILA</t>
         </is>
       </c>
       <c r="R277" s="0" t="inlineStr">
@@ -9602,7 +9592,7 @@
       </c>
       <c r="X277" s="0" t="inlineStr">
         <is>
-          <t>22000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z277" s="0" t="inlineStr">
@@ -9617,19 +9607,19 @@
       </c>
       <c r="AC277" s="0" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>87</t>
         </is>
       </c>
     </row>
     <row r="278" spans="1:29">
       <c r="A278" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>ANTY</t>
         </is>
       </c>
       <c r="B278" s="0" t="inlineStr">
         <is>
-          <t>NATA'ALA</t>
+          <t>NAS</t>
         </is>
       </c>
       <c r="R278" s="0" t="inlineStr">
@@ -9639,7 +9629,7 @@
       </c>
       <c r="X278" s="0" t="inlineStr">
         <is>
-          <t>17000.00</t>
+          <t>1579000.00</t>
         </is>
       </c>
       <c r="Z278" s="0" t="inlineStr">
@@ -9654,19 +9644,19 @@
       </c>
       <c r="AC278" s="0" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>78</t>
         </is>
       </c>
     </row>
     <row r="279" spans="1:29">
       <c r="A279" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>RUKAYYA</t>
         </is>
       </c>
       <c r="B279" s="0" t="inlineStr">
         <is>
-          <t>NINGI</t>
+          <t>NASIR</t>
         </is>
       </c>
       <c r="R279" s="0" t="inlineStr">
@@ -9676,7 +9666,7 @@
       </c>
       <c r="X279" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>402000.00</t>
         </is>
       </c>
       <c r="Z279" s="0" t="inlineStr">
@@ -9691,19 +9681,19 @@
       </c>
       <c r="AC279" s="0" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>188</t>
         </is>
       </c>
     </row>
     <row r="280" spans="1:29">
       <c r="A280" s="0" t="inlineStr">
         <is>
-          <t>BILKIS</t>
+          <t>HAFSAT</t>
         </is>
       </c>
       <c r="B280" s="0" t="inlineStr">
         <is>
-          <t>ONLINE</t>
+          <t>NASIR</t>
         </is>
       </c>
       <c r="R280" s="0" t="inlineStr">
@@ -9713,7 +9703,7 @@
       </c>
       <c r="X280" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>22000.00</t>
         </is>
       </c>
       <c r="Z280" s="0" t="inlineStr">
@@ -9728,19 +9718,19 @@
       </c>
       <c r="AC280" s="0" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>228</t>
         </is>
       </c>
     </row>
     <row r="281" spans="1:29">
       <c r="A281" s="0" t="inlineStr">
         <is>
-          <t>MADAM</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B281" s="0" t="inlineStr">
         <is>
-          <t>RONKE</t>
+          <t>NATA'ALA</t>
         </is>
       </c>
       <c r="R281" s="0" t="inlineStr">
@@ -9750,7 +9740,7 @@
       </c>
       <c r="X281" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>17000.00</t>
         </is>
       </c>
       <c r="Z281" s="0" t="inlineStr">
@@ -9765,19 +9755,19 @@
       </c>
       <c r="AC281" s="0" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>74</t>
         </is>
       </c>
     </row>
     <row r="282" spans="1:29">
       <c r="A282" s="0" t="inlineStr">
         <is>
-          <t>ASH</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B282" s="0" t="inlineStr">
         <is>
-          <t>RUKY</t>
+          <t>NINGI</t>
         </is>
       </c>
       <c r="R282" s="0" t="inlineStr">
@@ -9802,19 +9792,19 @@
       </c>
       <c r="AC282" s="0" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>132</t>
         </is>
       </c>
     </row>
     <row r="283" spans="1:29">
       <c r="A283" s="0" t="inlineStr">
         <is>
-          <t>IKILIMA</t>
+          <t>BILKIS</t>
         </is>
       </c>
       <c r="B283" s="0" t="inlineStr">
         <is>
-          <t>RUWAN DORAWA</t>
+          <t>ONLINE</t>
         </is>
       </c>
       <c r="R283" s="0" t="inlineStr">
@@ -9839,19 +9829,19 @@
       </c>
       <c r="AC283" s="0" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>170</t>
         </is>
       </c>
     </row>
     <row r="284" spans="1:29">
       <c r="A284" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>MADAM</t>
         </is>
       </c>
       <c r="B284" s="0" t="inlineStr">
         <is>
-          <t>SAFWAN</t>
+          <t>RONKE</t>
         </is>
       </c>
       <c r="R284" s="0" t="inlineStr">
@@ -9861,7 +9851,7 @@
       </c>
       <c r="X284" s="0" t="inlineStr">
         <is>
-          <t>32000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z284" s="0" t="inlineStr">
@@ -9876,19 +9866,19 @@
       </c>
       <c r="AC284" s="0" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>226</t>
         </is>
       </c>
     </row>
     <row r="285" spans="1:29">
       <c r="A285" s="0" t="inlineStr">
         <is>
-          <t>SALMA</t>
+          <t>ASH</t>
         </is>
       </c>
       <c r="B285" s="0" t="inlineStr">
         <is>
-          <t>SALMUR</t>
+          <t>RUKY</t>
         </is>
       </c>
       <c r="R285" s="0" t="inlineStr">
@@ -9898,7 +9888,7 @@
       </c>
       <c r="X285" s="0" t="inlineStr">
         <is>
-          <t>47500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z285" s="0" t="inlineStr">
@@ -9913,19 +9903,19 @@
       </c>
       <c r="AC285" s="0" t="inlineStr">
         <is>
-          <t>254</t>
+          <t>76</t>
         </is>
       </c>
     </row>
     <row r="286" spans="1:29">
       <c r="A286" s="0" t="inlineStr">
         <is>
-          <t>ASMI</t>
+          <t>IKILIMA</t>
         </is>
       </c>
       <c r="B286" s="0" t="inlineStr">
         <is>
-          <t>SAMBO</t>
+          <t>RUWAN DORAWA</t>
         </is>
       </c>
       <c r="R286" s="0" t="inlineStr">
@@ -9950,19 +9940,19 @@
       </c>
       <c r="AC286" s="0" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>139</t>
         </is>
       </c>
     </row>
     <row r="287" spans="1:29">
       <c r="A287" s="0" t="inlineStr">
         <is>
-          <t>SAMIHA</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B287" s="0" t="inlineStr">
         <is>
-          <t>SANI</t>
+          <t>SAFWAN</t>
         </is>
       </c>
       <c r="R287" s="0" t="inlineStr">
@@ -9972,7 +9962,7 @@
       </c>
       <c r="X287" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>32000.00</t>
         </is>
       </c>
       <c r="Z287" s="0" t="inlineStr">
@@ -9987,19 +9977,19 @@
       </c>
       <c r="AC287" s="0" t="inlineStr">
         <is>
-          <t>285</t>
+          <t>105</t>
         </is>
       </c>
     </row>
     <row r="288" spans="1:29">
       <c r="A288" s="0" t="inlineStr">
         <is>
-          <t>JAMILA</t>
+          <t>SALMA</t>
         </is>
       </c>
       <c r="B288" s="0" t="inlineStr">
         <is>
-          <t>SHANONO</t>
+          <t>SALMUR</t>
         </is>
       </c>
       <c r="R288" s="0" t="inlineStr">
@@ -10009,7 +9999,7 @@
       </c>
       <c r="X288" s="0" t="inlineStr">
         <is>
-          <t>443000.00</t>
+          <t>47500.00</t>
         </is>
       </c>
       <c r="Z288" s="0" t="inlineStr">
@@ -10024,19 +10014,19 @@
       </c>
       <c r="AC288" s="0" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>254</t>
         </is>
       </c>
     </row>
     <row r="289" spans="1:29">
       <c r="A289" s="0" t="inlineStr">
         <is>
-          <t>FARIDA</t>
+          <t>ASMI</t>
         </is>
       </c>
       <c r="B289" s="0" t="inlineStr">
         <is>
-          <t>SHARADA</t>
+          <t>SAMBO</t>
         </is>
       </c>
       <c r="R289" s="0" t="inlineStr">
@@ -10046,7 +10036,7 @@
       </c>
       <c r="X289" s="0" t="inlineStr">
         <is>
-          <t>95000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z289" s="0" t="inlineStr">
@@ -10061,19 +10051,19 @@
       </c>
       <c r="AC289" s="0" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>243</t>
         </is>
       </c>
     </row>
     <row r="290" spans="1:29">
       <c r="A290" s="0" t="inlineStr">
         <is>
-          <t>FANNE</t>
+          <t>SAMIHA</t>
         </is>
       </c>
       <c r="B290" s="0" t="inlineStr">
         <is>
-          <t>SHARIF</t>
+          <t>SANI</t>
         </is>
       </c>
       <c r="R290" s="0" t="inlineStr">
@@ -10098,19 +10088,19 @@
       </c>
       <c r="AC290" s="0" t="inlineStr">
         <is>
-          <t>179</t>
+          <t>285</t>
         </is>
       </c>
     </row>
     <row r="291" spans="1:29">
       <c r="A291" s="0" t="inlineStr">
         <is>
-          <t>SAMIRA</t>
+          <t>JAMILA</t>
         </is>
       </c>
       <c r="B291" s="0" t="inlineStr">
         <is>
-          <t>SHIRA</t>
+          <t>SHANONO</t>
         </is>
       </c>
       <c r="R291" s="0" t="inlineStr">
@@ -10120,7 +10110,7 @@
       </c>
       <c r="X291" s="0" t="inlineStr">
         <is>
-          <t>156000.00</t>
+          <t>443000.00</t>
         </is>
       </c>
       <c r="Z291" s="0" t="inlineStr">
@@ -10135,19 +10125,19 @@
       </c>
       <c r="AC291" s="0" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>83</t>
         </is>
       </c>
     </row>
     <row r="292" spans="1:29">
       <c r="A292" s="0" t="inlineStr">
         <is>
-          <t>FATIMA </t>
+          <t>FARIDA</t>
         </is>
       </c>
       <c r="B292" s="0" t="inlineStr">
         <is>
-          <t>SIDI</t>
+          <t>SHARADA</t>
         </is>
       </c>
       <c r="R292" s="0" t="inlineStr">
@@ -10157,7 +10147,7 @@
       </c>
       <c r="X292" s="0" t="inlineStr">
         <is>
-          <t>40000.00</t>
+          <t>95000.00</t>
         </is>
       </c>
       <c r="Z292" s="0" t="inlineStr">
@@ -10172,19 +10162,19 @@
       </c>
       <c r="AC292" s="0" t="inlineStr">
         <is>
-          <t>313</t>
+          <t>115</t>
         </is>
       </c>
     </row>
     <row r="293" spans="1:29">
       <c r="A293" s="0" t="inlineStr">
         <is>
-          <t>HADIZA</t>
+          <t>FANNE</t>
         </is>
       </c>
       <c r="B293" s="0" t="inlineStr">
         <is>
-          <t>SOKOTO</t>
+          <t>SHARIF</t>
         </is>
       </c>
       <c r="R293" s="0" t="inlineStr">
@@ -10194,7 +10184,7 @@
       </c>
       <c r="X293" s="0" t="inlineStr">
         <is>
-          <t>852500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z293" s="0" t="inlineStr">
@@ -10209,19 +10199,19 @@
       </c>
       <c r="AC293" s="0" t="inlineStr">
         <is>
-          <t>118</t>
+          <t>179</t>
         </is>
       </c>
     </row>
     <row r="294" spans="1:29">
       <c r="A294" s="0" t="inlineStr">
         <is>
-          <t>FARIDA</t>
+          <t>SAMIRA</t>
         </is>
       </c>
       <c r="B294" s="0" t="inlineStr">
         <is>
-          <t>SULAIMAN</t>
+          <t>SHIRA</t>
         </is>
       </c>
       <c r="R294" s="0" t="inlineStr">
@@ -10231,7 +10221,7 @@
       </c>
       <c r="X294" s="0" t="inlineStr">
         <is>
-          <t>80000.00</t>
+          <t>156000.00</t>
         </is>
       </c>
       <c r="Z294" s="0" t="inlineStr">
@@ -10246,19 +10236,19 @@
       </c>
       <c r="AC294" s="0" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>98</t>
         </is>
       </c>
     </row>
     <row r="295" spans="1:29">
       <c r="A295" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>FATIMA </t>
         </is>
       </c>
       <c r="B295" s="0" t="inlineStr">
         <is>
-          <t>TRENDY</t>
+          <t>SIDI</t>
         </is>
       </c>
       <c r="R295" s="0" t="inlineStr">
@@ -10268,7 +10258,7 @@
       </c>
       <c r="X295" s="0" t="inlineStr">
         <is>
-          <t>18000.00</t>
+          <t>40000.00</t>
         </is>
       </c>
       <c r="Z295" s="0" t="inlineStr">
@@ -10283,19 +10273,19 @@
       </c>
       <c r="AC295" s="0" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>313</t>
         </is>
       </c>
     </row>
     <row r="296" spans="1:29">
       <c r="A296" s="0" t="inlineStr">
         <is>
-          <t>JAMILA</t>
+          <t>HADIZA</t>
         </is>
       </c>
       <c r="B296" s="0" t="inlineStr">
         <is>
-          <t>TUKUR</t>
+          <t>SOKOTO</t>
         </is>
       </c>
       <c r="R296" s="0" t="inlineStr">
@@ -10305,7 +10295,7 @@
       </c>
       <c r="X296" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>852500.00</t>
         </is>
       </c>
       <c r="Z296" s="0" t="inlineStr">
@@ -10320,19 +10310,19 @@
       </c>
       <c r="AC296" s="0" t="inlineStr">
         <is>
-          <t>251</t>
+          <t>118</t>
         </is>
       </c>
     </row>
     <row r="297" spans="1:29">
       <c r="A297" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>FARIDA</t>
         </is>
       </c>
       <c r="B297" s="0" t="inlineStr">
         <is>
-          <t>TURARE</t>
+          <t>SULAIMAN</t>
         </is>
       </c>
       <c r="R297" s="0" t="inlineStr">
@@ -10342,7 +10332,7 @@
       </c>
       <c r="X297" s="0" t="inlineStr">
         <is>
-          <t>21000.00</t>
+          <t>80000.00</t>
         </is>
       </c>
       <c r="Z297" s="0" t="inlineStr">
@@ -10357,19 +10347,19 @@
       </c>
       <c r="AC297" s="0" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>246</t>
         </is>
       </c>
     </row>
     <row r="298" spans="1:29">
       <c r="A298" s="0" t="inlineStr">
         <is>
-          <t>ZAINAB</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B298" s="0" t="inlineStr">
         <is>
-          <t>UMAR</t>
+          <t>TRENDY</t>
         </is>
       </c>
       <c r="R298" s="0" t="inlineStr">
@@ -10379,7 +10369,7 @@
       </c>
       <c r="X298" s="0" t="inlineStr">
         <is>
-          <t>65000.00</t>
+          <t>18000.00</t>
         </is>
       </c>
       <c r="Z298" s="0" t="inlineStr">
@@ -10394,19 +10384,19 @@
       </c>
       <c r="AC298" s="0" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="299" spans="1:29">
       <c r="A299" s="0" t="inlineStr">
         <is>
-          <t>ZAINAB</t>
+          <t>JAMILA</t>
         </is>
       </c>
       <c r="B299" s="0" t="inlineStr">
         <is>
-          <t>USMAN</t>
+          <t>TUKUR</t>
         </is>
       </c>
       <c r="R299" s="0" t="inlineStr">
@@ -10431,19 +10421,19 @@
       </c>
       <c r="AC299" s="0" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>251</t>
         </is>
       </c>
     </row>
     <row r="300" spans="1:29">
       <c r="A300" s="0" t="inlineStr">
         <is>
-          <t>HAJ SADIYA</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B300" s="0" t="inlineStr">
         <is>
-          <t>WAILO</t>
+          <t>TURARE</t>
         </is>
       </c>
       <c r="R300" s="0" t="inlineStr">
@@ -10453,7 +10443,7 @@
       </c>
       <c r="X300" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>21000.00</t>
         </is>
       </c>
       <c r="Z300" s="0" t="inlineStr">
@@ -10468,19 +10458,19 @@
       </c>
       <c r="AC300" s="0" t="inlineStr">
         <is>
-          <t>259</t>
+          <t>153</t>
         </is>
       </c>
     </row>
     <row r="301" spans="1:29">
       <c r="A301" s="0" t="inlineStr">
         <is>
-          <t>SALIHU</t>
+          <t>ZAINAB</t>
         </is>
       </c>
       <c r="B301" s="0" t="inlineStr">
         <is>
-          <t>YABATEX</t>
+          <t>UMAR</t>
         </is>
       </c>
       <c r="R301" s="0" t="inlineStr">
@@ -10490,7 +10480,7 @@
       </c>
       <c r="X301" s="0" t="inlineStr">
         <is>
-          <t>541000.00</t>
+          <t>65000.00</t>
         </is>
       </c>
       <c r="Z301" s="0" t="inlineStr">
@@ -10505,19 +10495,19 @@
       </c>
       <c r="AC301" s="0" t="inlineStr">
         <is>
-          <t>258</t>
+          <t>203</t>
         </is>
       </c>
     </row>
     <row r="302" spans="1:29">
       <c r="A302" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>ZAINAB</t>
         </is>
       </c>
       <c r="B302" s="0" t="inlineStr">
         <is>
-          <t>YAN BIYU</t>
+          <t>USMAN</t>
         </is>
       </c>
       <c r="R302" s="0" t="inlineStr">
@@ -10527,7 +10517,7 @@
       </c>
       <c r="X302" s="0" t="inlineStr">
         <is>
-          <t>2501200.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z302" s="0" t="inlineStr">
@@ -10542,19 +10532,19 @@
       </c>
       <c r="AC302" s="0" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>152</t>
         </is>
       </c>
     </row>
     <row r="303" spans="1:29">
       <c r="A303" s="0" t="inlineStr">
         <is>
-          <t>ZULAIHA</t>
+          <t>HAJ SADIYA</t>
         </is>
       </c>
       <c r="B303" s="0" t="inlineStr">
         <is>
-          <t>YOLA</t>
+          <t>WAILO</t>
         </is>
       </c>
       <c r="R303" s="0" t="inlineStr">
@@ -10564,7 +10554,7 @@
       </c>
       <c r="X303" s="0" t="inlineStr">
         <is>
-          <t>372000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z303" s="0" t="inlineStr">
@@ -10579,19 +10569,19 @@
       </c>
       <c r="AC303" s="0" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>259</t>
         </is>
       </c>
     </row>
     <row r="304" spans="1:29">
       <c r="A304" s="0" t="inlineStr">
         <is>
-          <t>FAUZIYYA</t>
+          <t>SALIHU</t>
         </is>
       </c>
       <c r="B304" s="0" t="inlineStr">
         <is>
-          <t>YOLA</t>
+          <t>YABATEX</t>
         </is>
       </c>
       <c r="R304" s="0" t="inlineStr">
@@ -10601,7 +10591,7 @@
       </c>
       <c r="X304" s="0" t="inlineStr">
         <is>
-          <t>17000.00</t>
+          <t>541000.00</t>
         </is>
       </c>
       <c r="Z304" s="0" t="inlineStr">
@@ -10616,19 +10606,19 @@
       </c>
       <c r="AC304" s="0" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>258</t>
         </is>
       </c>
     </row>
     <row r="305" spans="1:29">
       <c r="A305" s="0" t="inlineStr">
         <is>
-          <t>HAJ RUKAYYA</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B305" s="0" t="inlineStr">
         <is>
-          <t>YUSUF</t>
+          <t>YAN BIYU</t>
         </is>
       </c>
       <c r="R305" s="0" t="inlineStr">
@@ -10638,7 +10628,7 @@
       </c>
       <c r="X305" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>2501200.00</t>
         </is>
       </c>
       <c r="Z305" s="0" t="inlineStr">
@@ -10653,19 +10643,19 @@
       </c>
       <c r="AC305" s="0" t="inlineStr">
         <is>
-          <t>248</t>
+          <t>121</t>
         </is>
       </c>
     </row>
     <row r="306" spans="1:29">
       <c r="A306" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>ZULAIHA</t>
         </is>
       </c>
       <c r="B306" s="0" t="inlineStr">
         <is>
-          <t>ZAHRA ONLINE</t>
+          <t>YOLA</t>
         </is>
       </c>
       <c r="R306" s="0" t="inlineStr">
@@ -10675,7 +10665,7 @@
       </c>
       <c r="X306" s="0" t="inlineStr">
         <is>
-          <t>379500.00</t>
+          <t>372000.00</t>
         </is>
       </c>
       <c r="Z306" s="0" t="inlineStr">
@@ -10690,42 +10680,153 @@
       </c>
       <c r="AC306" s="0" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>110</t>
         </is>
       </c>
     </row>
     <row r="307" spans="1:29">
       <c r="A307" s="0" t="inlineStr">
         <is>
+          <t>FAUZIYYA</t>
+        </is>
+      </c>
+      <c r="B307" s="0" t="inlineStr">
+        <is>
+          <t>YOLA</t>
+        </is>
+      </c>
+      <c r="R307" s="0" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="X307" s="0" t="inlineStr">
+        <is>
+          <t>17000.00</t>
+        </is>
+      </c>
+      <c r="Z307" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA307" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AC307" s="0" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+    </row>
+    <row r="308" spans="1:29">
+      <c r="A308" s="0" t="inlineStr">
+        <is>
+          <t>HAJ RUKAYYA</t>
+        </is>
+      </c>
+      <c r="B308" s="0" t="inlineStr">
+        <is>
+          <t>YUSUF</t>
+        </is>
+      </c>
+      <c r="R308" s="0" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="X308" s="0" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="Z308" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA308" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AC308" s="0" t="inlineStr">
+        <is>
+          <t>248</t>
+        </is>
+      </c>
+    </row>
+    <row r="309" spans="1:29">
+      <c r="A309" s="0" t="inlineStr">
+        <is>
+          <t>MAMAN</t>
+        </is>
+      </c>
+      <c r="B309" s="0" t="inlineStr">
+        <is>
+          <t>ZAHRA ONLINE</t>
+        </is>
+      </c>
+      <c r="R309" s="0" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="X309" s="0" t="inlineStr">
+        <is>
+          <t>379500.00</t>
+        </is>
+      </c>
+      <c r="Z309" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA309" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AC309" s="0" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+    </row>
+    <row r="310" spans="1:29">
+      <c r="A310" s="0" t="inlineStr">
+        <is>
           <t>FATIMA</t>
         </is>
       </c>
-      <c r="B307" s="0" t="inlineStr">
+      <c r="B310" s="0" t="inlineStr">
         <is>
           <t>ZARAMI</t>
         </is>
       </c>
-      <c r="R307" s="0" t="inlineStr">
-        <is>
-          <t>y</t>
-        </is>
-      </c>
-      <c r="X307" s="0" t="inlineStr">
+      <c r="R310" s="0" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="X310" s="0" t="inlineStr">
         <is>
           <t>698500.00</t>
         </is>
       </c>
-      <c r="Z307" s="0" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="AA307" s="0" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="AC307" s="0" t="inlineStr">
+      <c r="Z310" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA310" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AC310" s="0" t="inlineStr">
         <is>
           <t>97</t>
         </is>

</xml_diff>

<commit_message>
Create Sales Report Generator
</commit_message>
<xml_diff>
--- a/Excels/Customers.xlsx
+++ b/Excels/Customers.xlsx
@@ -212,7 +212,7 @@
       </c>
       <c r="X2" s="0" t="inlineStr">
         <is>
-          <t>2460700.00</t>
+          <t>2864500.00</t>
         </is>
       </c>
       <c r="Z2" s="0" t="inlineStr">
@@ -244,7 +244,7 @@
       </c>
       <c r="X3" s="0" t="inlineStr">
         <is>
-          <t>3315600.00</t>
+          <t>3352300.00</t>
         </is>
       </c>
       <c r="Z3" s="0" t="inlineStr">
@@ -372,7 +372,7 @@
       </c>
       <c r="X7" s="0" t="inlineStr">
         <is>
-          <t>2818000.00</t>
+          <t>3414000.00</t>
         </is>
       </c>
       <c r="Z7" s="0" t="inlineStr">
@@ -500,7 +500,7 @@
       </c>
       <c r="X11" s="0" t="inlineStr">
         <is>
-          <t>451000.00</t>
+          <t>591000.00</t>
         </is>
       </c>
       <c r="Z11" s="0" t="inlineStr">
@@ -532,7 +532,7 @@
       </c>
       <c r="X12" s="0" t="inlineStr">
         <is>
-          <t>109427700.00</t>
+          <t>110765800.00</t>
         </is>
       </c>
       <c r="Z12" s="0" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="X14" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>19000.00</t>
         </is>
       </c>
       <c r="Z14" s="0" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="X22" s="0" t="inlineStr">
         <is>
-          <t>15592500.00</t>
+          <t>17135000.00</t>
         </is>
       </c>
       <c r="Z22" s="0" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="X23" s="0" t="inlineStr">
         <is>
-          <t>15089300.00</t>
+          <t>15869800.00</t>
         </is>
       </c>
       <c r="Z23" s="0" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="X27" s="0" t="inlineStr">
         <is>
-          <t>5176000.00</t>
+          <t>10392500.00</t>
         </is>
       </c>
       <c r="Z27" s="0" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="X28" s="0" t="inlineStr">
         <is>
-          <t>4081000.00</t>
+          <t>5172000.00</t>
         </is>
       </c>
       <c r="Z28" s="0" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="X30" s="0" t="inlineStr">
         <is>
-          <t>1134000.00</t>
+          <t>1244000.00</t>
         </is>
       </c>
       <c r="Z30" s="0" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="X34" s="0" t="inlineStr">
         <is>
-          <t>2157000.00</t>
+          <t>2173000.00</t>
         </is>
       </c>
       <c r="Z34" s="0" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="X36" s="0" t="inlineStr">
         <is>
-          <t>2580000.00</t>
+          <t>5795000.00</t>
         </is>
       </c>
       <c r="Z36" s="0" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="X43" s="0" t="inlineStr">
         <is>
-          <t>2925800.00</t>
+          <t>3118800.00</t>
         </is>
       </c>
       <c r="Z43" s="0" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="X48" s="0" t="inlineStr">
         <is>
-          <t>9224900.00</t>
+          <t>10224400.00</t>
         </is>
       </c>
       <c r="Z48" s="0" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="X49" s="0" t="inlineStr">
         <is>
-          <t>7496000.00</t>
+          <t>7856000.00</t>
         </is>
       </c>
       <c r="Z49" s="0" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="X51" s="0" t="inlineStr">
         <is>
-          <t>3446000.00</t>
+          <t>3676000.00</t>
         </is>
       </c>
       <c r="Z51" s="0" t="inlineStr">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="X57" s="0" t="inlineStr">
         <is>
-          <t>648000.00</t>
+          <t>753000.00</t>
         </is>
       </c>
       <c r="Z57" s="0" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="X61" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>150000.00</t>
         </is>
       </c>
       <c r="Z61" s="0" t="inlineStr">
@@ -2548,7 +2548,7 @@
       </c>
       <c r="X75" s="0" t="inlineStr">
         <is>
-          <t>198500.00</t>
+          <t>428500.00</t>
         </is>
       </c>
       <c r="Z75" s="0" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="X79" s="0" t="inlineStr">
         <is>
-          <t>588000.00</t>
+          <t>2475000.00</t>
         </is>
       </c>
       <c r="Z79" s="0" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="X83" s="0" t="inlineStr">
         <is>
-          <t>948000.00</t>
+          <t>1161000.00</t>
         </is>
       </c>
       <c r="Z83" s="0" t="inlineStr">
@@ -3252,7 +3252,7 @@
       </c>
       <c r="X97" s="0" t="inlineStr">
         <is>
-          <t>756000.00</t>
+          <t>866000.00</t>
         </is>
       </c>
       <c r="Z97" s="0" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="X100" s="0" t="inlineStr">
         <is>
-          <t>360000.00</t>
+          <t>440000.00</t>
         </is>
       </c>
       <c r="Z100" s="0" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="X101" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>195000.00</t>
         </is>
       </c>
       <c r="Z101" s="0" t="inlineStr">
@@ -3673,7 +3673,7 @@
       </c>
       <c r="X110" s="0" t="inlineStr">
         <is>
-          <t>1079000.00</t>
+          <t>1115000.00</t>
         </is>
       </c>
       <c r="Z110" s="0" t="inlineStr">
@@ -4153,7 +4153,7 @@
       </c>
       <c r="X125" s="0" t="inlineStr">
         <is>
-          <t>168000.00</t>
+          <t>248000.00</t>
         </is>
       </c>
       <c r="Z125" s="0" t="inlineStr">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="X154" s="0" t="inlineStr">
         <is>
-          <t>174500.00</t>
+          <t>212500.00</t>
         </is>
       </c>
       <c r="Z154" s="0" t="inlineStr">
@@ -5305,7 +5305,7 @@
       </c>
       <c r="X161" s="0" t="inlineStr">
         <is>
-          <t>175000.00</t>
+          <t>229000.00</t>
         </is>
       </c>
       <c r="Z161" s="0" t="inlineStr">
@@ -5881,7 +5881,7 @@
       </c>
       <c r="X179" s="0" t="inlineStr">
         <is>
-          <t>234600.00</t>
+          <t>518600.00</t>
         </is>
       </c>
       <c r="Z179" s="0" t="inlineStr">
@@ -6095,12 +6095,7 @@
     <row r="186" spans="1:29">
       <c r="A186" s="0" t="inlineStr">
         <is>
-          <t>HASIYA</t>
-        </is>
-      </c>
-      <c r="B186" s="0" t="inlineStr">
-        <is>
-          <t> TURAKI - ABK</t>
+          <t>ZAINAB CAMEROON</t>
         </is>
       </c>
       <c r="R186" s="0" t="inlineStr">
@@ -6110,7 +6105,7 @@
       </c>
       <c r="X186" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>20000.00</t>
         </is>
       </c>
       <c r="Z186" s="0" t="inlineStr">
@@ -6125,19 +6120,14 @@
       </c>
       <c r="AC186" s="0" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>337</t>
         </is>
       </c>
     </row>
     <row r="187" spans="1:29">
       <c r="A187" s="0" t="inlineStr">
         <is>
-          <t>HAJ SAMIRA</t>
-        </is>
-      </c>
-      <c r="B187" s="0" t="inlineStr">
-        <is>
-          <t>- ABK</t>
+          <t>UMMI AISHA</t>
         </is>
       </c>
       <c r="R187" s="0" t="inlineStr">
@@ -6147,7 +6137,7 @@
       </c>
       <c r="X187" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>572500.00</t>
         </is>
       </c>
       <c r="Z187" s="0" t="inlineStr">
@@ -6162,19 +6152,14 @@
       </c>
       <c r="AC187" s="0" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>338</t>
         </is>
       </c>
     </row>
     <row r="188" spans="1:29">
       <c r="A188" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
-        </is>
-      </c>
-      <c r="B188" s="0" t="inlineStr">
-        <is>
-          <t>ABANA</t>
+          <t>RAHAMA S FULANI</t>
         </is>
       </c>
       <c r="R188" s="0" t="inlineStr">
@@ -6184,7 +6169,7 @@
       </c>
       <c r="X188" s="0" t="inlineStr">
         <is>
-          <t>251500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z188" s="0" t="inlineStr">
@@ -6199,19 +6184,14 @@
       </c>
       <c r="AC188" s="0" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>339</t>
         </is>
       </c>
     </row>
     <row r="189" spans="1:29">
       <c r="A189" s="0" t="inlineStr">
         <is>
-          <t>KHADIJA</t>
-        </is>
-      </c>
-      <c r="B189" s="0" t="inlineStr">
-        <is>
-          <t>ABDULQADIR</t>
+          <t>MAMAN NABILA</t>
         </is>
       </c>
       <c r="R189" s="0" t="inlineStr">
@@ -6221,7 +6201,7 @@
       </c>
       <c r="X189" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>257500.00</t>
         </is>
       </c>
       <c r="Z189" s="0" t="inlineStr">
@@ -6236,19 +6216,14 @@
       </c>
       <c r="AC189" s="0" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>340</t>
         </is>
       </c>
     </row>
     <row r="190" spans="1:29">
       <c r="A190" s="0" t="inlineStr">
         <is>
-          <t>MARIA</t>
-        </is>
-      </c>
-      <c r="B190" s="0" t="inlineStr">
-        <is>
-          <t>ABDULQADIR</t>
+          <t>UMMI KATSINA</t>
         </is>
       </c>
       <c r="R190" s="0" t="inlineStr">
@@ -6258,7 +6233,7 @@
       </c>
       <c r="X190" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>333500.00</t>
         </is>
       </c>
       <c r="Z190" s="0" t="inlineStr">
@@ -6273,19 +6248,19 @@
       </c>
       <c r="AC190" s="0" t="inlineStr">
         <is>
-          <t>328</t>
+          <t>341</t>
         </is>
       </c>
     </row>
     <row r="191" spans="1:29">
       <c r="A191" s="0" t="inlineStr">
         <is>
-          <t>NURIYYAH</t>
+          <t>HASIYA</t>
         </is>
       </c>
       <c r="B191" s="0" t="inlineStr">
         <is>
-          <t>AHMAD</t>
+          <t> TURAKI - ABK</t>
         </is>
       </c>
       <c r="R191" s="0" t="inlineStr">
@@ -6295,7 +6270,7 @@
       </c>
       <c r="X191" s="0" t="inlineStr">
         <is>
-          <t>443000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z191" s="0" t="inlineStr">
@@ -6310,19 +6285,19 @@
       </c>
       <c r="AC191" s="0" t="inlineStr">
         <is>
-          <t>112</t>
+          <t>222</t>
         </is>
       </c>
     </row>
     <row r="192" spans="1:29">
       <c r="A192" s="0" t="inlineStr">
         <is>
-          <t>HAJ MAIMUNA</t>
+          <t>HAJ SAMIRA</t>
         </is>
       </c>
       <c r="B192" s="0" t="inlineStr">
         <is>
-          <t>AHMAD</t>
+          <t>- ABK</t>
         </is>
       </c>
       <c r="R192" s="0" t="inlineStr">
@@ -6347,19 +6322,19 @@
       </c>
       <c r="AC192" s="0" t="inlineStr">
         <is>
-          <t>279</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="193" spans="1:29">
       <c r="A193" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B193" s="0" t="inlineStr">
         <is>
-          <t>AIRFORCE</t>
+          <t>ABANA</t>
         </is>
       </c>
       <c r="R193" s="0" t="inlineStr">
@@ -6369,7 +6344,7 @@
       </c>
       <c r="X193" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>251500.00</t>
         </is>
       </c>
       <c r="Z193" s="0" t="inlineStr">
@@ -6384,19 +6359,19 @@
       </c>
       <c r="AC193" s="0" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>281</t>
         </is>
       </c>
     </row>
     <row r="194" spans="1:29">
       <c r="A194" s="0" t="inlineStr">
         <is>
-          <t>SADIYA</t>
+          <t>KHADIJA</t>
         </is>
       </c>
       <c r="B194" s="0" t="inlineStr">
         <is>
-          <t>ALA</t>
+          <t>ABDULQADIR</t>
         </is>
       </c>
       <c r="R194" s="0" t="inlineStr">
@@ -6421,19 +6396,19 @@
       </c>
       <c r="AC194" s="0" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>191</t>
         </is>
       </c>
     </row>
     <row r="195" spans="1:29">
       <c r="A195" s="0" t="inlineStr">
         <is>
-          <t>HAJ ZALIHATU</t>
+          <t>MARIA</t>
         </is>
       </c>
       <c r="B195" s="0" t="inlineStr">
         <is>
-          <t>ALERU</t>
+          <t>ABDULQADIR</t>
         </is>
       </c>
       <c r="R195" s="0" t="inlineStr">
@@ -6458,19 +6433,19 @@
       </c>
       <c r="AC195" s="0" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>328</t>
         </is>
       </c>
     </row>
     <row r="196" spans="1:29">
       <c r="A196" s="0" t="inlineStr">
         <is>
-          <t>MA'U</t>
+          <t>NURIYYAH</t>
         </is>
       </c>
       <c r="B196" s="0" t="inlineStr">
         <is>
-          <t>ALHASSAN</t>
+          <t>AHMAD</t>
         </is>
       </c>
       <c r="R196" s="0" t="inlineStr">
@@ -6480,7 +6455,7 @@
       </c>
       <c r="X196" s="0" t="inlineStr">
         <is>
-          <t>48000.00</t>
+          <t>443000.00</t>
         </is>
       </c>
       <c r="Z196" s="0" t="inlineStr">
@@ -6495,19 +6470,19 @@
       </c>
       <c r="AC196" s="0" t="inlineStr">
         <is>
-          <t>183</t>
+          <t>112</t>
         </is>
       </c>
     </row>
     <row r="197" spans="1:29">
       <c r="A197" s="0" t="inlineStr">
         <is>
-          <t>BILKISU</t>
+          <t>HAJ MAIMUNA</t>
         </is>
       </c>
       <c r="B197" s="0" t="inlineStr">
         <is>
-          <t>ALI BALA</t>
+          <t>AHMAD</t>
         </is>
       </c>
       <c r="R197" s="0" t="inlineStr">
@@ -6517,7 +6492,7 @@
       </c>
       <c r="X197" s="0" t="inlineStr">
         <is>
-          <t>922000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z197" s="0" t="inlineStr">
@@ -6532,19 +6507,19 @@
       </c>
       <c r="AC197" s="0" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>279</t>
         </is>
       </c>
     </row>
     <row r="198" spans="1:29">
       <c r="A198" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B198" s="0" t="inlineStr">
         <is>
-          <t>AMATU</t>
+          <t>AIRFORCE</t>
         </is>
       </c>
       <c r="R198" s="0" t="inlineStr">
@@ -6569,19 +6544,19 @@
       </c>
       <c r="AC198" s="0" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>111</t>
         </is>
       </c>
     </row>
     <row r="199" spans="1:29">
       <c r="A199" s="0" t="inlineStr">
         <is>
-          <t>BILKISU</t>
+          <t>SADIYA</t>
         </is>
       </c>
       <c r="B199" s="0" t="inlineStr">
         <is>
-          <t>AMMANI</t>
+          <t>ALA</t>
         </is>
       </c>
       <c r="R199" s="0" t="inlineStr">
@@ -6591,7 +6566,7 @@
       </c>
       <c r="X199" s="0" t="inlineStr">
         <is>
-          <t>65000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z199" s="0" t="inlineStr">
@@ -6606,19 +6581,19 @@
       </c>
       <c r="AC199" s="0" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>126</t>
         </is>
       </c>
     </row>
     <row r="200" spans="1:29">
       <c r="A200" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>HAJ ZALIHATU</t>
         </is>
       </c>
       <c r="B200" s="0" t="inlineStr">
         <is>
-          <t>AMMI</t>
+          <t>ALERU</t>
         </is>
       </c>
       <c r="R200" s="0" t="inlineStr">
@@ -6628,7 +6603,7 @@
       </c>
       <c r="X200" s="0" t="inlineStr">
         <is>
-          <t>279600.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z200" s="0" t="inlineStr">
@@ -6643,19 +6618,19 @@
       </c>
       <c r="AC200" s="0" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>287</t>
         </is>
       </c>
     </row>
     <row r="201" spans="1:29">
       <c r="A201" s="0" t="inlineStr">
         <is>
-          <t>SAMIRA</t>
+          <t>MA'U</t>
         </is>
       </c>
       <c r="B201" s="0" t="inlineStr">
         <is>
-          <t>ARC</t>
+          <t>ALHASSAN</t>
         </is>
       </c>
       <c r="R201" s="0" t="inlineStr">
@@ -6665,7 +6640,7 @@
       </c>
       <c r="X201" s="0" t="inlineStr">
         <is>
-          <t>166500.00</t>
+          <t>48000.00</t>
         </is>
       </c>
       <c r="Z201" s="0" t="inlineStr">
@@ -6680,19 +6655,19 @@
       </c>
       <c r="AC201" s="0" t="inlineStr">
         <is>
-          <t>187</t>
+          <t>183</t>
         </is>
       </c>
     </row>
     <row r="202" spans="1:29">
       <c r="A202" s="0" t="inlineStr">
         <is>
-          <t>HAJ HAUWA</t>
+          <t>BILKISU</t>
         </is>
       </c>
       <c r="B202" s="0" t="inlineStr">
         <is>
-          <t>AWAISU</t>
+          <t>ALI BALA</t>
         </is>
       </c>
       <c r="R202" s="0" t="inlineStr">
@@ -6702,7 +6677,7 @@
       </c>
       <c r="X202" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1342000.00</t>
         </is>
       </c>
       <c r="Z202" s="0" t="inlineStr">
@@ -6717,19 +6692,19 @@
       </c>
       <c r="AC202" s="0" t="inlineStr">
         <is>
-          <t>284</t>
+          <t>79</t>
         </is>
       </c>
     </row>
     <row r="203" spans="1:29">
       <c r="A203" s="0" t="inlineStr">
         <is>
-          <t>ZAINAB</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B203" s="0" t="inlineStr">
         <is>
-          <t>AZARE</t>
+          <t>AMATU</t>
         </is>
       </c>
       <c r="R203" s="0" t="inlineStr">
@@ -6754,19 +6729,19 @@
       </c>
       <c r="AC203" s="0" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>134</t>
         </is>
       </c>
     </row>
     <row r="204" spans="1:29">
       <c r="A204" s="0" t="inlineStr">
         <is>
-          <t>RAHAMA</t>
+          <t>BILKISU</t>
         </is>
       </c>
       <c r="B204" s="0" t="inlineStr">
         <is>
-          <t>BAMALLI</t>
+          <t>AMMANI</t>
         </is>
       </c>
       <c r="R204" s="0" t="inlineStr">
@@ -6776,7 +6751,7 @@
       </c>
       <c r="X204" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>65000.00</t>
         </is>
       </c>
       <c r="Z204" s="0" t="inlineStr">
@@ -6791,19 +6766,19 @@
       </c>
       <c r="AC204" s="0" t="inlineStr">
         <is>
-          <t>265</t>
+          <t>189</t>
         </is>
       </c>
     </row>
     <row r="205" spans="1:29">
       <c r="A205" s="0" t="inlineStr">
         <is>
-          <t>NAFISA</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B205" s="0" t="inlineStr">
         <is>
-          <t>BARAU</t>
+          <t>AMMI</t>
         </is>
       </c>
       <c r="R205" s="0" t="inlineStr">
@@ -6813,7 +6788,7 @@
       </c>
       <c r="X205" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>288100.00</t>
         </is>
       </c>
       <c r="Z205" s="0" t="inlineStr">
@@ -6828,19 +6803,19 @@
       </c>
       <c r="AC205" s="0" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>130</t>
         </is>
       </c>
     </row>
     <row r="206" spans="1:29">
       <c r="A206" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>SAMIRA</t>
         </is>
       </c>
       <c r="B206" s="0" t="inlineStr">
         <is>
-          <t>BAUCHI</t>
+          <t>ARC</t>
         </is>
       </c>
       <c r="R206" s="0" t="inlineStr">
@@ -6850,7 +6825,7 @@
       </c>
       <c r="X206" s="0" t="inlineStr">
         <is>
-          <t>195000.00</t>
+          <t>166500.00</t>
         </is>
       </c>
       <c r="Z206" s="0" t="inlineStr">
@@ -6865,19 +6840,19 @@
       </c>
       <c r="AC206" s="0" t="inlineStr">
         <is>
-          <t>314</t>
+          <t>187</t>
         </is>
       </c>
     </row>
     <row r="207" spans="1:29">
       <c r="A207" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>HAJ HAUWA</t>
         </is>
       </c>
       <c r="B207" s="0" t="inlineStr">
         <is>
-          <t>BAWA ROAD</t>
+          <t>AWAISU</t>
         </is>
       </c>
       <c r="R207" s="0" t="inlineStr">
@@ -6887,7 +6862,7 @@
       </c>
       <c r="X207" s="0" t="inlineStr">
         <is>
-          <t>1298000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z207" s="0" t="inlineStr">
@@ -6902,19 +6877,19 @@
       </c>
       <c r="AC207" s="0" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>284</t>
         </is>
       </c>
     </row>
     <row r="208" spans="1:29">
       <c r="A208" s="0" t="inlineStr">
         <is>
-          <t>HAUWA</t>
+          <t>ZAINAB</t>
         </is>
       </c>
       <c r="B208" s="0" t="inlineStr">
         <is>
-          <t>BELLO</t>
+          <t>AZARE</t>
         </is>
       </c>
       <c r="R208" s="0" t="inlineStr">
@@ -6939,19 +6914,19 @@
       </c>
       <c r="AC208" s="0" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>144</t>
         </is>
       </c>
     </row>
     <row r="209" spans="1:29">
       <c r="A209" s="0" t="inlineStr">
         <is>
-          <t>FARIDA</t>
+          <t>RAHAMA</t>
         </is>
       </c>
       <c r="B209" s="0" t="inlineStr">
         <is>
-          <t>BINDAWA</t>
+          <t>BAMALLI</t>
         </is>
       </c>
       <c r="R209" s="0" t="inlineStr">
@@ -6976,19 +6951,19 @@
       </c>
       <c r="AC209" s="0" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>265</t>
         </is>
       </c>
     </row>
     <row r="210" spans="1:29">
       <c r="A210" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>NAFISA</t>
         </is>
       </c>
       <c r="B210" s="0" t="inlineStr">
         <is>
-          <t>BINDAWA</t>
+          <t>BARAU</t>
         </is>
       </c>
       <c r="R210" s="0" t="inlineStr">
@@ -6998,7 +6973,7 @@
       </c>
       <c r="X210" s="0" t="inlineStr">
         <is>
-          <t>937000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z210" s="0" t="inlineStr">
@@ -7013,19 +6988,19 @@
       </c>
       <c r="AC210" s="0" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>148</t>
         </is>
       </c>
     </row>
     <row r="211" spans="1:29">
       <c r="A211" s="0" t="inlineStr">
         <is>
-          <t>MARIA</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B211" s="0" t="inlineStr">
         <is>
-          <t>BOSE</t>
+          <t>BAUCHI</t>
         </is>
       </c>
       <c r="R211" s="0" t="inlineStr">
@@ -7035,7 +7010,7 @@
       </c>
       <c r="X211" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>195000.00</t>
         </is>
       </c>
       <c r="Z211" s="0" t="inlineStr">
@@ -7050,19 +7025,19 @@
       </c>
       <c r="AC211" s="0" t="inlineStr">
         <is>
-          <t>295</t>
+          <t>314</t>
         </is>
       </c>
     </row>
     <row r="212" spans="1:29">
       <c r="A212" s="0" t="inlineStr">
         <is>
-          <t>HAJ MARYAM</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B212" s="0" t="inlineStr">
         <is>
-          <t>BUHARI</t>
+          <t>BAWA ROAD</t>
         </is>
       </c>
       <c r="R212" s="0" t="inlineStr">
@@ -7072,7 +7047,7 @@
       </c>
       <c r="X212" s="0" t="inlineStr">
         <is>
-          <t>115000.00</t>
+          <t>1298000.00</t>
         </is>
       </c>
       <c r="Z212" s="0" t="inlineStr">
@@ -7087,19 +7062,19 @@
       </c>
       <c r="AC212" s="0" t="inlineStr">
         <is>
-          <t>312</t>
+          <t>113</t>
         </is>
       </c>
     </row>
     <row r="213" spans="1:29">
       <c r="A213" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>HAUWA</t>
         </is>
       </c>
       <c r="B213" s="0" t="inlineStr">
         <is>
-          <t>BULAMA</t>
+          <t>BELLO</t>
         </is>
       </c>
       <c r="R213" s="0" t="inlineStr">
@@ -7124,19 +7099,19 @@
       </c>
       <c r="AC213" s="0" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>125</t>
         </is>
       </c>
     </row>
     <row r="214" spans="1:29">
       <c r="A214" s="0" t="inlineStr">
         <is>
-          <t>KHADIJA</t>
+          <t>FARIDA</t>
         </is>
       </c>
       <c r="B214" s="0" t="inlineStr">
         <is>
-          <t>CHIROMA</t>
+          <t>BINDAWA</t>
         </is>
       </c>
       <c r="R214" s="0" t="inlineStr">
@@ -7146,7 +7121,7 @@
       </c>
       <c r="X214" s="0" t="inlineStr">
         <is>
-          <t>8500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z214" s="0" t="inlineStr">
@@ -7161,19 +7136,19 @@
       </c>
       <c r="AC214" s="0" t="inlineStr">
         <is>
-          <t>184</t>
+          <t>93</t>
         </is>
       </c>
     </row>
     <row r="215" spans="1:29">
       <c r="A215" s="0" t="inlineStr">
         <is>
-          <t>ZAHRA</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B215" s="0" t="inlineStr">
         <is>
-          <t>COLLECTION</t>
+          <t>BINDAWA</t>
         </is>
       </c>
       <c r="R215" s="0" t="inlineStr">
@@ -7183,7 +7158,7 @@
       </c>
       <c r="X215" s="0" t="inlineStr">
         <is>
-          <t>171000.00</t>
+          <t>937000.00</t>
         </is>
       </c>
       <c r="Z215" s="0" t="inlineStr">
@@ -7198,19 +7173,19 @@
       </c>
       <c r="AC215" s="0" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>123</t>
         </is>
       </c>
     </row>
     <row r="216" spans="1:29">
       <c r="A216" s="0" t="inlineStr">
         <is>
-          <t>MAIMUNA</t>
+          <t>MARIA</t>
         </is>
       </c>
       <c r="B216" s="0" t="inlineStr">
         <is>
-          <t>CUSTOM</t>
+          <t>BOSE</t>
         </is>
       </c>
       <c r="R216" s="0" t="inlineStr">
@@ -7220,7 +7195,7 @@
       </c>
       <c r="X216" s="0" t="inlineStr">
         <is>
-          <t>20000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z216" s="0" t="inlineStr">
@@ -7235,19 +7210,19 @@
       </c>
       <c r="AC216" s="0" t="inlineStr">
         <is>
-          <t>227</t>
+          <t>295</t>
         </is>
       </c>
     </row>
     <row r="217" spans="1:29">
       <c r="A217" s="0" t="inlineStr">
         <is>
-          <t>MAMAN AISHA</t>
+          <t>HAJ MARYAM</t>
         </is>
       </c>
       <c r="B217" s="0" t="inlineStr">
         <is>
-          <t>DAHIRU</t>
+          <t>BUHARI</t>
         </is>
       </c>
       <c r="R217" s="0" t="inlineStr">
@@ -7257,7 +7232,7 @@
       </c>
       <c r="X217" s="0" t="inlineStr">
         <is>
-          <t>75000.00</t>
+          <t>115000.00</t>
         </is>
       </c>
       <c r="Z217" s="0" t="inlineStr">
@@ -7272,19 +7247,19 @@
       </c>
       <c r="AC217" s="0" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>312</t>
         </is>
       </c>
     </row>
     <row r="218" spans="1:29">
       <c r="A218" s="0" t="inlineStr">
         <is>
-          <t>MAIMUNA</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B218" s="0" t="inlineStr">
         <is>
-          <t>DAN ASABE</t>
+          <t>BULAMA</t>
         </is>
       </c>
       <c r="R218" s="0" t="inlineStr">
@@ -7309,19 +7284,19 @@
       </c>
       <c r="AC218" s="0" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>253</t>
         </is>
       </c>
     </row>
     <row r="219" spans="1:29">
       <c r="A219" s="0" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>KHADIJA</t>
         </is>
       </c>
       <c r="B219" s="0" t="inlineStr">
         <is>
-          <t>DORAYI</t>
+          <t>CHIROMA</t>
         </is>
       </c>
       <c r="R219" s="0" t="inlineStr">
@@ -7331,7 +7306,7 @@
       </c>
       <c r="X219" s="0" t="inlineStr">
         <is>
-          <t>3667000.00</t>
+          <t>8500.00</t>
         </is>
       </c>
       <c r="Z219" s="0" t="inlineStr">
@@ -7346,19 +7321,19 @@
       </c>
       <c r="AC219" s="0" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>184</t>
         </is>
       </c>
     </row>
     <row r="220" spans="1:29">
       <c r="A220" s="0" t="inlineStr">
         <is>
-          <t>UMMI</t>
+          <t>ZAHRA</t>
         </is>
       </c>
       <c r="B220" s="0" t="inlineStr">
         <is>
-          <t>FAB SHOP</t>
+          <t>COLLECTION</t>
         </is>
       </c>
       <c r="R220" s="0" t="inlineStr">
@@ -7368,7 +7343,7 @@
       </c>
       <c r="X220" s="0" t="inlineStr">
         <is>
-          <t>1160000.00</t>
+          <t>171000.00</t>
         </is>
       </c>
       <c r="Z220" s="0" t="inlineStr">
@@ -7383,19 +7358,19 @@
       </c>
       <c r="AC220" s="0" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>136</t>
         </is>
       </c>
     </row>
     <row r="221" spans="1:29">
       <c r="A221" s="0" t="inlineStr">
         <is>
-          <t>JAMI</t>
+          <t>MAIMUNA</t>
         </is>
       </c>
       <c r="B221" s="0" t="inlineStr">
         <is>
-          <t>FABRICS</t>
+          <t>CUSTOM</t>
         </is>
       </c>
       <c r="R221" s="0" t="inlineStr">
@@ -7405,7 +7380,7 @@
       </c>
       <c r="X221" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>20000.00</t>
         </is>
       </c>
       <c r="Z221" s="0" t="inlineStr">
@@ -7420,19 +7395,19 @@
       </c>
       <c r="AC221" s="0" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>227</t>
         </is>
       </c>
     </row>
     <row r="222" spans="1:29">
       <c r="A222" s="0" t="inlineStr">
         <is>
-          <t>SAMIRA</t>
+          <t>MAMAN AISHA</t>
         </is>
       </c>
       <c r="B222" s="0" t="inlineStr">
         <is>
-          <t>FAGGE</t>
+          <t>DAHIRU</t>
         </is>
       </c>
       <c r="R222" s="0" t="inlineStr">
@@ -7442,7 +7417,7 @@
       </c>
       <c r="X222" s="0" t="inlineStr">
         <is>
-          <t>155000.00</t>
+          <t>75000.00</t>
         </is>
       </c>
       <c r="Z222" s="0" t="inlineStr">
@@ -7457,19 +7432,19 @@
       </c>
       <c r="AC222" s="0" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>194</t>
         </is>
       </c>
     </row>
     <row r="223" spans="1:29">
       <c r="A223" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>MAIMUNA</t>
         </is>
       </c>
       <c r="B223" s="0" t="inlineStr">
         <is>
-          <t>FAGGO</t>
+          <t>DAN ASABE</t>
         </is>
       </c>
       <c r="R223" s="0" t="inlineStr">
@@ -7479,7 +7454,7 @@
       </c>
       <c r="X223" s="0" t="inlineStr">
         <is>
-          <t>45000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z223" s="0" t="inlineStr">
@@ -7494,19 +7469,19 @@
       </c>
       <c r="AC223" s="0" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>169</t>
         </is>
       </c>
     </row>
     <row r="224" spans="1:29">
       <c r="A224" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="B224" s="0" t="inlineStr">
         <is>
-          <t>FAROUQ</t>
+          <t>DORAYI</t>
         </is>
       </c>
       <c r="R224" s="0" t="inlineStr">
@@ -7516,7 +7491,7 @@
       </c>
       <c r="X224" s="0" t="inlineStr">
         <is>
-          <t>290000.00</t>
+          <t>3667000.00</t>
         </is>
       </c>
       <c r="Z224" s="0" t="inlineStr">
@@ -7531,19 +7506,19 @@
       </c>
       <c r="AC224" s="0" t="inlineStr">
         <is>
-          <t>212</t>
+          <t>172</t>
         </is>
       </c>
     </row>
     <row r="225" spans="1:29">
       <c r="A225" s="0" t="inlineStr">
         <is>
-          <t>MUSA</t>
+          <t>UMMI</t>
         </is>
       </c>
       <c r="B225" s="0" t="inlineStr">
         <is>
-          <t>GARBA</t>
+          <t>FAB SHOP</t>
         </is>
       </c>
       <c r="R225" s="0" t="inlineStr">
@@ -7553,7 +7528,7 @@
       </c>
       <c r="X225" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1160000.00</t>
         </is>
       </c>
       <c r="Z225" s="0" t="inlineStr">
@@ -7568,19 +7543,19 @@
       </c>
       <c r="AC225" s="0" t="inlineStr">
         <is>
-          <t>214</t>
+          <t>100</t>
         </is>
       </c>
     </row>
     <row r="226" spans="1:29">
       <c r="A226" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>JAMI</t>
         </is>
       </c>
       <c r="B226" s="0" t="inlineStr">
         <is>
-          <t>GOMBE</t>
+          <t>FABRICS</t>
         </is>
       </c>
       <c r="R226" s="0" t="inlineStr">
@@ -7605,19 +7580,19 @@
       </c>
       <c r="AC226" s="0" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>142</t>
         </is>
       </c>
     </row>
     <row r="227" spans="1:29">
       <c r="A227" s="0" t="inlineStr">
         <is>
-          <t>MOMY</t>
+          <t>SAMIRA</t>
         </is>
       </c>
       <c r="B227" s="0" t="inlineStr">
         <is>
-          <t>GOMBE</t>
+          <t>FAGGE</t>
         </is>
       </c>
       <c r="R227" s="0" t="inlineStr">
@@ -7627,7 +7602,7 @@
       </c>
       <c r="X227" s="0" t="inlineStr">
         <is>
-          <t>335000.00</t>
+          <t>355000.00</t>
         </is>
       </c>
       <c r="Z227" s="0" t="inlineStr">
@@ -7642,19 +7617,19 @@
       </c>
       <c r="AC227" s="0" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>89</t>
         </is>
       </c>
     </row>
     <row r="228" spans="1:29">
       <c r="A228" s="0" t="inlineStr">
         <is>
-          <t>HAJ HAJARA</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B228" s="0" t="inlineStr">
         <is>
-          <t>GOMBE</t>
+          <t>FAGGO</t>
         </is>
       </c>
       <c r="R228" s="0" t="inlineStr">
@@ -7664,7 +7639,7 @@
       </c>
       <c r="X228" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>45000.00</t>
         </is>
       </c>
       <c r="Z228" s="0" t="inlineStr">
@@ -7679,19 +7654,19 @@
       </c>
       <c r="AC228" s="0" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>204</t>
         </is>
       </c>
     </row>
     <row r="229" spans="1:29">
       <c r="A229" s="0" t="inlineStr">
         <is>
-          <t>SAMIRA</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B229" s="0" t="inlineStr">
         <is>
-          <t>GUNU</t>
+          <t>FAROUQ</t>
         </is>
       </c>
       <c r="R229" s="0" t="inlineStr">
@@ -7701,7 +7676,7 @@
       </c>
       <c r="X229" s="0" t="inlineStr">
         <is>
-          <t>24000.00</t>
+          <t>290000.00</t>
         </is>
       </c>
       <c r="Z229" s="0" t="inlineStr">
@@ -7716,19 +7691,19 @@
       </c>
       <c r="AC229" s="0" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>212</t>
         </is>
       </c>
     </row>
     <row r="230" spans="1:29">
       <c r="A230" s="0" t="inlineStr">
         <is>
-          <t>BILKISU</t>
+          <t>MUSA</t>
         </is>
       </c>
       <c r="B230" s="0" t="inlineStr">
         <is>
-          <t>GWALABE</t>
+          <t>GARBA</t>
         </is>
       </c>
       <c r="R230" s="0" t="inlineStr">
@@ -7753,19 +7728,19 @@
       </c>
       <c r="AC230" s="0" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>214</t>
         </is>
       </c>
     </row>
     <row r="231" spans="1:29">
       <c r="A231" s="0" t="inlineStr">
         <is>
-          <t>HAUWA</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B231" s="0" t="inlineStr">
         <is>
-          <t>GWALABE</t>
+          <t>GOMBE</t>
         </is>
       </c>
       <c r="R231" s="0" t="inlineStr">
@@ -7775,7 +7750,7 @@
       </c>
       <c r="X231" s="0" t="inlineStr">
         <is>
-          <t>60000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z231" s="0" t="inlineStr">
@@ -7790,19 +7765,19 @@
       </c>
       <c r="AC231" s="0" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>103</t>
         </is>
       </c>
     </row>
     <row r="232" spans="1:29">
       <c r="A232" s="0" t="inlineStr">
         <is>
-          <t>MAMA</t>
+          <t>MOMY</t>
         </is>
       </c>
       <c r="B232" s="0" t="inlineStr">
         <is>
-          <t>H &amp; M</t>
+          <t>GOMBE</t>
         </is>
       </c>
       <c r="R232" s="0" t="inlineStr">
@@ -7812,7 +7787,7 @@
       </c>
       <c r="X232" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>375000.00</t>
         </is>
       </c>
       <c r="Z232" s="0" t="inlineStr">
@@ -7827,19 +7802,19 @@
       </c>
       <c r="AC232" s="0" t="inlineStr">
         <is>
-          <t>163</t>
+          <t>143</t>
         </is>
       </c>
     </row>
     <row r="233" spans="1:29">
       <c r="A233" s="0" t="inlineStr">
         <is>
-          <t>HAJ HAUWA</t>
+          <t>HAJ HAJARA</t>
         </is>
       </c>
       <c r="B233" s="0" t="inlineStr">
         <is>
-          <t>HABIB</t>
+          <t>GOMBE</t>
         </is>
       </c>
       <c r="R233" s="0" t="inlineStr">
@@ -7864,24 +7839,19 @@
       </c>
       <c r="AC233" s="0" t="inlineStr">
         <is>
-          <t>264</t>
+          <t>209</t>
         </is>
       </c>
     </row>
     <row r="234" spans="1:29">
       <c r="A234" s="0" t="inlineStr">
         <is>
-          <t>KAMILA</t>
+          <t>SAMIRA</t>
         </is>
       </c>
       <c r="B234" s="0" t="inlineStr">
         <is>
-          <t>HADEJA</t>
-        </is>
-      </c>
-      <c r="D234" s="0" t="inlineStr">
-        <is>
-          <t>+2347054680033</t>
+          <t>GUNU</t>
         </is>
       </c>
       <c r="R234" s="0" t="inlineStr">
@@ -7891,7 +7861,7 @@
       </c>
       <c r="X234" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>124000.00</t>
         </is>
       </c>
       <c r="Z234" s="0" t="inlineStr">
@@ -7906,19 +7876,19 @@
       </c>
       <c r="AC234" s="0" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>159</t>
         </is>
       </c>
     </row>
     <row r="235" spans="1:29">
       <c r="A235" s="0" t="inlineStr">
         <is>
-          <t>HAJ RAKIYA</t>
+          <t>BILKISU</t>
         </is>
       </c>
       <c r="B235" s="0" t="inlineStr">
         <is>
-          <t>HAMZA</t>
+          <t>GWALABE</t>
         </is>
       </c>
       <c r="R235" s="0" t="inlineStr">
@@ -7943,19 +7913,19 @@
       </c>
       <c r="AC235" s="0" t="inlineStr">
         <is>
-          <t>291</t>
+          <t>101</t>
         </is>
       </c>
     </row>
     <row r="236" spans="1:29">
       <c r="A236" s="0" t="inlineStr">
         <is>
-          <t>HAJ HAFSAT</t>
+          <t>HAUWA</t>
         </is>
       </c>
       <c r="B236" s="0" t="inlineStr">
         <is>
-          <t>HAMZA</t>
+          <t>GWALABE</t>
         </is>
       </c>
       <c r="R236" s="0" t="inlineStr">
@@ -7965,7 +7935,7 @@
       </c>
       <c r="X236" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>60000.00</t>
         </is>
       </c>
       <c r="Z236" s="0" t="inlineStr">
@@ -7980,19 +7950,19 @@
       </c>
       <c r="AC236" s="0" t="inlineStr">
         <is>
-          <t>306</t>
+          <t>321</t>
         </is>
       </c>
     </row>
     <row r="237" spans="1:29">
       <c r="A237" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>MAMA</t>
         </is>
       </c>
       <c r="B237" s="0" t="inlineStr">
         <is>
-          <t>HANIFA GOMBE</t>
+          <t>H &amp; M</t>
         </is>
       </c>
       <c r="R237" s="0" t="inlineStr">
@@ -8002,7 +7972,7 @@
       </c>
       <c r="X237" s="0" t="inlineStr">
         <is>
-          <t>279000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z237" s="0" t="inlineStr">
@@ -8017,19 +7987,19 @@
       </c>
       <c r="AC237" s="0" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>163</t>
         </is>
       </c>
     </row>
     <row r="238" spans="1:29">
       <c r="A238" s="0" t="inlineStr">
         <is>
-          <t>MAIMUNA</t>
+          <t>HAJ HAUWA</t>
         </is>
       </c>
       <c r="B238" s="0" t="inlineStr">
         <is>
-          <t>HASSAN</t>
+          <t>HABIB</t>
         </is>
       </c>
       <c r="R238" s="0" t="inlineStr">
@@ -8054,19 +8024,24 @@
       </c>
       <c r="AC238" s="0" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>264</t>
         </is>
       </c>
     </row>
     <row r="239" spans="1:29">
       <c r="A239" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>KAMILA</t>
         </is>
       </c>
       <c r="B239" s="0" t="inlineStr">
         <is>
-          <t>HASSAN</t>
+          <t>HADEJA</t>
+        </is>
+      </c>
+      <c r="D239" s="0" t="inlineStr">
+        <is>
+          <t>+2347054680033</t>
         </is>
       </c>
       <c r="R239" s="0" t="inlineStr">
@@ -8076,7 +8051,7 @@
       </c>
       <c r="X239" s="0" t="inlineStr">
         <is>
-          <t>26000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z239" s="0" t="inlineStr">
@@ -8091,19 +8066,19 @@
       </c>
       <c r="AC239" s="0" t="inlineStr">
         <is>
-          <t>326</t>
+          <t>199</t>
         </is>
       </c>
     </row>
     <row r="240" spans="1:29">
       <c r="A240" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>HAJ RAKIYA</t>
         </is>
       </c>
       <c r="B240" s="0" t="inlineStr">
         <is>
-          <t>HISHAM - ABK</t>
+          <t>HAMZA</t>
         </is>
       </c>
       <c r="R240" s="0" t="inlineStr">
@@ -8128,19 +8103,19 @@
       </c>
       <c r="AC240" s="0" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>291</t>
         </is>
       </c>
     </row>
     <row r="241" spans="1:29">
       <c r="A241" s="0" t="inlineStr">
         <is>
-          <t>MALAMA</t>
+          <t>HAJ HAFSAT</t>
         </is>
       </c>
       <c r="B241" s="0" t="inlineStr">
         <is>
-          <t>HUSSAINA</t>
+          <t>HAMZA</t>
         </is>
       </c>
       <c r="R241" s="0" t="inlineStr">
@@ -8150,7 +8125,7 @@
       </c>
       <c r="X241" s="0" t="inlineStr">
         <is>
-          <t>590000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z241" s="0" t="inlineStr">
@@ -8165,19 +8140,19 @@
       </c>
       <c r="AC241" s="0" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>306</t>
         </is>
       </c>
     </row>
     <row r="242" spans="1:29">
       <c r="A242" s="0" t="inlineStr">
         <is>
-          <t>SA'ADATU </t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B242" s="0" t="inlineStr">
         <is>
-          <t>HUSSAINI</t>
+          <t>HANIFA GOMBE</t>
         </is>
       </c>
       <c r="R242" s="0" t="inlineStr">
@@ -8187,7 +8162,7 @@
       </c>
       <c r="X242" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>279000.00</t>
         </is>
       </c>
       <c r="Z242" s="0" t="inlineStr">
@@ -8202,19 +8177,19 @@
       </c>
       <c r="AC242" s="0" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>120</t>
         </is>
       </c>
     </row>
     <row r="243" spans="1:29">
       <c r="A243" s="0" t="inlineStr">
         <is>
-          <t>UMRATU</t>
+          <t>MAIMUNA</t>
         </is>
       </c>
       <c r="B243" s="0" t="inlineStr">
         <is>
-          <t>HUSSAINI</t>
+          <t>HASSAN</t>
         </is>
       </c>
       <c r="R243" s="0" t="inlineStr">
@@ -8239,19 +8214,19 @@
       </c>
       <c r="AC243" s="0" t="inlineStr">
         <is>
-          <t>322</t>
+          <t>323</t>
         </is>
       </c>
     </row>
     <row r="244" spans="1:29">
       <c r="A244" s="0" t="inlineStr">
         <is>
-          <t>FARIDA </t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B244" s="0" t="inlineStr">
         <is>
-          <t>IBRAHIM</t>
+          <t>HASSAN</t>
         </is>
       </c>
       <c r="R244" s="0" t="inlineStr">
@@ -8261,7 +8236,7 @@
       </c>
       <c r="X244" s="0" t="inlineStr">
         <is>
-          <t>8500.00</t>
+          <t>26000.00</t>
         </is>
       </c>
       <c r="Z244" s="0" t="inlineStr">
@@ -8276,19 +8251,19 @@
       </c>
       <c r="AC244" s="0" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>326</t>
         </is>
       </c>
     </row>
     <row r="245" spans="1:29">
       <c r="A245" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B245" s="0" t="inlineStr">
         <is>
-          <t>IBRAHIM</t>
+          <t>HISHAM - ABK</t>
         </is>
       </c>
       <c r="R245" s="0" t="inlineStr">
@@ -8298,7 +8273,7 @@
       </c>
       <c r="X245" s="0" t="inlineStr">
         <is>
-          <t>35000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z245" s="0" t="inlineStr">
@@ -8313,24 +8288,19 @@
       </c>
       <c r="AC245" s="0" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>215</t>
         </is>
       </c>
     </row>
     <row r="246" spans="1:29">
       <c r="A246" s="0" t="inlineStr">
         <is>
-          <t>SALISU</t>
+          <t>MALAMA</t>
         </is>
       </c>
       <c r="B246" s="0" t="inlineStr">
         <is>
-          <t>IDRIS</t>
-        </is>
-      </c>
-      <c r="D246" s="0" t="inlineStr">
-        <is>
-          <t>08184133063</t>
+          <t>HUSSAINA</t>
         </is>
       </c>
       <c r="R246" s="0" t="inlineStr">
@@ -8340,7 +8310,7 @@
       </c>
       <c r="X246" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>590000.00</t>
         </is>
       </c>
       <c r="Z246" s="0" t="inlineStr">
@@ -8355,54 +8325,19 @@
       </c>
       <c r="AC246" s="0" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>141</t>
         </is>
       </c>
     </row>
     <row r="247" spans="1:29">
       <c r="A247" s="0" t="inlineStr">
         <is>
-          <t>Ibrahim BB</t>
+          <t>SA'ADATU </t>
         </is>
       </c>
       <c r="B247" s="0" t="inlineStr">
         <is>
-          <t>Jafar</t>
-        </is>
-      </c>
-      <c r="D247" s="0" t="inlineStr">
-        <is>
-          <t>08146595795</t>
-        </is>
-      </c>
-      <c r="J247" s="0" t="inlineStr">
-        <is>
-          <t>No 393 Rangi Quaters, Tudun Murtala, Nassarawa Kano</t>
-        </is>
-      </c>
-      <c r="L247" s="0" t="inlineStr">
-        <is>
-          <t>Kano</t>
-        </is>
-      </c>
-      <c r="M247" s="0" t="inlineStr">
-        <is>
-          <t>Kano</t>
-        </is>
-      </c>
-      <c r="N247" s="0" t="inlineStr">
-        <is>
-          <t>700281</t>
-        </is>
-      </c>
-      <c r="O247" s="0" t="inlineStr">
-        <is>
-          <t>Nigeria</t>
-        </is>
-      </c>
-      <c r="Q247" s="0" t="inlineStr">
-        <is>
-          <t>1522263645</t>
+          <t>HUSSAINI</t>
         </is>
       </c>
       <c r="R247" s="0" t="inlineStr">
@@ -8410,31 +8345,11 @@
           <t>y</t>
         </is>
       </c>
-      <c r="T247" s="0" t="inlineStr">
-        <is>
-          <t>Tahir General Merchant</t>
-        </is>
-      </c>
-      <c r="V247" s="0" t="inlineStr">
-        <is>
-          <t>High-value returning customer. Frequently purchases in bulk during seasonal periods. Offer priority support and notify early about new stock arrivals or discounts.</t>
-        </is>
-      </c>
-      <c r="W247" s="0" t="inlineStr">
-        <is>
-          <t>REGULAR customer, with less than 5% discounts on sales.</t>
-        </is>
-      </c>
       <c r="X247" s="0" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>
       </c>
-      <c r="Y247" s="0" t="inlineStr">
-        <is>
-          <t>50000000.00</t>
-        </is>
-      </c>
       <c r="Z247" s="0" t="inlineStr">
         <is>
           <t>n</t>
@@ -8447,19 +8362,19 @@
       </c>
       <c r="AC247" s="0" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>131</t>
         </is>
       </c>
     </row>
     <row r="248" spans="1:29">
       <c r="A248" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>UMRATU</t>
         </is>
       </c>
       <c r="B248" s="0" t="inlineStr">
         <is>
-          <t>JARMA</t>
+          <t>HUSSAINI</t>
         </is>
       </c>
       <c r="R248" s="0" t="inlineStr">
@@ -8484,19 +8399,19 @@
       </c>
       <c r="AC248" s="0" t="inlineStr">
         <is>
-          <t>274</t>
+          <t>322</t>
         </is>
       </c>
     </row>
     <row r="249" spans="1:29">
       <c r="A249" s="0" t="inlineStr">
         <is>
-          <t>SUMAYYA</t>
+          <t>FARIDA </t>
         </is>
       </c>
       <c r="B249" s="0" t="inlineStr">
         <is>
-          <t>JEGA</t>
+          <t>IBRAHIM</t>
         </is>
       </c>
       <c r="R249" s="0" t="inlineStr">
@@ -8506,7 +8421,7 @@
       </c>
       <c r="X249" s="0" t="inlineStr">
         <is>
-          <t>10000.00</t>
+          <t>8500.00</t>
         </is>
       </c>
       <c r="Z249" s="0" t="inlineStr">
@@ -8521,19 +8436,19 @@
       </c>
       <c r="AC249" s="0" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>224</t>
         </is>
       </c>
     </row>
     <row r="250" spans="1:29">
       <c r="A250" s="0" t="inlineStr">
         <is>
-          <t>PHIL</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B250" s="0" t="inlineStr">
         <is>
-          <t>JULIUS</t>
+          <t>IBRAHIM</t>
         </is>
       </c>
       <c r="R250" s="0" t="inlineStr">
@@ -8543,7 +8458,7 @@
       </c>
       <c r="X250" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>35000.00</t>
         </is>
       </c>
       <c r="Z250" s="0" t="inlineStr">
@@ -8558,19 +8473,24 @@
       </c>
       <c r="AC250" s="0" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>225</t>
         </is>
       </c>
     </row>
     <row r="251" spans="1:29">
       <c r="A251" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>SALISU</t>
         </is>
       </c>
       <c r="B251" s="0" t="inlineStr">
         <is>
-          <t>JUMARE</t>
+          <t>IDRIS</t>
+        </is>
+      </c>
+      <c r="D251" s="0" t="inlineStr">
+        <is>
+          <t>08184133063</t>
         </is>
       </c>
       <c r="R251" s="0" t="inlineStr">
@@ -8580,7 +8500,7 @@
       </c>
       <c r="X251" s="0" t="inlineStr">
         <is>
-          <t>298000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z251" s="0" t="inlineStr">
@@ -8595,29 +8515,54 @@
       </c>
       <c r="AC251" s="0" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>17</t>
         </is>
       </c>
     </row>
     <row r="252" spans="1:29">
       <c r="A252" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>Ibrahim BB</t>
         </is>
       </c>
       <c r="B252" s="0" t="inlineStr">
         <is>
-          <t>KADUNA</t>
+          <t>Jafar</t>
+        </is>
+      </c>
+      <c r="D252" s="0" t="inlineStr">
+        <is>
+          <t>08146595795</t>
+        </is>
+      </c>
+      <c r="J252" s="0" t="inlineStr">
+        <is>
+          <t>No 393 Rangi Quaters, Tudun Murtala, Nassarawa Kano</t>
         </is>
       </c>
       <c r="L252" s="0" t="inlineStr">
         <is>
-          <t>KADUNA</t>
+          <t>Kano</t>
         </is>
       </c>
       <c r="M252" s="0" t="inlineStr">
         <is>
-          <t>KADUNA</t>
+          <t>Kano</t>
+        </is>
+      </c>
+      <c r="N252" s="0" t="inlineStr">
+        <is>
+          <t>700281</t>
+        </is>
+      </c>
+      <c r="O252" s="0" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="Q252" s="0" t="inlineStr">
+        <is>
+          <t>1522263645</t>
         </is>
       </c>
       <c r="R252" s="0" t="inlineStr">
@@ -8625,9 +8570,29 @@
           <t>y</t>
         </is>
       </c>
+      <c r="T252" s="0" t="inlineStr">
+        <is>
+          <t>Tahir General Merchant</t>
+        </is>
+      </c>
+      <c r="V252" s="0" t="inlineStr">
+        <is>
+          <t>High-value returning customer. Frequently purchases in bulk during seasonal periods. Offer priority support and notify early about new stock arrivals or discounts.</t>
+        </is>
+      </c>
+      <c r="W252" s="0" t="inlineStr">
+        <is>
+          <t>REGULAR customer, with less than 5% discounts on sales.</t>
+        </is>
+      </c>
       <c r="X252" s="0" t="inlineStr">
         <is>
-          <t>151500.00</t>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="Y252" s="0" t="inlineStr">
+        <is>
+          <t>50000000.00</t>
         </is>
       </c>
       <c r="Z252" s="0" t="inlineStr">
@@ -8642,19 +8607,19 @@
       </c>
       <c r="AC252" s="0" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>31</t>
         </is>
       </c>
     </row>
     <row r="253" spans="1:29">
       <c r="A253" s="0" t="inlineStr">
         <is>
-          <t>HAJ FATIMA</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B253" s="0" t="inlineStr">
         <is>
-          <t>KADUNA</t>
+          <t>JARMA</t>
         </is>
       </c>
       <c r="R253" s="0" t="inlineStr">
@@ -8664,7 +8629,7 @@
       </c>
       <c r="X253" s="0" t="inlineStr">
         <is>
-          <t>582000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z253" s="0" t="inlineStr">
@@ -8679,19 +8644,19 @@
       </c>
       <c r="AC253" s="0" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>274</t>
         </is>
       </c>
     </row>
     <row r="254" spans="1:29">
       <c r="A254" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>SUMAYYA</t>
         </is>
       </c>
       <c r="B254" s="0" t="inlineStr">
         <is>
-          <t>KADUNA</t>
+          <t>JEGA</t>
         </is>
       </c>
       <c r="R254" s="0" t="inlineStr">
@@ -8701,7 +8666,7 @@
       </c>
       <c r="X254" s="0" t="inlineStr">
         <is>
-          <t>127500.00</t>
+          <t>10000.00</t>
         </is>
       </c>
       <c r="Z254" s="0" t="inlineStr">
@@ -8716,19 +8681,19 @@
       </c>
       <c r="AC254" s="0" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>114</t>
         </is>
       </c>
     </row>
     <row r="255" spans="1:29">
       <c r="A255" s="0" t="inlineStr">
         <is>
-          <t>SA'ADATU</t>
+          <t>PHIL</t>
         </is>
       </c>
       <c r="B255" s="0" t="inlineStr">
         <is>
-          <t>KANGIWA</t>
+          <t>JULIUS</t>
         </is>
       </c>
       <c r="R255" s="0" t="inlineStr">
@@ -8738,7 +8703,7 @@
       </c>
       <c r="X255" s="0" t="inlineStr">
         <is>
-          <t>200000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z255" s="0" t="inlineStr">
@@ -8753,19 +8718,19 @@
       </c>
       <c r="AC255" s="0" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>255</t>
         </is>
       </c>
     </row>
     <row r="256" spans="1:29">
       <c r="A256" s="0" t="inlineStr">
         <is>
-          <t>MOMY</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B256" s="0" t="inlineStr">
         <is>
-          <t>KARETO</t>
+          <t>JUMARE</t>
         </is>
       </c>
       <c r="R256" s="0" t="inlineStr">
@@ -8775,7 +8740,7 @@
       </c>
       <c r="X256" s="0" t="inlineStr">
         <is>
-          <t>240000.00</t>
+          <t>298000.00</t>
         </is>
       </c>
       <c r="Z256" s="0" t="inlineStr">
@@ -8790,19 +8755,29 @@
       </c>
       <c r="AC256" s="0" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>129</t>
         </is>
       </c>
     </row>
     <row r="257" spans="1:29">
       <c r="A257" s="0" t="inlineStr">
         <is>
-          <t>JIDDAH</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B257" s="0" t="inlineStr">
         <is>
-          <t>KATSINA</t>
+          <t>KADUNA</t>
+        </is>
+      </c>
+      <c r="L257" s="0" t="inlineStr">
+        <is>
+          <t>KADUNA</t>
+        </is>
+      </c>
+      <c r="M257" s="0" t="inlineStr">
+        <is>
+          <t>KADUNA</t>
         </is>
       </c>
       <c r="R257" s="0" t="inlineStr">
@@ -8812,7 +8787,7 @@
       </c>
       <c r="X257" s="0" t="inlineStr">
         <is>
-          <t>45000.00</t>
+          <t>397500.00</t>
         </is>
       </c>
       <c r="Z257" s="0" t="inlineStr">
@@ -8827,19 +8802,19 @@
       </c>
       <c r="AC257" s="0" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>82</t>
         </is>
       </c>
     </row>
     <row r="258" spans="1:29">
       <c r="A258" s="0" t="inlineStr">
         <is>
-          <t>ANTY FATIMA</t>
+          <t>HAJ FATIMA</t>
         </is>
       </c>
       <c r="B258" s="0" t="inlineStr">
         <is>
-          <t>KATSINA</t>
+          <t>KADUNA</t>
         </is>
       </c>
       <c r="R258" s="0" t="inlineStr">
@@ -8849,7 +8824,7 @@
       </c>
       <c r="X258" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>630500.00</t>
         </is>
       </c>
       <c r="Z258" s="0" t="inlineStr">
@@ -8864,19 +8839,19 @@
       </c>
       <c r="AC258" s="0" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>91</t>
         </is>
       </c>
     </row>
     <row r="259" spans="1:29">
       <c r="A259" s="0" t="inlineStr">
         <is>
-          <t>HAJ ZAINAB</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B259" s="0" t="inlineStr">
         <is>
-          <t>KATSINA</t>
+          <t>KADUNA</t>
         </is>
       </c>
       <c r="R259" s="0" t="inlineStr">
@@ -8886,7 +8861,7 @@
       </c>
       <c r="X259" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>127500.00</t>
         </is>
       </c>
       <c r="Z259" s="0" t="inlineStr">
@@ -8901,19 +8876,19 @@
       </c>
       <c r="AC259" s="0" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>95</t>
         </is>
       </c>
     </row>
     <row r="260" spans="1:29">
       <c r="A260" s="0" t="inlineStr">
         <is>
-          <t>HAJ HADIZA</t>
+          <t>SA'ADATU</t>
         </is>
       </c>
       <c r="B260" s="0" t="inlineStr">
         <is>
-          <t>KATSINA</t>
+          <t>KANGIWA</t>
         </is>
       </c>
       <c r="R260" s="0" t="inlineStr">
@@ -8923,7 +8898,7 @@
       </c>
       <c r="X260" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>200000.00</t>
         </is>
       </c>
       <c r="Z260" s="0" t="inlineStr">
@@ -8938,19 +8913,19 @@
       </c>
       <c r="AC260" s="0" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>109</t>
         </is>
       </c>
     </row>
     <row r="261" spans="1:29">
       <c r="A261" s="0" t="inlineStr">
         <is>
-          <t>SUMAYYA</t>
+          <t>MOMY</t>
         </is>
       </c>
       <c r="B261" s="0" t="inlineStr">
         <is>
-          <t>KATSINA</t>
+          <t>KARETO</t>
         </is>
       </c>
       <c r="R261" s="0" t="inlineStr">
@@ -8960,7 +8935,7 @@
       </c>
       <c r="X261" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>240000.00</t>
         </is>
       </c>
       <c r="Z261" s="0" t="inlineStr">
@@ -8975,14 +8950,14 @@
       </c>
       <c r="AC261" s="0" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>157</t>
         </is>
       </c>
     </row>
     <row r="262" spans="1:29">
       <c r="A262" s="0" t="inlineStr">
         <is>
-          <t>HADIZA</t>
+          <t>JIDDAH</t>
         </is>
       </c>
       <c r="B262" s="0" t="inlineStr">
@@ -8997,7 +8972,7 @@
       </c>
       <c r="X262" s="0" t="inlineStr">
         <is>
-          <t>12000.00</t>
+          <t>45000.00</t>
         </is>
       </c>
       <c r="Z262" s="0" t="inlineStr">
@@ -9012,19 +8987,19 @@
       </c>
       <c r="AC262" s="0" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>77</t>
         </is>
       </c>
     </row>
     <row r="263" spans="1:29">
       <c r="A263" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>ANTY FATIMA</t>
         </is>
       </c>
       <c r="B263" s="0" t="inlineStr">
         <is>
-          <t>KAUSAR</t>
+          <t>KATSINA</t>
         </is>
       </c>
       <c r="R263" s="0" t="inlineStr">
@@ -9049,19 +9024,19 @@
       </c>
       <c r="AC263" s="0" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="264" spans="1:29">
       <c r="A264" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>HAJ ZAINAB</t>
         </is>
       </c>
       <c r="B264" s="0" t="inlineStr">
         <is>
-          <t>KHALIFA KATSINA</t>
+          <t>KATSINA</t>
         </is>
       </c>
       <c r="R264" s="0" t="inlineStr">
@@ -9071,7 +9046,7 @@
       </c>
       <c r="X264" s="0" t="inlineStr">
         <is>
-          <t>324500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z264" s="0" t="inlineStr">
@@ -9086,19 +9061,19 @@
       </c>
       <c r="AC264" s="0" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>92</t>
         </is>
       </c>
     </row>
     <row r="265" spans="1:29">
       <c r="A265" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>HAJ HADIZA</t>
         </is>
       </c>
       <c r="B265" s="0" t="inlineStr">
         <is>
-          <t>KOLMANI</t>
+          <t>KATSINA</t>
         </is>
       </c>
       <c r="R265" s="0" t="inlineStr">
@@ -9108,7 +9083,7 @@
       </c>
       <c r="X265" s="0" t="inlineStr">
         <is>
-          <t>40000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z265" s="0" t="inlineStr">
@@ -9123,19 +9098,19 @@
       </c>
       <c r="AC265" s="0" t="inlineStr">
         <is>
-          <t>205</t>
+          <t>108</t>
         </is>
       </c>
     </row>
     <row r="266" spans="1:29">
       <c r="A266" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>SUMAYYA</t>
         </is>
       </c>
       <c r="B266" s="0" t="inlineStr">
         <is>
-          <t>KWAIRANGA</t>
+          <t>KATSINA</t>
         </is>
       </c>
       <c r="R266" s="0" t="inlineStr">
@@ -9145,7 +9120,7 @@
       </c>
       <c r="X266" s="0" t="inlineStr">
         <is>
-          <t>1469000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z266" s="0" t="inlineStr">
@@ -9160,19 +9135,19 @@
       </c>
       <c r="AC266" s="0" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>186</t>
         </is>
       </c>
     </row>
     <row r="267" spans="1:29">
       <c r="A267" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>HADIZA</t>
         </is>
       </c>
       <c r="B267" s="0" t="inlineStr">
         <is>
-          <t>KYARI</t>
+          <t>KATSINA</t>
         </is>
       </c>
       <c r="R267" s="0" t="inlineStr">
@@ -9182,7 +9157,7 @@
       </c>
       <c r="X267" s="0" t="inlineStr">
         <is>
-          <t>40000.00</t>
+          <t>12000.00</t>
         </is>
       </c>
       <c r="Z267" s="0" t="inlineStr">
@@ -9197,19 +9172,19 @@
       </c>
       <c r="AC267" s="0" t="inlineStr">
         <is>
-          <t>292</t>
+          <t>213</t>
         </is>
       </c>
     </row>
     <row r="268" spans="1:29">
       <c r="A268" s="0" t="inlineStr">
         <is>
-          <t>HADIZA</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B268" s="0" t="inlineStr">
         <is>
-          <t>LABO</t>
+          <t>KAUSAR</t>
         </is>
       </c>
       <c r="R268" s="0" t="inlineStr">
@@ -9219,7 +9194,7 @@
       </c>
       <c r="X268" s="0" t="inlineStr">
         <is>
-          <t>1056900.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z268" s="0" t="inlineStr">
@@ -9234,19 +9209,19 @@
       </c>
       <c r="AC268" s="0" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>160</t>
         </is>
       </c>
     </row>
     <row r="269" spans="1:29">
       <c r="A269" s="0" t="inlineStr">
         <is>
-          <t>UMMI</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B269" s="0" t="inlineStr">
         <is>
-          <t>LABO</t>
+          <t>KHALIFA KATSINA</t>
         </is>
       </c>
       <c r="R269" s="0" t="inlineStr">
@@ -9256,7 +9231,7 @@
       </c>
       <c r="X269" s="0" t="inlineStr">
         <is>
-          <t>1678300.00</t>
+          <t>324500.00</t>
         </is>
       </c>
       <c r="Z269" s="0" t="inlineStr">
@@ -9271,19 +9246,19 @@
       </c>
       <c r="AC269" s="0" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>106</t>
         </is>
       </c>
     </row>
     <row r="270" spans="1:29">
       <c r="A270" s="0" t="inlineStr">
         <is>
-          <t>INNAN</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B270" s="0" t="inlineStr">
         <is>
-          <t>LARAI</t>
+          <t>KOLMANI</t>
         </is>
       </c>
       <c r="R270" s="0" t="inlineStr">
@@ -9293,7 +9268,7 @@
       </c>
       <c r="X270" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>40000.00</t>
         </is>
       </c>
       <c r="Z270" s="0" t="inlineStr">
@@ -9308,19 +9283,19 @@
       </c>
       <c r="AC270" s="0" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>205</t>
         </is>
       </c>
     </row>
     <row r="271" spans="1:29">
       <c r="A271" s="0" t="inlineStr">
         <is>
-          <t>RAHAMA</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B271" s="0" t="inlineStr">
         <is>
-          <t>LAWAL</t>
+          <t>KWAIRANGA</t>
         </is>
       </c>
       <c r="R271" s="0" t="inlineStr">
@@ -9330,7 +9305,7 @@
       </c>
       <c r="X271" s="0" t="inlineStr">
         <is>
-          <t>35000.00</t>
+          <t>1469000.00</t>
         </is>
       </c>
       <c r="Z271" s="0" t="inlineStr">
@@ -9345,19 +9320,19 @@
       </c>
       <c r="AC271" s="0" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>104</t>
         </is>
       </c>
     </row>
     <row r="272" spans="1:29">
       <c r="A272" s="0" t="inlineStr">
         <is>
-          <t>HAJ HADIZA</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B272" s="0" t="inlineStr">
         <is>
-          <t>LAWAL</t>
+          <t>KYARI</t>
         </is>
       </c>
       <c r="R272" s="0" t="inlineStr">
@@ -9367,7 +9342,7 @@
       </c>
       <c r="X272" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>40000.00</t>
         </is>
       </c>
       <c r="Z272" s="0" t="inlineStr">
@@ -9382,19 +9357,19 @@
       </c>
       <c r="AC272" s="0" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>292</t>
         </is>
       </c>
     </row>
     <row r="273" spans="1:29">
       <c r="A273" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>HADIZA</t>
         </is>
       </c>
       <c r="B273" s="0" t="inlineStr">
         <is>
-          <t>MACHINA</t>
+          <t>LABO</t>
         </is>
       </c>
       <c r="R273" s="0" t="inlineStr">
@@ -9404,7 +9379,7 @@
       </c>
       <c r="X273" s="0" t="inlineStr">
         <is>
-          <t>116000.00</t>
+          <t>1056900.00</t>
         </is>
       </c>
       <c r="Z273" s="0" t="inlineStr">
@@ -9419,19 +9394,19 @@
       </c>
       <c r="AC273" s="0" t="inlineStr">
         <is>
-          <t>296</t>
+          <t>88</t>
         </is>
       </c>
     </row>
     <row r="274" spans="1:29">
       <c r="A274" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>UMMI</t>
         </is>
       </c>
       <c r="B274" s="0" t="inlineStr">
         <is>
-          <t>MADU</t>
+          <t>LABO</t>
         </is>
       </c>
       <c r="R274" s="0" t="inlineStr">
@@ -9441,7 +9416,7 @@
       </c>
       <c r="X274" s="0" t="inlineStr">
         <is>
-          <t>48000.00</t>
+          <t>1678300.00</t>
         </is>
       </c>
       <c r="Z274" s="0" t="inlineStr">
@@ -9456,19 +9431,19 @@
       </c>
       <c r="AC274" s="0" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>119</t>
         </is>
       </c>
     </row>
     <row r="275" spans="1:29">
       <c r="A275" s="0" t="inlineStr">
         <is>
-          <t>RAHAMA</t>
+          <t>INNAN</t>
         </is>
       </c>
       <c r="B275" s="0" t="inlineStr">
         <is>
-          <t>MAHMUD</t>
+          <t>LARAI</t>
         </is>
       </c>
       <c r="R275" s="0" t="inlineStr">
@@ -9493,19 +9468,19 @@
       </c>
       <c r="AC275" s="0" t="inlineStr">
         <is>
-          <t>311</t>
+          <t>84</t>
         </is>
       </c>
     </row>
     <row r="276" spans="1:29">
       <c r="A276" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>RAHAMA</t>
         </is>
       </c>
       <c r="B276" s="0" t="inlineStr">
         <is>
-          <t>MAIGARI</t>
+          <t>LAWAL</t>
         </is>
       </c>
       <c r="R276" s="0" t="inlineStr">
@@ -9515,7 +9490,7 @@
       </c>
       <c r="X276" s="0" t="inlineStr">
         <is>
-          <t>2261300.00</t>
+          <t>35000.00</t>
         </is>
       </c>
       <c r="Z276" s="0" t="inlineStr">
@@ -9530,19 +9505,19 @@
       </c>
       <c r="AC276" s="0" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>80</t>
         </is>
       </c>
     </row>
     <row r="277" spans="1:29">
       <c r="A277" s="0" t="inlineStr">
         <is>
-          <t>ZUWAIRA</t>
+          <t>HAJ HADIZA</t>
         </is>
       </c>
       <c r="B277" s="0" t="inlineStr">
         <is>
-          <t>MAJIDADI</t>
+          <t>LAWAL</t>
         </is>
       </c>
       <c r="R277" s="0" t="inlineStr">
@@ -9552,7 +9527,7 @@
       </c>
       <c r="X277" s="0" t="inlineStr">
         <is>
-          <t>74800.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z277" s="0" t="inlineStr">
@@ -9567,19 +9542,19 @@
       </c>
       <c r="AC277" s="0" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>310</t>
         </is>
       </c>
     </row>
     <row r="278" spans="1:29">
       <c r="A278" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B278" s="0" t="inlineStr">
         <is>
-          <t>MALAM</t>
+          <t>MACHINA</t>
         </is>
       </c>
       <c r="R278" s="0" t="inlineStr">
@@ -9589,7 +9564,7 @@
       </c>
       <c r="X278" s="0" t="inlineStr">
         <is>
-          <t>26500.00</t>
+          <t>136000.00</t>
         </is>
       </c>
       <c r="Z278" s="0" t="inlineStr">
@@ -9604,7 +9579,7 @@
       </c>
       <c r="AC278" s="0" t="inlineStr">
         <is>
-          <t>316</t>
+          <t>296</t>
         </is>
       </c>
     </row>
@@ -9616,7 +9591,7 @@
       </c>
       <c r="B279" s="0" t="inlineStr">
         <is>
-          <t>MALUMFASHI</t>
+          <t>MADU</t>
         </is>
       </c>
       <c r="R279" s="0" t="inlineStr">
@@ -9626,7 +9601,7 @@
       </c>
       <c r="X279" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>48000.00</t>
         </is>
       </c>
       <c r="Z279" s="0" t="inlineStr">
@@ -9641,19 +9616,19 @@
       </c>
       <c r="AC279" s="0" t="inlineStr">
         <is>
-          <t>124</t>
+          <t>151</t>
         </is>
       </c>
     </row>
     <row r="280" spans="1:29">
       <c r="A280" s="0" t="inlineStr">
         <is>
-          <t>DJA</t>
+          <t>RAHAMA</t>
         </is>
       </c>
       <c r="B280" s="0" t="inlineStr">
         <is>
-          <t>MAMAN ABDALLAH</t>
+          <t>MAHMUD</t>
         </is>
       </c>
       <c r="R280" s="0" t="inlineStr">
@@ -9663,7 +9638,7 @@
       </c>
       <c r="X280" s="0" t="inlineStr">
         <is>
-          <t>147000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z280" s="0" t="inlineStr">
@@ -9678,19 +9653,19 @@
       </c>
       <c r="AC280" s="0" t="inlineStr">
         <is>
-          <t>178</t>
+          <t>311</t>
         </is>
       </c>
     </row>
     <row r="281" spans="1:29">
       <c r="A281" s="0" t="inlineStr">
         <is>
-          <t>UMMU</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B281" s="0" t="inlineStr">
         <is>
-          <t>MAMAN UWAIS</t>
+          <t>MAIGARI</t>
         </is>
       </c>
       <c r="R281" s="0" t="inlineStr">
@@ -9700,7 +9675,7 @@
       </c>
       <c r="X281" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>2498300.00</t>
         </is>
       </c>
       <c r="Z281" s="0" t="inlineStr">
@@ -9715,19 +9690,19 @@
       </c>
       <c r="AC281" s="0" t="inlineStr">
         <is>
-          <t>271</t>
+          <t>162</t>
         </is>
       </c>
     </row>
     <row r="282" spans="1:29">
       <c r="A282" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>ZUWAIRA</t>
         </is>
       </c>
       <c r="B282" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>MAJIDADI</t>
         </is>
       </c>
       <c r="R282" s="0" t="inlineStr">
@@ -9737,7 +9712,7 @@
       </c>
       <c r="X282" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>74800.00</t>
         </is>
       </c>
       <c r="Z282" s="0" t="inlineStr">
@@ -9752,19 +9727,19 @@
       </c>
       <c r="AC282" s="0" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>207</t>
         </is>
       </c>
     </row>
     <row r="283" spans="1:29">
       <c r="A283" s="0" t="inlineStr">
         <is>
-          <t>HAJ FATIMA</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B283" s="0" t="inlineStr">
         <is>
-          <t>MUHD</t>
+          <t>MALAM</t>
         </is>
       </c>
       <c r="R283" s="0" t="inlineStr">
@@ -9774,7 +9749,7 @@
       </c>
       <c r="X283" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>26500.00</t>
         </is>
       </c>
       <c r="Z283" s="0" t="inlineStr">
@@ -9789,19 +9764,19 @@
       </c>
       <c r="AC283" s="0" t="inlineStr">
         <is>
-          <t>247</t>
+          <t>316</t>
         </is>
       </c>
     </row>
     <row r="284" spans="1:29">
       <c r="A284" s="0" t="inlineStr">
         <is>
-          <t>SHAMSIYYAH</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B284" s="0" t="inlineStr">
         <is>
-          <t>MUHD</t>
+          <t>MALUMFASHI</t>
         </is>
       </c>
       <c r="R284" s="0" t="inlineStr">
@@ -9826,19 +9801,19 @@
       </c>
       <c r="AC284" s="0" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>124</t>
         </is>
       </c>
     </row>
     <row r="285" spans="1:29">
       <c r="A285" s="0" t="inlineStr">
         <is>
-          <t>BILKISU</t>
+          <t>DJA</t>
         </is>
       </c>
       <c r="B285" s="0" t="inlineStr">
         <is>
-          <t>MUKHTAR</t>
+          <t>MAMAN ABDALLAH</t>
         </is>
       </c>
       <c r="R285" s="0" t="inlineStr">
@@ -9848,7 +9823,7 @@
       </c>
       <c r="X285" s="0" t="inlineStr">
         <is>
-          <t>173000.00</t>
+          <t>147000.00</t>
         </is>
       </c>
       <c r="Z285" s="0" t="inlineStr">
@@ -9863,19 +9838,19 @@
       </c>
       <c r="AC285" s="0" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>178</t>
         </is>
       </c>
     </row>
     <row r="286" spans="1:29">
       <c r="A286" s="0" t="inlineStr">
         <is>
-          <t>UMMI</t>
+          <t>UMMU</t>
         </is>
       </c>
       <c r="B286" s="0" t="inlineStr">
         <is>
-          <t>MUMTAZ</t>
+          <t>MAMAN UWAIS</t>
         </is>
       </c>
       <c r="R286" s="0" t="inlineStr">
@@ -9885,7 +9860,7 @@
       </c>
       <c r="X286" s="0" t="inlineStr">
         <is>
-          <t>2507000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z286" s="0" t="inlineStr">
@@ -9900,19 +9875,19 @@
       </c>
       <c r="AC286" s="0" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>271</t>
         </is>
       </c>
     </row>
     <row r="287" spans="1:29">
       <c r="A287" s="0" t="inlineStr">
         <is>
-          <t>MAMAN </t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B287" s="0" t="inlineStr">
         <is>
-          <t>NABILA</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="R287" s="0" t="inlineStr">
@@ -9937,19 +9912,19 @@
       </c>
       <c r="AC287" s="0" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>94</t>
         </is>
       </c>
     </row>
     <row r="288" spans="1:29">
       <c r="A288" s="0" t="inlineStr">
         <is>
-          <t>ANTY</t>
+          <t>HAJ FATIMA</t>
         </is>
       </c>
       <c r="B288" s="0" t="inlineStr">
         <is>
-          <t>NAS</t>
+          <t>MUHD</t>
         </is>
       </c>
       <c r="R288" s="0" t="inlineStr">
@@ -9959,7 +9934,7 @@
       </c>
       <c r="X288" s="0" t="inlineStr">
         <is>
-          <t>1579000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z288" s="0" t="inlineStr">
@@ -9974,19 +9949,19 @@
       </c>
       <c r="AC288" s="0" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>247</t>
         </is>
       </c>
     </row>
     <row r="289" spans="1:29">
       <c r="A289" s="0" t="inlineStr">
         <is>
-          <t>RUKAYYA</t>
+          <t>SHAMSIYYAH</t>
         </is>
       </c>
       <c r="B289" s="0" t="inlineStr">
         <is>
-          <t>NASIR</t>
+          <t>MUHD</t>
         </is>
       </c>
       <c r="R289" s="0" t="inlineStr">
@@ -9996,7 +9971,7 @@
       </c>
       <c r="X289" s="0" t="inlineStr">
         <is>
-          <t>402000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z289" s="0" t="inlineStr">
@@ -10011,19 +9986,19 @@
       </c>
       <c r="AC289" s="0" t="inlineStr">
         <is>
-          <t>188</t>
+          <t>257</t>
         </is>
       </c>
     </row>
     <row r="290" spans="1:29">
       <c r="A290" s="0" t="inlineStr">
         <is>
-          <t>HAFSAT</t>
+          <t>BILKISU</t>
         </is>
       </c>
       <c r="B290" s="0" t="inlineStr">
         <is>
-          <t>NASIR</t>
+          <t>MUKHTAR</t>
         </is>
       </c>
       <c r="R290" s="0" t="inlineStr">
@@ -10033,7 +10008,7 @@
       </c>
       <c r="X290" s="0" t="inlineStr">
         <is>
-          <t>22000.00</t>
+          <t>173000.00</t>
         </is>
       </c>
       <c r="Z290" s="0" t="inlineStr">
@@ -10048,19 +10023,19 @@
       </c>
       <c r="AC290" s="0" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>138</t>
         </is>
       </c>
     </row>
     <row r="291" spans="1:29">
       <c r="A291" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>UMMI</t>
         </is>
       </c>
       <c r="B291" s="0" t="inlineStr">
         <is>
-          <t>NATA'ALA</t>
+          <t>MUMTAZ</t>
         </is>
       </c>
       <c r="R291" s="0" t="inlineStr">
@@ -10070,7 +10045,7 @@
       </c>
       <c r="X291" s="0" t="inlineStr">
         <is>
-          <t>33000.00</t>
+          <t>3419000.00</t>
         </is>
       </c>
       <c r="Z291" s="0" t="inlineStr">
@@ -10085,19 +10060,19 @@
       </c>
       <c r="AC291" s="0" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>140</t>
         </is>
       </c>
     </row>
     <row r="292" spans="1:29">
       <c r="A292" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>MAMAN </t>
         </is>
       </c>
       <c r="B292" s="0" t="inlineStr">
         <is>
-          <t>NINGI</t>
+          <t>NABILA</t>
         </is>
       </c>
       <c r="R292" s="0" t="inlineStr">
@@ -10122,19 +10097,19 @@
       </c>
       <c r="AC292" s="0" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>87</t>
         </is>
       </c>
     </row>
     <row r="293" spans="1:29">
       <c r="A293" s="0" t="inlineStr">
         <is>
-          <t>BILKIS</t>
+          <t>ANTY</t>
         </is>
       </c>
       <c r="B293" s="0" t="inlineStr">
         <is>
-          <t>ONLINE</t>
+          <t>NAS</t>
         </is>
       </c>
       <c r="R293" s="0" t="inlineStr">
@@ -10144,7 +10119,7 @@
       </c>
       <c r="X293" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1579000.00</t>
         </is>
       </c>
       <c r="Z293" s="0" t="inlineStr">
@@ -10159,19 +10134,19 @@
       </c>
       <c r="AC293" s="0" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>78</t>
         </is>
       </c>
     </row>
     <row r="294" spans="1:29">
       <c r="A294" s="0" t="inlineStr">
         <is>
-          <t>MADAM</t>
+          <t>RUKAYYA</t>
         </is>
       </c>
       <c r="B294" s="0" t="inlineStr">
         <is>
-          <t>RONKE</t>
+          <t>NASIR</t>
         </is>
       </c>
       <c r="R294" s="0" t="inlineStr">
@@ -10181,7 +10156,7 @@
       </c>
       <c r="X294" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>516000.00</t>
         </is>
       </c>
       <c r="Z294" s="0" t="inlineStr">
@@ -10196,19 +10171,19 @@
       </c>
       <c r="AC294" s="0" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>188</t>
         </is>
       </c>
     </row>
     <row r="295" spans="1:29">
       <c r="A295" s="0" t="inlineStr">
         <is>
-          <t>ASH</t>
+          <t>HAFSAT</t>
         </is>
       </c>
       <c r="B295" s="0" t="inlineStr">
         <is>
-          <t>RUKY</t>
+          <t>NASIR</t>
         </is>
       </c>
       <c r="R295" s="0" t="inlineStr">
@@ -10218,7 +10193,7 @@
       </c>
       <c r="X295" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>22000.00</t>
         </is>
       </c>
       <c r="Z295" s="0" t="inlineStr">
@@ -10233,19 +10208,19 @@
       </c>
       <c r="AC295" s="0" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>228</t>
         </is>
       </c>
     </row>
     <row r="296" spans="1:29">
       <c r="A296" s="0" t="inlineStr">
         <is>
-          <t>IKILIMA</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B296" s="0" t="inlineStr">
         <is>
-          <t>RUWAN DORAWA</t>
+          <t>NATA'ALA</t>
         </is>
       </c>
       <c r="R296" s="0" t="inlineStr">
@@ -10255,7 +10230,7 @@
       </c>
       <c r="X296" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>33000.00</t>
         </is>
       </c>
       <c r="Z296" s="0" t="inlineStr">
@@ -10270,19 +10245,19 @@
       </c>
       <c r="AC296" s="0" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>74</t>
         </is>
       </c>
     </row>
     <row r="297" spans="1:29">
       <c r="A297" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B297" s="0" t="inlineStr">
         <is>
-          <t>SAFWAN</t>
+          <t>NINGI</t>
         </is>
       </c>
       <c r="R297" s="0" t="inlineStr">
@@ -10292,7 +10267,7 @@
       </c>
       <c r="X297" s="0" t="inlineStr">
         <is>
-          <t>32000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z297" s="0" t="inlineStr">
@@ -10307,19 +10282,19 @@
       </c>
       <c r="AC297" s="0" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>132</t>
         </is>
       </c>
     </row>
     <row r="298" spans="1:29">
       <c r="A298" s="0" t="inlineStr">
         <is>
-          <t>SALMA</t>
+          <t>BILKIS</t>
         </is>
       </c>
       <c r="B298" s="0" t="inlineStr">
         <is>
-          <t>SALMUR</t>
+          <t>ONLINE</t>
         </is>
       </c>
       <c r="R298" s="0" t="inlineStr">
@@ -10329,7 +10304,7 @@
       </c>
       <c r="X298" s="0" t="inlineStr">
         <is>
-          <t>47500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z298" s="0" t="inlineStr">
@@ -10344,19 +10319,19 @@
       </c>
       <c r="AC298" s="0" t="inlineStr">
         <is>
-          <t>254</t>
+          <t>170</t>
         </is>
       </c>
     </row>
     <row r="299" spans="1:29">
       <c r="A299" s="0" t="inlineStr">
         <is>
-          <t>ASMI</t>
+          <t>MADAM</t>
         </is>
       </c>
       <c r="B299" s="0" t="inlineStr">
         <is>
-          <t>SAMBO</t>
+          <t>RONKE</t>
         </is>
       </c>
       <c r="R299" s="0" t="inlineStr">
@@ -10381,19 +10356,19 @@
       </c>
       <c r="AC299" s="0" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>226</t>
         </is>
       </c>
     </row>
     <row r="300" spans="1:29">
       <c r="A300" s="0" t="inlineStr">
         <is>
-          <t>SAMIHA</t>
+          <t>ASH</t>
         </is>
       </c>
       <c r="B300" s="0" t="inlineStr">
         <is>
-          <t>SANI</t>
+          <t>RUKY</t>
         </is>
       </c>
       <c r="R300" s="0" t="inlineStr">
@@ -10418,19 +10393,19 @@
       </c>
       <c r="AC300" s="0" t="inlineStr">
         <is>
-          <t>285</t>
+          <t>76</t>
         </is>
       </c>
     </row>
     <row r="301" spans="1:29">
       <c r="A301" s="0" t="inlineStr">
         <is>
-          <t>JAMILA</t>
+          <t>IKILIMA</t>
         </is>
       </c>
       <c r="B301" s="0" t="inlineStr">
         <is>
-          <t>SHANONO</t>
+          <t>RUWAN DORAWA</t>
         </is>
       </c>
       <c r="R301" s="0" t="inlineStr">
@@ -10440,7 +10415,7 @@
       </c>
       <c r="X301" s="0" t="inlineStr">
         <is>
-          <t>443000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z301" s="0" t="inlineStr">
@@ -10455,19 +10430,19 @@
       </c>
       <c r="AC301" s="0" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>139</t>
         </is>
       </c>
     </row>
     <row r="302" spans="1:29">
       <c r="A302" s="0" t="inlineStr">
         <is>
-          <t>FARIDA</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B302" s="0" t="inlineStr">
         <is>
-          <t>SHARADA</t>
+          <t>SAFWAN</t>
         </is>
       </c>
       <c r="R302" s="0" t="inlineStr">
@@ -10477,7 +10452,7 @@
       </c>
       <c r="X302" s="0" t="inlineStr">
         <is>
-          <t>95000.00</t>
+          <t>32000.00</t>
         </is>
       </c>
       <c r="Z302" s="0" t="inlineStr">
@@ -10492,19 +10467,19 @@
       </c>
       <c r="AC302" s="0" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>105</t>
         </is>
       </c>
     </row>
     <row r="303" spans="1:29">
       <c r="A303" s="0" t="inlineStr">
         <is>
-          <t>FANNE</t>
+          <t>SALMA</t>
         </is>
       </c>
       <c r="B303" s="0" t="inlineStr">
         <is>
-          <t>SHARIF</t>
+          <t>SALMUR</t>
         </is>
       </c>
       <c r="R303" s="0" t="inlineStr">
@@ -10514,7 +10489,7 @@
       </c>
       <c r="X303" s="0" t="inlineStr">
         <is>
-          <t>350000.00</t>
+          <t>47500.00</t>
         </is>
       </c>
       <c r="Z303" s="0" t="inlineStr">
@@ -10529,19 +10504,19 @@
       </c>
       <c r="AC303" s="0" t="inlineStr">
         <is>
-          <t>179</t>
+          <t>254</t>
         </is>
       </c>
     </row>
     <row r="304" spans="1:29">
       <c r="A304" s="0" t="inlineStr">
         <is>
-          <t>SAMIRA</t>
+          <t>ASMI</t>
         </is>
       </c>
       <c r="B304" s="0" t="inlineStr">
         <is>
-          <t>SHIRA</t>
+          <t>SAMBO</t>
         </is>
       </c>
       <c r="R304" s="0" t="inlineStr">
@@ -10551,7 +10526,7 @@
       </c>
       <c r="X304" s="0" t="inlineStr">
         <is>
-          <t>156000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z304" s="0" t="inlineStr">
@@ -10566,19 +10541,19 @@
       </c>
       <c r="AC304" s="0" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>243</t>
         </is>
       </c>
     </row>
     <row r="305" spans="1:29">
       <c r="A305" s="0" t="inlineStr">
         <is>
-          <t>FATIMA </t>
+          <t>SAMIHA</t>
         </is>
       </c>
       <c r="B305" s="0" t="inlineStr">
         <is>
-          <t>SIDI</t>
+          <t>SANI</t>
         </is>
       </c>
       <c r="R305" s="0" t="inlineStr">
@@ -10588,7 +10563,7 @@
       </c>
       <c r="X305" s="0" t="inlineStr">
         <is>
-          <t>40000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z305" s="0" t="inlineStr">
@@ -10603,19 +10578,19 @@
       </c>
       <c r="AC305" s="0" t="inlineStr">
         <is>
-          <t>313</t>
+          <t>285</t>
         </is>
       </c>
     </row>
     <row r="306" spans="1:29">
       <c r="A306" s="0" t="inlineStr">
         <is>
-          <t>HADIZA</t>
+          <t>JAMILA</t>
         </is>
       </c>
       <c r="B306" s="0" t="inlineStr">
         <is>
-          <t>SOKOTO</t>
+          <t>SHANONO</t>
         </is>
       </c>
       <c r="R306" s="0" t="inlineStr">
@@ -10625,7 +10600,7 @@
       </c>
       <c r="X306" s="0" t="inlineStr">
         <is>
-          <t>852500.00</t>
+          <t>443000.00</t>
         </is>
       </c>
       <c r="Z306" s="0" t="inlineStr">
@@ -10640,7 +10615,7 @@
       </c>
       <c r="AC306" s="0" t="inlineStr">
         <is>
-          <t>118</t>
+          <t>83</t>
         </is>
       </c>
     </row>
@@ -10652,7 +10627,7 @@
       </c>
       <c r="B307" s="0" t="inlineStr">
         <is>
-          <t>SULAIMAN</t>
+          <t>SHARADA</t>
         </is>
       </c>
       <c r="R307" s="0" t="inlineStr">
@@ -10662,7 +10637,7 @@
       </c>
       <c r="X307" s="0" t="inlineStr">
         <is>
-          <t>80000.00</t>
+          <t>95000.00</t>
         </is>
       </c>
       <c r="Z307" s="0" t="inlineStr">
@@ -10677,19 +10652,19 @@
       </c>
       <c r="AC307" s="0" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>115</t>
         </is>
       </c>
     </row>
     <row r="308" spans="1:29">
       <c r="A308" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>FANNE</t>
         </is>
       </c>
       <c r="B308" s="0" t="inlineStr">
         <is>
-          <t>TRENDY</t>
+          <t>SHARIF</t>
         </is>
       </c>
       <c r="R308" s="0" t="inlineStr">
@@ -10699,7 +10674,7 @@
       </c>
       <c r="X308" s="0" t="inlineStr">
         <is>
-          <t>110500.00</t>
+          <t>350000.00</t>
         </is>
       </c>
       <c r="Z308" s="0" t="inlineStr">
@@ -10714,19 +10689,19 @@
       </c>
       <c r="AC308" s="0" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>179</t>
         </is>
       </c>
     </row>
     <row r="309" spans="1:29">
       <c r="A309" s="0" t="inlineStr">
         <is>
-          <t>JAMILA</t>
+          <t>SAMIRA</t>
         </is>
       </c>
       <c r="B309" s="0" t="inlineStr">
         <is>
-          <t>TUKUR</t>
+          <t>SHIRA</t>
         </is>
       </c>
       <c r="R309" s="0" t="inlineStr">
@@ -10736,7 +10711,7 @@
       </c>
       <c r="X309" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>156000.00</t>
         </is>
       </c>
       <c r="Z309" s="0" t="inlineStr">
@@ -10751,19 +10726,19 @@
       </c>
       <c r="AC309" s="0" t="inlineStr">
         <is>
-          <t>251</t>
+          <t>98</t>
         </is>
       </c>
     </row>
     <row r="310" spans="1:29">
       <c r="A310" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>FATIMA </t>
         </is>
       </c>
       <c r="B310" s="0" t="inlineStr">
         <is>
-          <t>TURARE</t>
+          <t>SIDI</t>
         </is>
       </c>
       <c r="R310" s="0" t="inlineStr">
@@ -10773,7 +10748,7 @@
       </c>
       <c r="X310" s="0" t="inlineStr">
         <is>
-          <t>21000.00</t>
+          <t>40000.00</t>
         </is>
       </c>
       <c r="Z310" s="0" t="inlineStr">
@@ -10788,19 +10763,19 @@
       </c>
       <c r="AC310" s="0" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>313</t>
         </is>
       </c>
     </row>
     <row r="311" spans="1:29">
       <c r="A311" s="0" t="inlineStr">
         <is>
-          <t>ZAINAB</t>
+          <t>HADIZA</t>
         </is>
       </c>
       <c r="B311" s="0" t="inlineStr">
         <is>
-          <t>UMAR</t>
+          <t>SOKOTO</t>
         </is>
       </c>
       <c r="R311" s="0" t="inlineStr">
@@ -10810,7 +10785,7 @@
       </c>
       <c r="X311" s="0" t="inlineStr">
         <is>
-          <t>65000.00</t>
+          <t>852500.00</t>
         </is>
       </c>
       <c r="Z311" s="0" t="inlineStr">
@@ -10825,19 +10800,19 @@
       </c>
       <c r="AC311" s="0" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>118</t>
         </is>
       </c>
     </row>
     <row r="312" spans="1:29">
       <c r="A312" s="0" t="inlineStr">
         <is>
-          <t>ZAINAB</t>
+          <t>FARIDA</t>
         </is>
       </c>
       <c r="B312" s="0" t="inlineStr">
         <is>
-          <t>USMAN</t>
+          <t>SULAIMAN</t>
         </is>
       </c>
       <c r="R312" s="0" t="inlineStr">
@@ -10847,7 +10822,7 @@
       </c>
       <c r="X312" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>99500.00</t>
         </is>
       </c>
       <c r="Z312" s="0" t="inlineStr">
@@ -10862,19 +10837,19 @@
       </c>
       <c r="AC312" s="0" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>246</t>
         </is>
       </c>
     </row>
     <row r="313" spans="1:29">
       <c r="A313" s="0" t="inlineStr">
         <is>
-          <t>HAJ SADIYA</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B313" s="0" t="inlineStr">
         <is>
-          <t>WAILO</t>
+          <t>TRENDY</t>
         </is>
       </c>
       <c r="R313" s="0" t="inlineStr">
@@ -10884,7 +10859,7 @@
       </c>
       <c r="X313" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>110500.00</t>
         </is>
       </c>
       <c r="Z313" s="0" t="inlineStr">
@@ -10899,19 +10874,19 @@
       </c>
       <c r="AC313" s="0" t="inlineStr">
         <is>
-          <t>259</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="314" spans="1:29">
       <c r="A314" s="0" t="inlineStr">
         <is>
-          <t>SALIHU</t>
+          <t>JAMILA</t>
         </is>
       </c>
       <c r="B314" s="0" t="inlineStr">
         <is>
-          <t>YABATEX</t>
+          <t>TUKUR</t>
         </is>
       </c>
       <c r="R314" s="0" t="inlineStr">
@@ -10921,7 +10896,7 @@
       </c>
       <c r="X314" s="0" t="inlineStr">
         <is>
-          <t>681000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z314" s="0" t="inlineStr">
@@ -10936,19 +10911,19 @@
       </c>
       <c r="AC314" s="0" t="inlineStr">
         <is>
-          <t>258</t>
+          <t>251</t>
         </is>
       </c>
     </row>
     <row r="315" spans="1:29">
       <c r="A315" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B315" s="0" t="inlineStr">
         <is>
-          <t>YAN BIYU</t>
+          <t>TURARE</t>
         </is>
       </c>
       <c r="R315" s="0" t="inlineStr">
@@ -10958,7 +10933,7 @@
       </c>
       <c r="X315" s="0" t="inlineStr">
         <is>
-          <t>2501200.00</t>
+          <t>21000.00</t>
         </is>
       </c>
       <c r="Z315" s="0" t="inlineStr">
@@ -10973,19 +10948,19 @@
       </c>
       <c r="AC315" s="0" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>153</t>
         </is>
       </c>
     </row>
     <row r="316" spans="1:29">
       <c r="A316" s="0" t="inlineStr">
         <is>
-          <t>ZULAIHA</t>
+          <t>ZAINAB</t>
         </is>
       </c>
       <c r="B316" s="0" t="inlineStr">
         <is>
-          <t>YOLA</t>
+          <t>UMAR</t>
         </is>
       </c>
       <c r="R316" s="0" t="inlineStr">
@@ -10995,7 +10970,7 @@
       </c>
       <c r="X316" s="0" t="inlineStr">
         <is>
-          <t>392000.00</t>
+          <t>65000.00</t>
         </is>
       </c>
       <c r="Z316" s="0" t="inlineStr">
@@ -11010,19 +10985,19 @@
       </c>
       <c r="AC316" s="0" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>203</t>
         </is>
       </c>
     </row>
     <row r="317" spans="1:29">
       <c r="A317" s="0" t="inlineStr">
         <is>
-          <t>FAUZIYYA</t>
+          <t>ZAINAB</t>
         </is>
       </c>
       <c r="B317" s="0" t="inlineStr">
         <is>
-          <t>YOLA</t>
+          <t>USMAN</t>
         </is>
       </c>
       <c r="R317" s="0" t="inlineStr">
@@ -11032,7 +11007,7 @@
       </c>
       <c r="X317" s="0" t="inlineStr">
         <is>
-          <t>17000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z317" s="0" t="inlineStr">
@@ -11047,19 +11022,19 @@
       </c>
       <c r="AC317" s="0" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>152</t>
         </is>
       </c>
     </row>
     <row r="318" spans="1:29">
       <c r="A318" s="0" t="inlineStr">
         <is>
-          <t>HAJ RUKAYYA</t>
+          <t>HAJ SADIYA</t>
         </is>
       </c>
       <c r="B318" s="0" t="inlineStr">
         <is>
-          <t>YUSUF</t>
+          <t>WAILO</t>
         </is>
       </c>
       <c r="R318" s="0" t="inlineStr">
@@ -11084,19 +11059,19 @@
       </c>
       <c r="AC318" s="0" t="inlineStr">
         <is>
-          <t>248</t>
+          <t>259</t>
         </is>
       </c>
     </row>
     <row r="319" spans="1:29">
       <c r="A319" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>SALIHU</t>
         </is>
       </c>
       <c r="B319" s="0" t="inlineStr">
         <is>
-          <t>ZAHRA ONLINE</t>
+          <t>YABATEX</t>
         </is>
       </c>
       <c r="R319" s="0" t="inlineStr">
@@ -11106,7 +11081,7 @@
       </c>
       <c r="X319" s="0" t="inlineStr">
         <is>
-          <t>406500.00</t>
+          <t>681000.00</t>
         </is>
       </c>
       <c r="Z319" s="0" t="inlineStr">
@@ -11121,42 +11096,227 @@
       </c>
       <c r="AC319" s="0" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>258</t>
         </is>
       </c>
     </row>
     <row r="320" spans="1:29">
       <c r="A320" s="0" t="inlineStr">
         <is>
+          <t>MAMAN</t>
+        </is>
+      </c>
+      <c r="B320" s="0" t="inlineStr">
+        <is>
+          <t>YAN BIYU</t>
+        </is>
+      </c>
+      <c r="R320" s="0" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="X320" s="0" t="inlineStr">
+        <is>
+          <t>2501200.00</t>
+        </is>
+      </c>
+      <c r="Z320" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA320" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AC320" s="0" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+    </row>
+    <row r="321" spans="1:29">
+      <c r="A321" s="0" t="inlineStr">
+        <is>
+          <t>ZULAIHA</t>
+        </is>
+      </c>
+      <c r="B321" s="0" t="inlineStr">
+        <is>
+          <t>YOLA</t>
+        </is>
+      </c>
+      <c r="R321" s="0" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="X321" s="0" t="inlineStr">
+        <is>
+          <t>392000.00</t>
+        </is>
+      </c>
+      <c r="Z321" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA321" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AC321" s="0" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+    </row>
+    <row r="322" spans="1:29">
+      <c r="A322" s="0" t="inlineStr">
+        <is>
+          <t>FAUZIYYA</t>
+        </is>
+      </c>
+      <c r="B322" s="0" t="inlineStr">
+        <is>
+          <t>YOLA</t>
+        </is>
+      </c>
+      <c r="R322" s="0" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="X322" s="0" t="inlineStr">
+        <is>
+          <t>17000.00</t>
+        </is>
+      </c>
+      <c r="Z322" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA322" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AC322" s="0" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+    </row>
+    <row r="323" spans="1:29">
+      <c r="A323" s="0" t="inlineStr">
+        <is>
+          <t>HAJ RUKAYYA</t>
+        </is>
+      </c>
+      <c r="B323" s="0" t="inlineStr">
+        <is>
+          <t>YUSUF</t>
+        </is>
+      </c>
+      <c r="R323" s="0" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="X323" s="0" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="Z323" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA323" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AC323" s="0" t="inlineStr">
+        <is>
+          <t>248</t>
+        </is>
+      </c>
+    </row>
+    <row r="324" spans="1:29">
+      <c r="A324" s="0" t="inlineStr">
+        <is>
+          <t>MAMAN</t>
+        </is>
+      </c>
+      <c r="B324" s="0" t="inlineStr">
+        <is>
+          <t>ZAHRA ONLINE</t>
+        </is>
+      </c>
+      <c r="R324" s="0" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="X324" s="0" t="inlineStr">
+        <is>
+          <t>406500.00</t>
+        </is>
+      </c>
+      <c r="Z324" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA324" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AC324" s="0" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+    </row>
+    <row r="325" spans="1:29">
+      <c r="A325" s="0" t="inlineStr">
+        <is>
           <t>FATIMA</t>
         </is>
       </c>
-      <c r="B320" s="0" t="inlineStr">
+      <c r="B325" s="0" t="inlineStr">
         <is>
           <t>ZARAMI</t>
         </is>
       </c>
-      <c r="R320" s="0" t="inlineStr">
-        <is>
-          <t>y</t>
-        </is>
-      </c>
-      <c r="X320" s="0" t="inlineStr">
+      <c r="R325" s="0" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="X325" s="0" t="inlineStr">
         <is>
           <t>768300.00</t>
         </is>
       </c>
-      <c r="Z320" s="0" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="AA320" s="0" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="AC320" s="0" t="inlineStr">
+      <c r="Z325" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA325" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AC325" s="0" t="inlineStr">
         <is>
           <t>97</t>
         </is>

</xml_diff>

<commit_message>
Fixed Some Data Type Issue
</commit_message>
<xml_diff>
--- a/Excels/Customers.xlsx
+++ b/Excels/Customers.xlsx
@@ -212,7 +212,7 @@
       </c>
       <c r="X2" s="0" t="inlineStr">
         <is>
-          <t>2864500.00</t>
+          <t>3308500.00</t>
         </is>
       </c>
       <c r="Z2" s="0" t="inlineStr">
@@ -372,7 +372,7 @@
       </c>
       <c r="X7" s="0" t="inlineStr">
         <is>
-          <t>3414000.00</t>
+          <t>3494000.00</t>
         </is>
       </c>
       <c r="Z7" s="0" t="inlineStr">
@@ -500,7 +500,7 @@
       </c>
       <c r="X11" s="0" t="inlineStr">
         <is>
-          <t>591000.00</t>
+          <t>719000.00</t>
         </is>
       </c>
       <c r="Z11" s="0" t="inlineStr">
@@ -532,7 +532,7 @@
       </c>
       <c r="X12" s="0" t="inlineStr">
         <is>
-          <t>110765800.00</t>
+          <t>111760200.00</t>
         </is>
       </c>
       <c r="Z12" s="0" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="X14" s="0" t="inlineStr">
         <is>
-          <t>19000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z14" s="0" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="X22" s="0" t="inlineStr">
         <is>
-          <t>17135000.00</t>
+          <t>17800600.00</t>
         </is>
       </c>
       <c r="Z22" s="0" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="X23" s="0" t="inlineStr">
         <is>
-          <t>15869800.00</t>
+          <t>16074300.00</t>
         </is>
       </c>
       <c r="Z23" s="0" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="X32" s="0" t="inlineStr">
         <is>
-          <t>3710900.00</t>
+          <t>3794900.00</t>
         </is>
       </c>
       <c r="Z32" s="0" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="X36" s="0" t="inlineStr">
         <is>
-          <t>5795000.00</t>
+          <t>6470000.00</t>
         </is>
       </c>
       <c r="Z36" s="0" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="X43" s="0" t="inlineStr">
         <is>
-          <t>3118800.00</t>
+          <t>3143300.00</t>
         </is>
       </c>
       <c r="Z43" s="0" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="X106" s="0" t="inlineStr">
         <is>
-          <t>837500.00</t>
+          <t>938500.00</t>
         </is>
       </c>
       <c r="Z106" s="0" t="inlineStr">
@@ -3673,7 +3673,7 @@
       </c>
       <c r="X110" s="0" t="inlineStr">
         <is>
-          <t>1115000.00</t>
+          <t>1127000.00</t>
         </is>
       </c>
       <c r="Z110" s="0" t="inlineStr">
@@ -4889,7 +4889,7 @@
       </c>
       <c r="X148" s="0" t="inlineStr">
         <is>
-          <t>44500.00</t>
+          <t>74500.00</t>
         </is>
       </c>
       <c r="Z148" s="0" t="inlineStr">
@@ -6255,12 +6255,7 @@
     <row r="191" spans="1:29">
       <c r="A191" s="0" t="inlineStr">
         <is>
-          <t>HASIYA</t>
-        </is>
-      </c>
-      <c r="B191" s="0" t="inlineStr">
-        <is>
-          <t> TURAKI - ABK</t>
+          <t>FARIDA MUHD</t>
         </is>
       </c>
       <c r="R191" s="0" t="inlineStr">
@@ -6285,19 +6280,19 @@
       </c>
       <c r="AC191" s="0" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>342</t>
         </is>
       </c>
     </row>
     <row r="192" spans="1:29">
       <c r="A192" s="0" t="inlineStr">
         <is>
-          <t>HAJ SAMIRA</t>
+          <t>HASIYA</t>
         </is>
       </c>
       <c r="B192" s="0" t="inlineStr">
         <is>
-          <t>- ABK</t>
+          <t> TURAKI - ABK</t>
         </is>
       </c>
       <c r="R192" s="0" t="inlineStr">
@@ -6322,19 +6317,19 @@
       </c>
       <c r="AC192" s="0" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>222</t>
         </is>
       </c>
     </row>
     <row r="193" spans="1:29">
       <c r="A193" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>HAJ SAMIRA</t>
         </is>
       </c>
       <c r="B193" s="0" t="inlineStr">
         <is>
-          <t>ABANA</t>
+          <t>- ABK</t>
         </is>
       </c>
       <c r="R193" s="0" t="inlineStr">
@@ -6344,7 +6339,7 @@
       </c>
       <c r="X193" s="0" t="inlineStr">
         <is>
-          <t>251500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z193" s="0" t="inlineStr">
@@ -6359,19 +6354,19 @@
       </c>
       <c r="AC193" s="0" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="194" spans="1:29">
       <c r="A194" s="0" t="inlineStr">
         <is>
-          <t>KHADIJA</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B194" s="0" t="inlineStr">
         <is>
-          <t>ABDULQADIR</t>
+          <t>ABANA</t>
         </is>
       </c>
       <c r="R194" s="0" t="inlineStr">
@@ -6381,7 +6376,7 @@
       </c>
       <c r="X194" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>251500.00</t>
         </is>
       </c>
       <c r="Z194" s="0" t="inlineStr">
@@ -6396,14 +6391,14 @@
       </c>
       <c r="AC194" s="0" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>281</t>
         </is>
       </c>
     </row>
     <row r="195" spans="1:29">
       <c r="A195" s="0" t="inlineStr">
         <is>
-          <t>MARIA</t>
+          <t>KHADIJA</t>
         </is>
       </c>
       <c r="B195" s="0" t="inlineStr">
@@ -6433,19 +6428,19 @@
       </c>
       <c r="AC195" s="0" t="inlineStr">
         <is>
-          <t>328</t>
+          <t>191</t>
         </is>
       </c>
     </row>
     <row r="196" spans="1:29">
       <c r="A196" s="0" t="inlineStr">
         <is>
-          <t>NURIYYAH</t>
+          <t>MARIA</t>
         </is>
       </c>
       <c r="B196" s="0" t="inlineStr">
         <is>
-          <t>AHMAD</t>
+          <t>ABDULQADIR</t>
         </is>
       </c>
       <c r="R196" s="0" t="inlineStr">
@@ -6455,7 +6450,7 @@
       </c>
       <c r="X196" s="0" t="inlineStr">
         <is>
-          <t>443000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z196" s="0" t="inlineStr">
@@ -6470,14 +6465,14 @@
       </c>
       <c r="AC196" s="0" t="inlineStr">
         <is>
-          <t>112</t>
+          <t>328</t>
         </is>
       </c>
     </row>
     <row r="197" spans="1:29">
       <c r="A197" s="0" t="inlineStr">
         <is>
-          <t>HAJ MAIMUNA</t>
+          <t>NURIYYAH</t>
         </is>
       </c>
       <c r="B197" s="0" t="inlineStr">
@@ -6492,7 +6487,7 @@
       </c>
       <c r="X197" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>443000.00</t>
         </is>
       </c>
       <c r="Z197" s="0" t="inlineStr">
@@ -6507,19 +6502,19 @@
       </c>
       <c r="AC197" s="0" t="inlineStr">
         <is>
-          <t>279</t>
+          <t>112</t>
         </is>
       </c>
     </row>
     <row r="198" spans="1:29">
       <c r="A198" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>HAJ MAIMUNA</t>
         </is>
       </c>
       <c r="B198" s="0" t="inlineStr">
         <is>
-          <t>AIRFORCE</t>
+          <t>AHMAD</t>
         </is>
       </c>
       <c r="R198" s="0" t="inlineStr">
@@ -6544,19 +6539,19 @@
       </c>
       <c r="AC198" s="0" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>279</t>
         </is>
       </c>
     </row>
     <row r="199" spans="1:29">
       <c r="A199" s="0" t="inlineStr">
         <is>
-          <t>SADIYA</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B199" s="0" t="inlineStr">
         <is>
-          <t>ALA</t>
+          <t>AIRFORCE</t>
         </is>
       </c>
       <c r="R199" s="0" t="inlineStr">
@@ -6581,19 +6576,19 @@
       </c>
       <c r="AC199" s="0" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>111</t>
         </is>
       </c>
     </row>
     <row r="200" spans="1:29">
       <c r="A200" s="0" t="inlineStr">
         <is>
-          <t>HAJ ZALIHATU</t>
+          <t>SADIYA</t>
         </is>
       </c>
       <c r="B200" s="0" t="inlineStr">
         <is>
-          <t>ALERU</t>
+          <t>ALA</t>
         </is>
       </c>
       <c r="R200" s="0" t="inlineStr">
@@ -6618,19 +6613,19 @@
       </c>
       <c r="AC200" s="0" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>126</t>
         </is>
       </c>
     </row>
     <row r="201" spans="1:29">
       <c r="A201" s="0" t="inlineStr">
         <is>
-          <t>MA'U</t>
+          <t>HAJ ZALIHATU</t>
         </is>
       </c>
       <c r="B201" s="0" t="inlineStr">
         <is>
-          <t>ALHASSAN</t>
+          <t>ALERU</t>
         </is>
       </c>
       <c r="R201" s="0" t="inlineStr">
@@ -6640,7 +6635,7 @@
       </c>
       <c r="X201" s="0" t="inlineStr">
         <is>
-          <t>48000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z201" s="0" t="inlineStr">
@@ -6655,19 +6650,19 @@
       </c>
       <c r="AC201" s="0" t="inlineStr">
         <is>
-          <t>183</t>
+          <t>287</t>
         </is>
       </c>
     </row>
     <row r="202" spans="1:29">
       <c r="A202" s="0" t="inlineStr">
         <is>
-          <t>BILKISU</t>
+          <t>MA'U</t>
         </is>
       </c>
       <c r="B202" s="0" t="inlineStr">
         <is>
-          <t>ALI BALA</t>
+          <t>ALHASSAN</t>
         </is>
       </c>
       <c r="R202" s="0" t="inlineStr">
@@ -6677,7 +6672,7 @@
       </c>
       <c r="X202" s="0" t="inlineStr">
         <is>
-          <t>1342000.00</t>
+          <t>48000.00</t>
         </is>
       </c>
       <c r="Z202" s="0" t="inlineStr">
@@ -6692,19 +6687,19 @@
       </c>
       <c r="AC202" s="0" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>183</t>
         </is>
       </c>
     </row>
     <row r="203" spans="1:29">
       <c r="A203" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>BILKISU</t>
         </is>
       </c>
       <c r="B203" s="0" t="inlineStr">
         <is>
-          <t>AMATU</t>
+          <t>ALI BALA</t>
         </is>
       </c>
       <c r="R203" s="0" t="inlineStr">
@@ -6714,7 +6709,7 @@
       </c>
       <c r="X203" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1342000.00</t>
         </is>
       </c>
       <c r="Z203" s="0" t="inlineStr">
@@ -6729,19 +6724,19 @@
       </c>
       <c r="AC203" s="0" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>79</t>
         </is>
       </c>
     </row>
     <row r="204" spans="1:29">
       <c r="A204" s="0" t="inlineStr">
         <is>
-          <t>BILKISU</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B204" s="0" t="inlineStr">
         <is>
-          <t>AMMANI</t>
+          <t>AMATU</t>
         </is>
       </c>
       <c r="R204" s="0" t="inlineStr">
@@ -6751,7 +6746,7 @@
       </c>
       <c r="X204" s="0" t="inlineStr">
         <is>
-          <t>65000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z204" s="0" t="inlineStr">
@@ -6766,19 +6761,19 @@
       </c>
       <c r="AC204" s="0" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>134</t>
         </is>
       </c>
     </row>
     <row r="205" spans="1:29">
       <c r="A205" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>BILKISU</t>
         </is>
       </c>
       <c r="B205" s="0" t="inlineStr">
         <is>
-          <t>AMMI</t>
+          <t>AMMANI</t>
         </is>
       </c>
       <c r="R205" s="0" t="inlineStr">
@@ -6788,7 +6783,7 @@
       </c>
       <c r="X205" s="0" t="inlineStr">
         <is>
-          <t>288100.00</t>
+          <t>65000.00</t>
         </is>
       </c>
       <c r="Z205" s="0" t="inlineStr">
@@ -6803,19 +6798,19 @@
       </c>
       <c r="AC205" s="0" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>189</t>
         </is>
       </c>
     </row>
     <row r="206" spans="1:29">
       <c r="A206" s="0" t="inlineStr">
         <is>
-          <t>SAMIRA</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B206" s="0" t="inlineStr">
         <is>
-          <t>ARC</t>
+          <t>AMMI</t>
         </is>
       </c>
       <c r="R206" s="0" t="inlineStr">
@@ -6825,7 +6820,7 @@
       </c>
       <c r="X206" s="0" t="inlineStr">
         <is>
-          <t>166500.00</t>
+          <t>288100.00</t>
         </is>
       </c>
       <c r="Z206" s="0" t="inlineStr">
@@ -6840,19 +6835,19 @@
       </c>
       <c r="AC206" s="0" t="inlineStr">
         <is>
-          <t>187</t>
+          <t>130</t>
         </is>
       </c>
     </row>
     <row r="207" spans="1:29">
       <c r="A207" s="0" t="inlineStr">
         <is>
-          <t>HAJ HAUWA</t>
+          <t>SAMIRA</t>
         </is>
       </c>
       <c r="B207" s="0" t="inlineStr">
         <is>
-          <t>AWAISU</t>
+          <t>ARC</t>
         </is>
       </c>
       <c r="R207" s="0" t="inlineStr">
@@ -6862,7 +6857,7 @@
       </c>
       <c r="X207" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>166500.00</t>
         </is>
       </c>
       <c r="Z207" s="0" t="inlineStr">
@@ -6877,19 +6872,19 @@
       </c>
       <c r="AC207" s="0" t="inlineStr">
         <is>
-          <t>284</t>
+          <t>187</t>
         </is>
       </c>
     </row>
     <row r="208" spans="1:29">
       <c r="A208" s="0" t="inlineStr">
         <is>
-          <t>ZAINAB</t>
+          <t>HAJ HAUWA</t>
         </is>
       </c>
       <c r="B208" s="0" t="inlineStr">
         <is>
-          <t>AZARE</t>
+          <t>AWAISU</t>
         </is>
       </c>
       <c r="R208" s="0" t="inlineStr">
@@ -6914,19 +6909,19 @@
       </c>
       <c r="AC208" s="0" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>284</t>
         </is>
       </c>
     </row>
     <row r="209" spans="1:29">
       <c r="A209" s="0" t="inlineStr">
         <is>
-          <t>RAHAMA</t>
+          <t>ZAINAB</t>
         </is>
       </c>
       <c r="B209" s="0" t="inlineStr">
         <is>
-          <t>BAMALLI</t>
+          <t>AZARE</t>
         </is>
       </c>
       <c r="R209" s="0" t="inlineStr">
@@ -6951,19 +6946,19 @@
       </c>
       <c r="AC209" s="0" t="inlineStr">
         <is>
-          <t>265</t>
+          <t>144</t>
         </is>
       </c>
     </row>
     <row r="210" spans="1:29">
       <c r="A210" s="0" t="inlineStr">
         <is>
-          <t>NAFISA</t>
+          <t>RAHAMA</t>
         </is>
       </c>
       <c r="B210" s="0" t="inlineStr">
         <is>
-          <t>BARAU</t>
+          <t>BAMALLI</t>
         </is>
       </c>
       <c r="R210" s="0" t="inlineStr">
@@ -6988,19 +6983,19 @@
       </c>
       <c r="AC210" s="0" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>265</t>
         </is>
       </c>
     </row>
     <row r="211" spans="1:29">
       <c r="A211" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>NAFISA</t>
         </is>
       </c>
       <c r="B211" s="0" t="inlineStr">
         <is>
-          <t>BAUCHI</t>
+          <t>BARAU</t>
         </is>
       </c>
       <c r="R211" s="0" t="inlineStr">
@@ -7010,7 +7005,7 @@
       </c>
       <c r="X211" s="0" t="inlineStr">
         <is>
-          <t>195000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z211" s="0" t="inlineStr">
@@ -7025,19 +7020,19 @@
       </c>
       <c r="AC211" s="0" t="inlineStr">
         <is>
-          <t>314</t>
+          <t>148</t>
         </is>
       </c>
     </row>
     <row r="212" spans="1:29">
       <c r="A212" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B212" s="0" t="inlineStr">
         <is>
-          <t>BAWA ROAD</t>
+          <t>BAUCHI</t>
         </is>
       </c>
       <c r="R212" s="0" t="inlineStr">
@@ -7047,7 +7042,7 @@
       </c>
       <c r="X212" s="0" t="inlineStr">
         <is>
-          <t>1298000.00</t>
+          <t>195000.00</t>
         </is>
       </c>
       <c r="Z212" s="0" t="inlineStr">
@@ -7062,19 +7057,19 @@
       </c>
       <c r="AC212" s="0" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>314</t>
         </is>
       </c>
     </row>
     <row r="213" spans="1:29">
       <c r="A213" s="0" t="inlineStr">
         <is>
-          <t>HAUWA</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B213" s="0" t="inlineStr">
         <is>
-          <t>BELLO</t>
+          <t>BAWA ROAD</t>
         </is>
       </c>
       <c r="R213" s="0" t="inlineStr">
@@ -7084,7 +7079,7 @@
       </c>
       <c r="X213" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1449200.00</t>
         </is>
       </c>
       <c r="Z213" s="0" t="inlineStr">
@@ -7099,19 +7094,19 @@
       </c>
       <c r="AC213" s="0" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>113</t>
         </is>
       </c>
     </row>
     <row r="214" spans="1:29">
       <c r="A214" s="0" t="inlineStr">
         <is>
-          <t>FARIDA</t>
+          <t>HAUWA</t>
         </is>
       </c>
       <c r="B214" s="0" t="inlineStr">
         <is>
-          <t>BINDAWA</t>
+          <t>BELLO</t>
         </is>
       </c>
       <c r="R214" s="0" t="inlineStr">
@@ -7136,14 +7131,14 @@
       </c>
       <c r="AC214" s="0" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>125</t>
         </is>
       </c>
     </row>
     <row r="215" spans="1:29">
       <c r="A215" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>FARIDA</t>
         </is>
       </c>
       <c r="B215" s="0" t="inlineStr">
@@ -7158,7 +7153,7 @@
       </c>
       <c r="X215" s="0" t="inlineStr">
         <is>
-          <t>937000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z215" s="0" t="inlineStr">
@@ -7173,19 +7168,19 @@
       </c>
       <c r="AC215" s="0" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>93</t>
         </is>
       </c>
     </row>
     <row r="216" spans="1:29">
       <c r="A216" s="0" t="inlineStr">
         <is>
-          <t>MARIA</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B216" s="0" t="inlineStr">
         <is>
-          <t>BOSE</t>
+          <t>BINDAWA</t>
         </is>
       </c>
       <c r="R216" s="0" t="inlineStr">
@@ -7195,7 +7190,7 @@
       </c>
       <c r="X216" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>967000.00</t>
         </is>
       </c>
       <c r="Z216" s="0" t="inlineStr">
@@ -7210,19 +7205,19 @@
       </c>
       <c r="AC216" s="0" t="inlineStr">
         <is>
-          <t>295</t>
+          <t>123</t>
         </is>
       </c>
     </row>
     <row r="217" spans="1:29">
       <c r="A217" s="0" t="inlineStr">
         <is>
-          <t>HAJ MARYAM</t>
+          <t>MARIA</t>
         </is>
       </c>
       <c r="B217" s="0" t="inlineStr">
         <is>
-          <t>BUHARI</t>
+          <t>BOSE</t>
         </is>
       </c>
       <c r="R217" s="0" t="inlineStr">
@@ -7232,7 +7227,7 @@
       </c>
       <c r="X217" s="0" t="inlineStr">
         <is>
-          <t>115000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z217" s="0" t="inlineStr">
@@ -7247,19 +7242,19 @@
       </c>
       <c r="AC217" s="0" t="inlineStr">
         <is>
-          <t>312</t>
+          <t>295</t>
         </is>
       </c>
     </row>
     <row r="218" spans="1:29">
       <c r="A218" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>HAJ MARYAM</t>
         </is>
       </c>
       <c r="B218" s="0" t="inlineStr">
         <is>
-          <t>BULAMA</t>
+          <t>BUHARI</t>
         </is>
       </c>
       <c r="R218" s="0" t="inlineStr">
@@ -7269,7 +7264,7 @@
       </c>
       <c r="X218" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>115000.00</t>
         </is>
       </c>
       <c r="Z218" s="0" t="inlineStr">
@@ -7284,19 +7279,19 @@
       </c>
       <c r="AC218" s="0" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>312</t>
         </is>
       </c>
     </row>
     <row r="219" spans="1:29">
       <c r="A219" s="0" t="inlineStr">
         <is>
-          <t>KHADIJA</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B219" s="0" t="inlineStr">
         <is>
-          <t>CHIROMA</t>
+          <t>BULAMA</t>
         </is>
       </c>
       <c r="R219" s="0" t="inlineStr">
@@ -7306,7 +7301,7 @@
       </c>
       <c r="X219" s="0" t="inlineStr">
         <is>
-          <t>8500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z219" s="0" t="inlineStr">
@@ -7321,19 +7316,19 @@
       </c>
       <c r="AC219" s="0" t="inlineStr">
         <is>
-          <t>184</t>
+          <t>253</t>
         </is>
       </c>
     </row>
     <row r="220" spans="1:29">
       <c r="A220" s="0" t="inlineStr">
         <is>
-          <t>ZAHRA</t>
+          <t>KHADIJA</t>
         </is>
       </c>
       <c r="B220" s="0" t="inlineStr">
         <is>
-          <t>COLLECTION</t>
+          <t>CHIROMA</t>
         </is>
       </c>
       <c r="R220" s="0" t="inlineStr">
@@ -7343,7 +7338,7 @@
       </c>
       <c r="X220" s="0" t="inlineStr">
         <is>
-          <t>171000.00</t>
+          <t>8500.00</t>
         </is>
       </c>
       <c r="Z220" s="0" t="inlineStr">
@@ -7358,19 +7353,19 @@
       </c>
       <c r="AC220" s="0" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>184</t>
         </is>
       </c>
     </row>
     <row r="221" spans="1:29">
       <c r="A221" s="0" t="inlineStr">
         <is>
-          <t>MAIMUNA</t>
+          <t>ZAHRA</t>
         </is>
       </c>
       <c r="B221" s="0" t="inlineStr">
         <is>
-          <t>CUSTOM</t>
+          <t>COLLECTION</t>
         </is>
       </c>
       <c r="R221" s="0" t="inlineStr">
@@ -7380,7 +7375,7 @@
       </c>
       <c r="X221" s="0" t="inlineStr">
         <is>
-          <t>20000.00</t>
+          <t>171000.00</t>
         </is>
       </c>
       <c r="Z221" s="0" t="inlineStr">
@@ -7395,19 +7390,19 @@
       </c>
       <c r="AC221" s="0" t="inlineStr">
         <is>
-          <t>227</t>
+          <t>136</t>
         </is>
       </c>
     </row>
     <row r="222" spans="1:29">
       <c r="A222" s="0" t="inlineStr">
         <is>
-          <t>MAMAN AISHA</t>
+          <t>MAIMUNA</t>
         </is>
       </c>
       <c r="B222" s="0" t="inlineStr">
         <is>
-          <t>DAHIRU</t>
+          <t>CUSTOM</t>
         </is>
       </c>
       <c r="R222" s="0" t="inlineStr">
@@ -7417,7 +7412,7 @@
       </c>
       <c r="X222" s="0" t="inlineStr">
         <is>
-          <t>75000.00</t>
+          <t>20000.00</t>
         </is>
       </c>
       <c r="Z222" s="0" t="inlineStr">
@@ -7432,19 +7427,19 @@
       </c>
       <c r="AC222" s="0" t="inlineStr">
         <is>
-          <t>194</t>
+          <t>227</t>
         </is>
       </c>
     </row>
     <row r="223" spans="1:29">
       <c r="A223" s="0" t="inlineStr">
         <is>
-          <t>MAIMUNA</t>
+          <t>MAMAN AISHA</t>
         </is>
       </c>
       <c r="B223" s="0" t="inlineStr">
         <is>
-          <t>DAN ASABE</t>
+          <t>DAHIRU</t>
         </is>
       </c>
       <c r="R223" s="0" t="inlineStr">
@@ -7454,7 +7449,7 @@
       </c>
       <c r="X223" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>75000.00</t>
         </is>
       </c>
       <c r="Z223" s="0" t="inlineStr">
@@ -7469,19 +7464,19 @@
       </c>
       <c r="AC223" s="0" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>194</t>
         </is>
       </c>
     </row>
     <row r="224" spans="1:29">
       <c r="A224" s="0" t="inlineStr">
         <is>
-          <t>KB</t>
+          <t>MAIMUNA</t>
         </is>
       </c>
       <c r="B224" s="0" t="inlineStr">
         <is>
-          <t>DORAYI</t>
+          <t>DAN ASABE</t>
         </is>
       </c>
       <c r="R224" s="0" t="inlineStr">
@@ -7491,7 +7486,7 @@
       </c>
       <c r="X224" s="0" t="inlineStr">
         <is>
-          <t>3667000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z224" s="0" t="inlineStr">
@@ -7506,19 +7501,19 @@
       </c>
       <c r="AC224" s="0" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>169</t>
         </is>
       </c>
     </row>
     <row r="225" spans="1:29">
       <c r="A225" s="0" t="inlineStr">
         <is>
-          <t>UMMI</t>
+          <t>KB</t>
         </is>
       </c>
       <c r="B225" s="0" t="inlineStr">
         <is>
-          <t>FAB SHOP</t>
+          <t>DORAYI</t>
         </is>
       </c>
       <c r="R225" s="0" t="inlineStr">
@@ -7528,7 +7523,7 @@
       </c>
       <c r="X225" s="0" t="inlineStr">
         <is>
-          <t>1160000.00</t>
+          <t>3667000.00</t>
         </is>
       </c>
       <c r="Z225" s="0" t="inlineStr">
@@ -7543,19 +7538,19 @@
       </c>
       <c r="AC225" s="0" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>172</t>
         </is>
       </c>
     </row>
     <row r="226" spans="1:29">
       <c r="A226" s="0" t="inlineStr">
         <is>
-          <t>JAMI</t>
+          <t>UMMI</t>
         </is>
       </c>
       <c r="B226" s="0" t="inlineStr">
         <is>
-          <t>FABRICS</t>
+          <t>FAB SHOP</t>
         </is>
       </c>
       <c r="R226" s="0" t="inlineStr">
@@ -7565,7 +7560,7 @@
       </c>
       <c r="X226" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1160000.00</t>
         </is>
       </c>
       <c r="Z226" s="0" t="inlineStr">
@@ -7580,19 +7575,19 @@
       </c>
       <c r="AC226" s="0" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>100</t>
         </is>
       </c>
     </row>
     <row r="227" spans="1:29">
       <c r="A227" s="0" t="inlineStr">
         <is>
-          <t>SAMIRA</t>
+          <t>JAMI</t>
         </is>
       </c>
       <c r="B227" s="0" t="inlineStr">
         <is>
-          <t>FAGGE</t>
+          <t>FABRICS</t>
         </is>
       </c>
       <c r="R227" s="0" t="inlineStr">
@@ -7602,7 +7597,7 @@
       </c>
       <c r="X227" s="0" t="inlineStr">
         <is>
-          <t>355000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z227" s="0" t="inlineStr">
@@ -7617,19 +7612,19 @@
       </c>
       <c r="AC227" s="0" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>142</t>
         </is>
       </c>
     </row>
     <row r="228" spans="1:29">
       <c r="A228" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>SAMIRA</t>
         </is>
       </c>
       <c r="B228" s="0" t="inlineStr">
         <is>
-          <t>FAGGO</t>
+          <t>FAGGE</t>
         </is>
       </c>
       <c r="R228" s="0" t="inlineStr">
@@ -7639,7 +7634,7 @@
       </c>
       <c r="X228" s="0" t="inlineStr">
         <is>
-          <t>45000.00</t>
+          <t>355000.00</t>
         </is>
       </c>
       <c r="Z228" s="0" t="inlineStr">
@@ -7654,19 +7649,19 @@
       </c>
       <c r="AC228" s="0" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>89</t>
         </is>
       </c>
     </row>
     <row r="229" spans="1:29">
       <c r="A229" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B229" s="0" t="inlineStr">
         <is>
-          <t>FAROUQ</t>
+          <t>FAGGO</t>
         </is>
       </c>
       <c r="R229" s="0" t="inlineStr">
@@ -7676,7 +7671,7 @@
       </c>
       <c r="X229" s="0" t="inlineStr">
         <is>
-          <t>290000.00</t>
+          <t>45000.00</t>
         </is>
       </c>
       <c r="Z229" s="0" t="inlineStr">
@@ -7691,19 +7686,19 @@
       </c>
       <c r="AC229" s="0" t="inlineStr">
         <is>
-          <t>212</t>
+          <t>204</t>
         </is>
       </c>
     </row>
     <row r="230" spans="1:29">
       <c r="A230" s="0" t="inlineStr">
         <is>
-          <t>MUSA</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B230" s="0" t="inlineStr">
         <is>
-          <t>GARBA</t>
+          <t>FAROUQ</t>
         </is>
       </c>
       <c r="R230" s="0" t="inlineStr">
@@ -7713,7 +7708,7 @@
       </c>
       <c r="X230" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>290000.00</t>
         </is>
       </c>
       <c r="Z230" s="0" t="inlineStr">
@@ -7728,19 +7723,19 @@
       </c>
       <c r="AC230" s="0" t="inlineStr">
         <is>
-          <t>214</t>
+          <t>212</t>
         </is>
       </c>
     </row>
     <row r="231" spans="1:29">
       <c r="A231" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>MUSA</t>
         </is>
       </c>
       <c r="B231" s="0" t="inlineStr">
         <is>
-          <t>GOMBE</t>
+          <t>GARBA</t>
         </is>
       </c>
       <c r="R231" s="0" t="inlineStr">
@@ -7765,14 +7760,14 @@
       </c>
       <c r="AC231" s="0" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>214</t>
         </is>
       </c>
     </row>
     <row r="232" spans="1:29">
       <c r="A232" s="0" t="inlineStr">
         <is>
-          <t>MOMY</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B232" s="0" t="inlineStr">
@@ -7787,7 +7782,7 @@
       </c>
       <c r="X232" s="0" t="inlineStr">
         <is>
-          <t>375000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z232" s="0" t="inlineStr">
@@ -7802,14 +7797,14 @@
       </c>
       <c r="AC232" s="0" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>103</t>
         </is>
       </c>
     </row>
     <row r="233" spans="1:29">
       <c r="A233" s="0" t="inlineStr">
         <is>
-          <t>HAJ HAJARA</t>
+          <t>MOMY</t>
         </is>
       </c>
       <c r="B233" s="0" t="inlineStr">
@@ -7824,7 +7819,7 @@
       </c>
       <c r="X233" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>375000.00</t>
         </is>
       </c>
       <c r="Z233" s="0" t="inlineStr">
@@ -7839,19 +7834,19 @@
       </c>
       <c r="AC233" s="0" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>143</t>
         </is>
       </c>
     </row>
     <row r="234" spans="1:29">
       <c r="A234" s="0" t="inlineStr">
         <is>
-          <t>SAMIRA</t>
+          <t>HAJ HAJARA</t>
         </is>
       </c>
       <c r="B234" s="0" t="inlineStr">
         <is>
-          <t>GUNU</t>
+          <t>GOMBE</t>
         </is>
       </c>
       <c r="R234" s="0" t="inlineStr">
@@ -7861,7 +7856,7 @@
       </c>
       <c r="X234" s="0" t="inlineStr">
         <is>
-          <t>124000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z234" s="0" t="inlineStr">
@@ -7876,19 +7871,19 @@
       </c>
       <c r="AC234" s="0" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>209</t>
         </is>
       </c>
     </row>
     <row r="235" spans="1:29">
       <c r="A235" s="0" t="inlineStr">
         <is>
-          <t>BILKISU</t>
+          <t>SAMIRA</t>
         </is>
       </c>
       <c r="B235" s="0" t="inlineStr">
         <is>
-          <t>GWALABE</t>
+          <t>GUNU</t>
         </is>
       </c>
       <c r="R235" s="0" t="inlineStr">
@@ -7898,7 +7893,7 @@
       </c>
       <c r="X235" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>124000.00</t>
         </is>
       </c>
       <c r="Z235" s="0" t="inlineStr">
@@ -7913,14 +7908,14 @@
       </c>
       <c r="AC235" s="0" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>159</t>
         </is>
       </c>
     </row>
     <row r="236" spans="1:29">
       <c r="A236" s="0" t="inlineStr">
         <is>
-          <t>HAUWA</t>
+          <t>BILKISU</t>
         </is>
       </c>
       <c r="B236" s="0" t="inlineStr">
@@ -7935,7 +7930,7 @@
       </c>
       <c r="X236" s="0" t="inlineStr">
         <is>
-          <t>60000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z236" s="0" t="inlineStr">
@@ -7950,19 +7945,19 @@
       </c>
       <c r="AC236" s="0" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>101</t>
         </is>
       </c>
     </row>
     <row r="237" spans="1:29">
       <c r="A237" s="0" t="inlineStr">
         <is>
-          <t>MAMA</t>
+          <t>HAUWA</t>
         </is>
       </c>
       <c r="B237" s="0" t="inlineStr">
         <is>
-          <t>H &amp; M</t>
+          <t>GWALABE</t>
         </is>
       </c>
       <c r="R237" s="0" t="inlineStr">
@@ -7972,7 +7967,7 @@
       </c>
       <c r="X237" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>60000.00</t>
         </is>
       </c>
       <c r="Z237" s="0" t="inlineStr">
@@ -7987,19 +7982,19 @@
       </c>
       <c r="AC237" s="0" t="inlineStr">
         <is>
-          <t>163</t>
+          <t>321</t>
         </is>
       </c>
     </row>
     <row r="238" spans="1:29">
       <c r="A238" s="0" t="inlineStr">
         <is>
-          <t>HAJ HAUWA</t>
+          <t>MAMA</t>
         </is>
       </c>
       <c r="B238" s="0" t="inlineStr">
         <is>
-          <t>HABIB</t>
+          <t>H &amp; M</t>
         </is>
       </c>
       <c r="R238" s="0" t="inlineStr">
@@ -8024,24 +8019,19 @@
       </c>
       <c r="AC238" s="0" t="inlineStr">
         <is>
-          <t>264</t>
+          <t>163</t>
         </is>
       </c>
     </row>
     <row r="239" spans="1:29">
       <c r="A239" s="0" t="inlineStr">
         <is>
-          <t>KAMILA</t>
+          <t>HAJ HAUWA</t>
         </is>
       </c>
       <c r="B239" s="0" t="inlineStr">
         <is>
-          <t>HADEJA</t>
-        </is>
-      </c>
-      <c r="D239" s="0" t="inlineStr">
-        <is>
-          <t>+2347054680033</t>
+          <t>HABIB</t>
         </is>
       </c>
       <c r="R239" s="0" t="inlineStr">
@@ -8066,19 +8056,24 @@
       </c>
       <c r="AC239" s="0" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>264</t>
         </is>
       </c>
     </row>
     <row r="240" spans="1:29">
       <c r="A240" s="0" t="inlineStr">
         <is>
-          <t>HAJ RAKIYA</t>
+          <t>KAMILA</t>
         </is>
       </c>
       <c r="B240" s="0" t="inlineStr">
         <is>
-          <t>HAMZA</t>
+          <t>HADEJA</t>
+        </is>
+      </c>
+      <c r="D240" s="0" t="inlineStr">
+        <is>
+          <t>+2347054680033</t>
         </is>
       </c>
       <c r="R240" s="0" t="inlineStr">
@@ -8103,14 +8098,14 @@
       </c>
       <c r="AC240" s="0" t="inlineStr">
         <is>
-          <t>291</t>
+          <t>199</t>
         </is>
       </c>
     </row>
     <row r="241" spans="1:29">
       <c r="A241" s="0" t="inlineStr">
         <is>
-          <t>HAJ HAFSAT</t>
+          <t>HAJ RAKIYA</t>
         </is>
       </c>
       <c r="B241" s="0" t="inlineStr">
@@ -8140,19 +8135,19 @@
       </c>
       <c r="AC241" s="0" t="inlineStr">
         <is>
-          <t>306</t>
+          <t>291</t>
         </is>
       </c>
     </row>
     <row r="242" spans="1:29">
       <c r="A242" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>HAJ HAFSAT</t>
         </is>
       </c>
       <c r="B242" s="0" t="inlineStr">
         <is>
-          <t>HANIFA GOMBE</t>
+          <t>HAMZA</t>
         </is>
       </c>
       <c r="R242" s="0" t="inlineStr">
@@ -8162,7 +8157,7 @@
       </c>
       <c r="X242" s="0" t="inlineStr">
         <is>
-          <t>279000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z242" s="0" t="inlineStr">
@@ -8177,19 +8172,19 @@
       </c>
       <c r="AC242" s="0" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>306</t>
         </is>
       </c>
     </row>
     <row r="243" spans="1:29">
       <c r="A243" s="0" t="inlineStr">
         <is>
-          <t>MAIMUNA</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B243" s="0" t="inlineStr">
         <is>
-          <t>HASSAN</t>
+          <t>HANIFA GOMBE</t>
         </is>
       </c>
       <c r="R243" s="0" t="inlineStr">
@@ -8199,7 +8194,7 @@
       </c>
       <c r="X243" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>279000.00</t>
         </is>
       </c>
       <c r="Z243" s="0" t="inlineStr">
@@ -8214,14 +8209,14 @@
       </c>
       <c r="AC243" s="0" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>120</t>
         </is>
       </c>
     </row>
     <row r="244" spans="1:29">
       <c r="A244" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>MAIMUNA</t>
         </is>
       </c>
       <c r="B244" s="0" t="inlineStr">
@@ -8236,7 +8231,7 @@
       </c>
       <c r="X244" s="0" t="inlineStr">
         <is>
-          <t>26000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z244" s="0" t="inlineStr">
@@ -8251,19 +8246,19 @@
       </c>
       <c r="AC244" s="0" t="inlineStr">
         <is>
-          <t>326</t>
+          <t>323</t>
         </is>
       </c>
     </row>
     <row r="245" spans="1:29">
       <c r="A245" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B245" s="0" t="inlineStr">
         <is>
-          <t>HISHAM - ABK</t>
+          <t>HASSAN</t>
         </is>
       </c>
       <c r="R245" s="0" t="inlineStr">
@@ -8273,7 +8268,7 @@
       </c>
       <c r="X245" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>26000.00</t>
         </is>
       </c>
       <c r="Z245" s="0" t="inlineStr">
@@ -8288,19 +8283,19 @@
       </c>
       <c r="AC245" s="0" t="inlineStr">
         <is>
-          <t>215</t>
+          <t>326</t>
         </is>
       </c>
     </row>
     <row r="246" spans="1:29">
       <c r="A246" s="0" t="inlineStr">
         <is>
-          <t>MALAMA</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B246" s="0" t="inlineStr">
         <is>
-          <t>HUSSAINA</t>
+          <t>HISHAM - ABK</t>
         </is>
       </c>
       <c r="R246" s="0" t="inlineStr">
@@ -8310,7 +8305,7 @@
       </c>
       <c r="X246" s="0" t="inlineStr">
         <is>
-          <t>590000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z246" s="0" t="inlineStr">
@@ -8325,19 +8320,19 @@
       </c>
       <c r="AC246" s="0" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>215</t>
         </is>
       </c>
     </row>
     <row r="247" spans="1:29">
       <c r="A247" s="0" t="inlineStr">
         <is>
-          <t>SA'ADATU </t>
+          <t>MALAMA</t>
         </is>
       </c>
       <c r="B247" s="0" t="inlineStr">
         <is>
-          <t>HUSSAINI</t>
+          <t>HUSSAINA</t>
         </is>
       </c>
       <c r="R247" s="0" t="inlineStr">
@@ -8347,7 +8342,7 @@
       </c>
       <c r="X247" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>590000.00</t>
         </is>
       </c>
       <c r="Z247" s="0" t="inlineStr">
@@ -8362,14 +8357,14 @@
       </c>
       <c r="AC247" s="0" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>141</t>
         </is>
       </c>
     </row>
     <row r="248" spans="1:29">
       <c r="A248" s="0" t="inlineStr">
         <is>
-          <t>UMRATU</t>
+          <t>SA'ADATU </t>
         </is>
       </c>
       <c r="B248" s="0" t="inlineStr">
@@ -8399,19 +8394,19 @@
       </c>
       <c r="AC248" s="0" t="inlineStr">
         <is>
-          <t>322</t>
+          <t>131</t>
         </is>
       </c>
     </row>
     <row r="249" spans="1:29">
       <c r="A249" s="0" t="inlineStr">
         <is>
-          <t>FARIDA </t>
+          <t>UMRATU</t>
         </is>
       </c>
       <c r="B249" s="0" t="inlineStr">
         <is>
-          <t>IBRAHIM</t>
+          <t>HUSSAINI</t>
         </is>
       </c>
       <c r="R249" s="0" t="inlineStr">
@@ -8421,7 +8416,7 @@
       </c>
       <c r="X249" s="0" t="inlineStr">
         <is>
-          <t>8500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z249" s="0" t="inlineStr">
@@ -8436,14 +8431,14 @@
       </c>
       <c r="AC249" s="0" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>322</t>
         </is>
       </c>
     </row>
     <row r="250" spans="1:29">
       <c r="A250" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>FARIDA </t>
         </is>
       </c>
       <c r="B250" s="0" t="inlineStr">
@@ -8458,7 +8453,7 @@
       </c>
       <c r="X250" s="0" t="inlineStr">
         <is>
-          <t>35000.00</t>
+          <t>8500.00</t>
         </is>
       </c>
       <c r="Z250" s="0" t="inlineStr">
@@ -8473,24 +8468,19 @@
       </c>
       <c r="AC250" s="0" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>224</t>
         </is>
       </c>
     </row>
     <row r="251" spans="1:29">
       <c r="A251" s="0" t="inlineStr">
         <is>
-          <t>SALISU</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B251" s="0" t="inlineStr">
         <is>
-          <t>IDRIS</t>
-        </is>
-      </c>
-      <c r="D251" s="0" t="inlineStr">
-        <is>
-          <t>08184133063</t>
+          <t>IBRAHIM</t>
         </is>
       </c>
       <c r="R251" s="0" t="inlineStr">
@@ -8500,7 +8490,7 @@
       </c>
       <c r="X251" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>35000.00</t>
         </is>
       </c>
       <c r="Z251" s="0" t="inlineStr">
@@ -8515,54 +8505,24 @@
       </c>
       <c r="AC251" s="0" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>225</t>
         </is>
       </c>
     </row>
     <row r="252" spans="1:29">
       <c r="A252" s="0" t="inlineStr">
         <is>
-          <t>Ibrahim BB</t>
+          <t>SALISU</t>
         </is>
       </c>
       <c r="B252" s="0" t="inlineStr">
         <is>
-          <t>Jafar</t>
+          <t>IDRIS</t>
         </is>
       </c>
       <c r="D252" s="0" t="inlineStr">
         <is>
-          <t>08146595795</t>
-        </is>
-      </c>
-      <c r="J252" s="0" t="inlineStr">
-        <is>
-          <t>No 393 Rangi Quaters, Tudun Murtala, Nassarawa Kano</t>
-        </is>
-      </c>
-      <c r="L252" s="0" t="inlineStr">
-        <is>
-          <t>Kano</t>
-        </is>
-      </c>
-      <c r="M252" s="0" t="inlineStr">
-        <is>
-          <t>Kano</t>
-        </is>
-      </c>
-      <c r="N252" s="0" t="inlineStr">
-        <is>
-          <t>700281</t>
-        </is>
-      </c>
-      <c r="O252" s="0" t="inlineStr">
-        <is>
-          <t>Nigeria</t>
-        </is>
-      </c>
-      <c r="Q252" s="0" t="inlineStr">
-        <is>
-          <t>1522263645</t>
+          <t>08184133063</t>
         </is>
       </c>
       <c r="R252" s="0" t="inlineStr">
@@ -8570,31 +8530,11 @@
           <t>y</t>
         </is>
       </c>
-      <c r="T252" s="0" t="inlineStr">
-        <is>
-          <t>Tahir General Merchant</t>
-        </is>
-      </c>
-      <c r="V252" s="0" t="inlineStr">
-        <is>
-          <t>High-value returning customer. Frequently purchases in bulk during seasonal periods. Offer priority support and notify early about new stock arrivals or discounts.</t>
-        </is>
-      </c>
-      <c r="W252" s="0" t="inlineStr">
-        <is>
-          <t>REGULAR customer, with less than 5% discounts on sales.</t>
-        </is>
-      </c>
       <c r="X252" s="0" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>
       </c>
-      <c r="Y252" s="0" t="inlineStr">
-        <is>
-          <t>50000000.00</t>
-        </is>
-      </c>
       <c r="Z252" s="0" t="inlineStr">
         <is>
           <t>n</t>
@@ -8607,19 +8547,54 @@
       </c>
       <c r="AC252" s="0" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>17</t>
         </is>
       </c>
     </row>
     <row r="253" spans="1:29">
       <c r="A253" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>Ibrahim BB</t>
         </is>
       </c>
       <c r="B253" s="0" t="inlineStr">
         <is>
-          <t>JARMA</t>
+          <t>Jafar</t>
+        </is>
+      </c>
+      <c r="D253" s="0" t="inlineStr">
+        <is>
+          <t>08146595795</t>
+        </is>
+      </c>
+      <c r="J253" s="0" t="inlineStr">
+        <is>
+          <t>No 393 Rangi Quaters, Tudun Murtala, Nassarawa Kano</t>
+        </is>
+      </c>
+      <c r="L253" s="0" t="inlineStr">
+        <is>
+          <t>Kano</t>
+        </is>
+      </c>
+      <c r="M253" s="0" t="inlineStr">
+        <is>
+          <t>Kano</t>
+        </is>
+      </c>
+      <c r="N253" s="0" t="inlineStr">
+        <is>
+          <t>700281</t>
+        </is>
+      </c>
+      <c r="O253" s="0" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="Q253" s="0" t="inlineStr">
+        <is>
+          <t>1522263645</t>
         </is>
       </c>
       <c r="R253" s="0" t="inlineStr">
@@ -8627,11 +8602,31 @@
           <t>y</t>
         </is>
       </c>
+      <c r="T253" s="0" t="inlineStr">
+        <is>
+          <t>Tahir General Merchant</t>
+        </is>
+      </c>
+      <c r="V253" s="0" t="inlineStr">
+        <is>
+          <t>High-value returning customer. Frequently purchases in bulk during seasonal periods. Offer priority support and notify early about new stock arrivals or discounts.</t>
+        </is>
+      </c>
+      <c r="W253" s="0" t="inlineStr">
+        <is>
+          <t>REGULAR customer, with less than 5% discounts on sales.</t>
+        </is>
+      </c>
       <c r="X253" s="0" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>
       </c>
+      <c r="Y253" s="0" t="inlineStr">
+        <is>
+          <t>50000000.00</t>
+        </is>
+      </c>
       <c r="Z253" s="0" t="inlineStr">
         <is>
           <t>n</t>
@@ -8644,19 +8639,19 @@
       </c>
       <c r="AC253" s="0" t="inlineStr">
         <is>
-          <t>274</t>
+          <t>31</t>
         </is>
       </c>
     </row>
     <row r="254" spans="1:29">
       <c r="A254" s="0" t="inlineStr">
         <is>
-          <t>SUMAYYA</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B254" s="0" t="inlineStr">
         <is>
-          <t>JEGA</t>
+          <t>JARMA</t>
         </is>
       </c>
       <c r="R254" s="0" t="inlineStr">
@@ -8666,7 +8661,7 @@
       </c>
       <c r="X254" s="0" t="inlineStr">
         <is>
-          <t>10000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z254" s="0" t="inlineStr">
@@ -8681,19 +8676,19 @@
       </c>
       <c r="AC254" s="0" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>274</t>
         </is>
       </c>
     </row>
     <row r="255" spans="1:29">
       <c r="A255" s="0" t="inlineStr">
         <is>
-          <t>PHIL</t>
+          <t>SUMAYYA</t>
         </is>
       </c>
       <c r="B255" s="0" t="inlineStr">
         <is>
-          <t>JULIUS</t>
+          <t>JEGA</t>
         </is>
       </c>
       <c r="R255" s="0" t="inlineStr">
@@ -8703,7 +8698,7 @@
       </c>
       <c r="X255" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>10000.00</t>
         </is>
       </c>
       <c r="Z255" s="0" t="inlineStr">
@@ -8718,19 +8713,19 @@
       </c>
       <c r="AC255" s="0" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>114</t>
         </is>
       </c>
     </row>
     <row r="256" spans="1:29">
       <c r="A256" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>PHIL</t>
         </is>
       </c>
       <c r="B256" s="0" t="inlineStr">
         <is>
-          <t>JUMARE</t>
+          <t>JULIUS</t>
         </is>
       </c>
       <c r="R256" s="0" t="inlineStr">
@@ -8740,7 +8735,7 @@
       </c>
       <c r="X256" s="0" t="inlineStr">
         <is>
-          <t>298000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z256" s="0" t="inlineStr">
@@ -8755,29 +8750,19 @@
       </c>
       <c r="AC256" s="0" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>255</t>
         </is>
       </c>
     </row>
     <row r="257" spans="1:29">
       <c r="A257" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B257" s="0" t="inlineStr">
         <is>
-          <t>KADUNA</t>
-        </is>
-      </c>
-      <c r="L257" s="0" t="inlineStr">
-        <is>
-          <t>KADUNA</t>
-        </is>
-      </c>
-      <c r="M257" s="0" t="inlineStr">
-        <is>
-          <t>KADUNA</t>
+          <t>JUMARE</t>
         </is>
       </c>
       <c r="R257" s="0" t="inlineStr">
@@ -8787,7 +8772,7 @@
       </c>
       <c r="X257" s="0" t="inlineStr">
         <is>
-          <t>397500.00</t>
+          <t>506500.00</t>
         </is>
       </c>
       <c r="Z257" s="0" t="inlineStr">
@@ -8802,14 +8787,14 @@
       </c>
       <c r="AC257" s="0" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>129</t>
         </is>
       </c>
     </row>
     <row r="258" spans="1:29">
       <c r="A258" s="0" t="inlineStr">
         <is>
-          <t>HAJ FATIMA</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B258" s="0" t="inlineStr">
@@ -8817,6 +8802,16 @@
           <t>KADUNA</t>
         </is>
       </c>
+      <c r="L258" s="0" t="inlineStr">
+        <is>
+          <t>KADUNA</t>
+        </is>
+      </c>
+      <c r="M258" s="0" t="inlineStr">
+        <is>
+          <t>KADUNA</t>
+        </is>
+      </c>
       <c r="R258" s="0" t="inlineStr">
         <is>
           <t>y</t>
@@ -8824,7 +8819,7 @@
       </c>
       <c r="X258" s="0" t="inlineStr">
         <is>
-          <t>630500.00</t>
+          <t>397500.00</t>
         </is>
       </c>
       <c r="Z258" s="0" t="inlineStr">
@@ -8839,14 +8834,14 @@
       </c>
       <c r="AC258" s="0" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>82</t>
         </is>
       </c>
     </row>
     <row r="259" spans="1:29">
       <c r="A259" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>HAJ FATIMA</t>
         </is>
       </c>
       <c r="B259" s="0" t="inlineStr">
@@ -8861,7 +8856,7 @@
       </c>
       <c r="X259" s="0" t="inlineStr">
         <is>
-          <t>127500.00</t>
+          <t>642500.00</t>
         </is>
       </c>
       <c r="Z259" s="0" t="inlineStr">
@@ -8876,19 +8871,19 @@
       </c>
       <c r="AC259" s="0" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>91</t>
         </is>
       </c>
     </row>
     <row r="260" spans="1:29">
       <c r="A260" s="0" t="inlineStr">
         <is>
-          <t>SA'ADATU</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B260" s="0" t="inlineStr">
         <is>
-          <t>KANGIWA</t>
+          <t>KADUNA</t>
         </is>
       </c>
       <c r="R260" s="0" t="inlineStr">
@@ -8898,7 +8893,7 @@
       </c>
       <c r="X260" s="0" t="inlineStr">
         <is>
-          <t>200000.00</t>
+          <t>127500.00</t>
         </is>
       </c>
       <c r="Z260" s="0" t="inlineStr">
@@ -8913,19 +8908,19 @@
       </c>
       <c r="AC260" s="0" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>95</t>
         </is>
       </c>
     </row>
     <row r="261" spans="1:29">
       <c r="A261" s="0" t="inlineStr">
         <is>
-          <t>MOMY</t>
+          <t>SA'ADATU</t>
         </is>
       </c>
       <c r="B261" s="0" t="inlineStr">
         <is>
-          <t>KARETO</t>
+          <t>KANGIWA</t>
         </is>
       </c>
       <c r="R261" s="0" t="inlineStr">
@@ -8935,7 +8930,7 @@
       </c>
       <c r="X261" s="0" t="inlineStr">
         <is>
-          <t>240000.00</t>
+          <t>200000.00</t>
         </is>
       </c>
       <c r="Z261" s="0" t="inlineStr">
@@ -8950,19 +8945,19 @@
       </c>
       <c r="AC261" s="0" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>109</t>
         </is>
       </c>
     </row>
     <row r="262" spans="1:29">
       <c r="A262" s="0" t="inlineStr">
         <is>
-          <t>JIDDAH</t>
+          <t>MOMY</t>
         </is>
       </c>
       <c r="B262" s="0" t="inlineStr">
         <is>
-          <t>KATSINA</t>
+          <t>KARETO</t>
         </is>
       </c>
       <c r="R262" s="0" t="inlineStr">
@@ -8972,7 +8967,7 @@
       </c>
       <c r="X262" s="0" t="inlineStr">
         <is>
-          <t>45000.00</t>
+          <t>240000.00</t>
         </is>
       </c>
       <c r="Z262" s="0" t="inlineStr">
@@ -8987,14 +8982,14 @@
       </c>
       <c r="AC262" s="0" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>157</t>
         </is>
       </c>
     </row>
     <row r="263" spans="1:29">
       <c r="A263" s="0" t="inlineStr">
         <is>
-          <t>ANTY FATIMA</t>
+          <t>JIDDAH</t>
         </is>
       </c>
       <c r="B263" s="0" t="inlineStr">
@@ -9009,7 +9004,7 @@
       </c>
       <c r="X263" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>45000.00</t>
         </is>
       </c>
       <c r="Z263" s="0" t="inlineStr">
@@ -9024,14 +9019,14 @@
       </c>
       <c r="AC263" s="0" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>77</t>
         </is>
       </c>
     </row>
     <row r="264" spans="1:29">
       <c r="A264" s="0" t="inlineStr">
         <is>
-          <t>HAJ ZAINAB</t>
+          <t>ANTY FATIMA</t>
         </is>
       </c>
       <c r="B264" s="0" t="inlineStr">
@@ -9061,14 +9056,14 @@
       </c>
       <c r="AC264" s="0" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="265" spans="1:29">
       <c r="A265" s="0" t="inlineStr">
         <is>
-          <t>HAJ HADIZA</t>
+          <t>HAJ ZAINAB</t>
         </is>
       </c>
       <c r="B265" s="0" t="inlineStr">
@@ -9098,14 +9093,14 @@
       </c>
       <c r="AC265" s="0" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>92</t>
         </is>
       </c>
     </row>
     <row r="266" spans="1:29">
       <c r="A266" s="0" t="inlineStr">
         <is>
-          <t>SUMAYYA</t>
+          <t>HAJ HADIZA</t>
         </is>
       </c>
       <c r="B266" s="0" t="inlineStr">
@@ -9135,14 +9130,14 @@
       </c>
       <c r="AC266" s="0" t="inlineStr">
         <is>
-          <t>186</t>
+          <t>108</t>
         </is>
       </c>
     </row>
     <row r="267" spans="1:29">
       <c r="A267" s="0" t="inlineStr">
         <is>
-          <t>HADIZA</t>
+          <t>SUMAYYA</t>
         </is>
       </c>
       <c r="B267" s="0" t="inlineStr">
@@ -9157,7 +9152,7 @@
       </c>
       <c r="X267" s="0" t="inlineStr">
         <is>
-          <t>12000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z267" s="0" t="inlineStr">
@@ -9172,19 +9167,19 @@
       </c>
       <c r="AC267" s="0" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>186</t>
         </is>
       </c>
     </row>
     <row r="268" spans="1:29">
       <c r="A268" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>HADIZA</t>
         </is>
       </c>
       <c r="B268" s="0" t="inlineStr">
         <is>
-          <t>KAUSAR</t>
+          <t>KATSINA</t>
         </is>
       </c>
       <c r="R268" s="0" t="inlineStr">
@@ -9194,7 +9189,7 @@
       </c>
       <c r="X268" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>12000.00</t>
         </is>
       </c>
       <c r="Z268" s="0" t="inlineStr">
@@ -9209,7 +9204,7 @@
       </c>
       <c r="AC268" s="0" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>213</t>
         </is>
       </c>
     </row>
@@ -9221,7 +9216,7 @@
       </c>
       <c r="B269" s="0" t="inlineStr">
         <is>
-          <t>KHALIFA KATSINA</t>
+          <t>KAUSAR</t>
         </is>
       </c>
       <c r="R269" s="0" t="inlineStr">
@@ -9231,7 +9226,7 @@
       </c>
       <c r="X269" s="0" t="inlineStr">
         <is>
-          <t>324500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z269" s="0" t="inlineStr">
@@ -9246,19 +9241,19 @@
       </c>
       <c r="AC269" s="0" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>160</t>
         </is>
       </c>
     </row>
     <row r="270" spans="1:29">
       <c r="A270" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B270" s="0" t="inlineStr">
         <is>
-          <t>KOLMANI</t>
+          <t>KHALIFA KATSINA</t>
         </is>
       </c>
       <c r="R270" s="0" t="inlineStr">
@@ -9268,7 +9263,7 @@
       </c>
       <c r="X270" s="0" t="inlineStr">
         <is>
-          <t>40000.00</t>
+          <t>324500.00</t>
         </is>
       </c>
       <c r="Z270" s="0" t="inlineStr">
@@ -9283,19 +9278,19 @@
       </c>
       <c r="AC270" s="0" t="inlineStr">
         <is>
-          <t>205</t>
+          <t>106</t>
         </is>
       </c>
     </row>
     <row r="271" spans="1:29">
       <c r="A271" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B271" s="0" t="inlineStr">
         <is>
-          <t>KWAIRANGA</t>
+          <t>KOLMANI</t>
         </is>
       </c>
       <c r="R271" s="0" t="inlineStr">
@@ -9305,7 +9300,7 @@
       </c>
       <c r="X271" s="0" t="inlineStr">
         <is>
-          <t>1469000.00</t>
+          <t>40000.00</t>
         </is>
       </c>
       <c r="Z271" s="0" t="inlineStr">
@@ -9320,19 +9315,19 @@
       </c>
       <c r="AC271" s="0" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>205</t>
         </is>
       </c>
     </row>
     <row r="272" spans="1:29">
       <c r="A272" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B272" s="0" t="inlineStr">
         <is>
-          <t>KYARI</t>
+          <t>KWAIRANGA</t>
         </is>
       </c>
       <c r="R272" s="0" t="inlineStr">
@@ -9342,7 +9337,7 @@
       </c>
       <c r="X272" s="0" t="inlineStr">
         <is>
-          <t>40000.00</t>
+          <t>1469000.00</t>
         </is>
       </c>
       <c r="Z272" s="0" t="inlineStr">
@@ -9357,19 +9352,19 @@
       </c>
       <c r="AC272" s="0" t="inlineStr">
         <is>
-          <t>292</t>
+          <t>104</t>
         </is>
       </c>
     </row>
     <row r="273" spans="1:29">
       <c r="A273" s="0" t="inlineStr">
         <is>
-          <t>HADIZA</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B273" s="0" t="inlineStr">
         <is>
-          <t>LABO</t>
+          <t>KYARI</t>
         </is>
       </c>
       <c r="R273" s="0" t="inlineStr">
@@ -9379,7 +9374,7 @@
       </c>
       <c r="X273" s="0" t="inlineStr">
         <is>
-          <t>1056900.00</t>
+          <t>40000.00</t>
         </is>
       </c>
       <c r="Z273" s="0" t="inlineStr">
@@ -9394,14 +9389,14 @@
       </c>
       <c r="AC273" s="0" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>292</t>
         </is>
       </c>
     </row>
     <row r="274" spans="1:29">
       <c r="A274" s="0" t="inlineStr">
         <is>
-          <t>UMMI</t>
+          <t>HADIZA</t>
         </is>
       </c>
       <c r="B274" s="0" t="inlineStr">
@@ -9416,7 +9411,7 @@
       </c>
       <c r="X274" s="0" t="inlineStr">
         <is>
-          <t>1678300.00</t>
+          <t>1056900.00</t>
         </is>
       </c>
       <c r="Z274" s="0" t="inlineStr">
@@ -9431,19 +9426,19 @@
       </c>
       <c r="AC274" s="0" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>88</t>
         </is>
       </c>
     </row>
     <row r="275" spans="1:29">
       <c r="A275" s="0" t="inlineStr">
         <is>
-          <t>INNAN</t>
+          <t>UMMI</t>
         </is>
       </c>
       <c r="B275" s="0" t="inlineStr">
         <is>
-          <t>LARAI</t>
+          <t>LABO</t>
         </is>
       </c>
       <c r="R275" s="0" t="inlineStr">
@@ -9453,7 +9448,7 @@
       </c>
       <c r="X275" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1678300.00</t>
         </is>
       </c>
       <c r="Z275" s="0" t="inlineStr">
@@ -9468,19 +9463,19 @@
       </c>
       <c r="AC275" s="0" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>119</t>
         </is>
       </c>
     </row>
     <row r="276" spans="1:29">
       <c r="A276" s="0" t="inlineStr">
         <is>
-          <t>RAHAMA</t>
+          <t>INNAN</t>
         </is>
       </c>
       <c r="B276" s="0" t="inlineStr">
         <is>
-          <t>LAWAL</t>
+          <t>LARAI</t>
         </is>
       </c>
       <c r="R276" s="0" t="inlineStr">
@@ -9490,7 +9485,7 @@
       </c>
       <c r="X276" s="0" t="inlineStr">
         <is>
-          <t>35000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z276" s="0" t="inlineStr">
@@ -9505,14 +9500,14 @@
       </c>
       <c r="AC276" s="0" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>84</t>
         </is>
       </c>
     </row>
     <row r="277" spans="1:29">
       <c r="A277" s="0" t="inlineStr">
         <is>
-          <t>HAJ HADIZA</t>
+          <t>RAHAMA</t>
         </is>
       </c>
       <c r="B277" s="0" t="inlineStr">
@@ -9527,7 +9522,7 @@
       </c>
       <c r="X277" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>55000.00</t>
         </is>
       </c>
       <c r="Z277" s="0" t="inlineStr">
@@ -9542,19 +9537,19 @@
       </c>
       <c r="AC277" s="0" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>80</t>
         </is>
       </c>
     </row>
     <row r="278" spans="1:29">
       <c r="A278" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>HAJ HADIZA</t>
         </is>
       </c>
       <c r="B278" s="0" t="inlineStr">
         <is>
-          <t>MACHINA</t>
+          <t>LAWAL</t>
         </is>
       </c>
       <c r="R278" s="0" t="inlineStr">
@@ -9564,7 +9559,7 @@
       </c>
       <c r="X278" s="0" t="inlineStr">
         <is>
-          <t>136000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z278" s="0" t="inlineStr">
@@ -9579,7 +9574,7 @@
       </c>
       <c r="AC278" s="0" t="inlineStr">
         <is>
-          <t>296</t>
+          <t>310</t>
         </is>
       </c>
     </row>
@@ -9591,7 +9586,7 @@
       </c>
       <c r="B279" s="0" t="inlineStr">
         <is>
-          <t>MADU</t>
+          <t>MACHINA</t>
         </is>
       </c>
       <c r="R279" s="0" t="inlineStr">
@@ -9601,7 +9596,7 @@
       </c>
       <c r="X279" s="0" t="inlineStr">
         <is>
-          <t>48000.00</t>
+          <t>136000.00</t>
         </is>
       </c>
       <c r="Z279" s="0" t="inlineStr">
@@ -9616,19 +9611,19 @@
       </c>
       <c r="AC279" s="0" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>296</t>
         </is>
       </c>
     </row>
     <row r="280" spans="1:29">
       <c r="A280" s="0" t="inlineStr">
         <is>
-          <t>RAHAMA</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B280" s="0" t="inlineStr">
         <is>
-          <t>MAHMUD</t>
+          <t>MADU</t>
         </is>
       </c>
       <c r="R280" s="0" t="inlineStr">
@@ -9638,7 +9633,7 @@
       </c>
       <c r="X280" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>48000.00</t>
         </is>
       </c>
       <c r="Z280" s="0" t="inlineStr">
@@ -9653,19 +9648,19 @@
       </c>
       <c r="AC280" s="0" t="inlineStr">
         <is>
-          <t>311</t>
+          <t>151</t>
         </is>
       </c>
     </row>
     <row r="281" spans="1:29">
       <c r="A281" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>RAHAMA</t>
         </is>
       </c>
       <c r="B281" s="0" t="inlineStr">
         <is>
-          <t>MAIGARI</t>
+          <t>MAHMUD</t>
         </is>
       </c>
       <c r="R281" s="0" t="inlineStr">
@@ -9675,7 +9670,7 @@
       </c>
       <c r="X281" s="0" t="inlineStr">
         <is>
-          <t>2498300.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z281" s="0" t="inlineStr">
@@ -9690,19 +9685,19 @@
       </c>
       <c r="AC281" s="0" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>311</t>
         </is>
       </c>
     </row>
     <row r="282" spans="1:29">
       <c r="A282" s="0" t="inlineStr">
         <is>
-          <t>ZUWAIRA</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B282" s="0" t="inlineStr">
         <is>
-          <t>MAJIDADI</t>
+          <t>MAIGARI</t>
         </is>
       </c>
       <c r="R282" s="0" t="inlineStr">
@@ -9712,7 +9707,7 @@
       </c>
       <c r="X282" s="0" t="inlineStr">
         <is>
-          <t>74800.00</t>
+          <t>2498300.00</t>
         </is>
       </c>
       <c r="Z282" s="0" t="inlineStr">
@@ -9727,19 +9722,19 @@
       </c>
       <c r="AC282" s="0" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>162</t>
         </is>
       </c>
     </row>
     <row r="283" spans="1:29">
       <c r="A283" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>ZUWAIRA</t>
         </is>
       </c>
       <c r="B283" s="0" t="inlineStr">
         <is>
-          <t>MALAM</t>
+          <t>MAJIDADI</t>
         </is>
       </c>
       <c r="R283" s="0" t="inlineStr">
@@ -9749,7 +9744,7 @@
       </c>
       <c r="X283" s="0" t="inlineStr">
         <is>
-          <t>26500.00</t>
+          <t>74800.00</t>
         </is>
       </c>
       <c r="Z283" s="0" t="inlineStr">
@@ -9764,19 +9759,19 @@
       </c>
       <c r="AC283" s="0" t="inlineStr">
         <is>
-          <t>316</t>
+          <t>207</t>
         </is>
       </c>
     </row>
     <row r="284" spans="1:29">
       <c r="A284" s="0" t="inlineStr">
         <is>
-          <t>AISHA</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B284" s="0" t="inlineStr">
         <is>
-          <t>MALUMFASHI</t>
+          <t>MALAM</t>
         </is>
       </c>
       <c r="R284" s="0" t="inlineStr">
@@ -9786,7 +9781,7 @@
       </c>
       <c r="X284" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>26500.00</t>
         </is>
       </c>
       <c r="Z284" s="0" t="inlineStr">
@@ -9801,19 +9796,19 @@
       </c>
       <c r="AC284" s="0" t="inlineStr">
         <is>
-          <t>124</t>
+          <t>316</t>
         </is>
       </c>
     </row>
     <row r="285" spans="1:29">
       <c r="A285" s="0" t="inlineStr">
         <is>
-          <t>DJA</t>
+          <t>AISHA</t>
         </is>
       </c>
       <c r="B285" s="0" t="inlineStr">
         <is>
-          <t>MAMAN ABDALLAH</t>
+          <t>MALUMFASHI</t>
         </is>
       </c>
       <c r="R285" s="0" t="inlineStr">
@@ -9823,7 +9818,7 @@
       </c>
       <c r="X285" s="0" t="inlineStr">
         <is>
-          <t>147000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z285" s="0" t="inlineStr">
@@ -9838,19 +9833,19 @@
       </c>
       <c r="AC285" s="0" t="inlineStr">
         <is>
-          <t>178</t>
+          <t>124</t>
         </is>
       </c>
     </row>
     <row r="286" spans="1:29">
       <c r="A286" s="0" t="inlineStr">
         <is>
-          <t>UMMU</t>
+          <t>DJA</t>
         </is>
       </c>
       <c r="B286" s="0" t="inlineStr">
         <is>
-          <t>MAMAN UWAIS</t>
+          <t>MAMAN ABDALLAH</t>
         </is>
       </c>
       <c r="R286" s="0" t="inlineStr">
@@ -9860,7 +9855,7 @@
       </c>
       <c r="X286" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>147000.00</t>
         </is>
       </c>
       <c r="Z286" s="0" t="inlineStr">
@@ -9875,19 +9870,19 @@
       </c>
       <c r="AC286" s="0" t="inlineStr">
         <is>
-          <t>271</t>
+          <t>178</t>
         </is>
       </c>
     </row>
     <row r="287" spans="1:29">
       <c r="A287" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>UMMU</t>
         </is>
       </c>
       <c r="B287" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>MAMAN UWAIS</t>
         </is>
       </c>
       <c r="R287" s="0" t="inlineStr">
@@ -9912,19 +9907,19 @@
       </c>
       <c r="AC287" s="0" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>271</t>
         </is>
       </c>
     </row>
     <row r="288" spans="1:29">
       <c r="A288" s="0" t="inlineStr">
         <is>
-          <t>HAJ FATIMA</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B288" s="0" t="inlineStr">
         <is>
-          <t>MUHD</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="R288" s="0" t="inlineStr">
@@ -9949,14 +9944,14 @@
       </c>
       <c r="AC288" s="0" t="inlineStr">
         <is>
-          <t>247</t>
+          <t>94</t>
         </is>
       </c>
     </row>
     <row r="289" spans="1:29">
       <c r="A289" s="0" t="inlineStr">
         <is>
-          <t>SHAMSIYYAH</t>
+          <t>HAJ FATIMA</t>
         </is>
       </c>
       <c r="B289" s="0" t="inlineStr">
@@ -9986,19 +9981,19 @@
       </c>
       <c r="AC289" s="0" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>247</t>
         </is>
       </c>
     </row>
     <row r="290" spans="1:29">
       <c r="A290" s="0" t="inlineStr">
         <is>
-          <t>BILKISU</t>
+          <t>SHAMSIYYAH</t>
         </is>
       </c>
       <c r="B290" s="0" t="inlineStr">
         <is>
-          <t>MUKHTAR</t>
+          <t>MUHD</t>
         </is>
       </c>
       <c r="R290" s="0" t="inlineStr">
@@ -10008,7 +10003,7 @@
       </c>
       <c r="X290" s="0" t="inlineStr">
         <is>
-          <t>173000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z290" s="0" t="inlineStr">
@@ -10023,19 +10018,19 @@
       </c>
       <c r="AC290" s="0" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>257</t>
         </is>
       </c>
     </row>
     <row r="291" spans="1:29">
       <c r="A291" s="0" t="inlineStr">
         <is>
-          <t>UMMI</t>
+          <t>BILKISU</t>
         </is>
       </c>
       <c r="B291" s="0" t="inlineStr">
         <is>
-          <t>MUMTAZ</t>
+          <t>MUKHTAR</t>
         </is>
       </c>
       <c r="R291" s="0" t="inlineStr">
@@ -10045,7 +10040,7 @@
       </c>
       <c r="X291" s="0" t="inlineStr">
         <is>
-          <t>3419000.00</t>
+          <t>173000.00</t>
         </is>
       </c>
       <c r="Z291" s="0" t="inlineStr">
@@ -10060,19 +10055,19 @@
       </c>
       <c r="AC291" s="0" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>138</t>
         </is>
       </c>
     </row>
     <row r="292" spans="1:29">
       <c r="A292" s="0" t="inlineStr">
         <is>
-          <t>MAMAN </t>
+          <t>UMMI</t>
         </is>
       </c>
       <c r="B292" s="0" t="inlineStr">
         <is>
-          <t>NABILA</t>
+          <t>MUMTAZ</t>
         </is>
       </c>
       <c r="R292" s="0" t="inlineStr">
@@ -10082,7 +10077,7 @@
       </c>
       <c r="X292" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>3419000.00</t>
         </is>
       </c>
       <c r="Z292" s="0" t="inlineStr">
@@ -10097,19 +10092,19 @@
       </c>
       <c r="AC292" s="0" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>140</t>
         </is>
       </c>
     </row>
     <row r="293" spans="1:29">
       <c r="A293" s="0" t="inlineStr">
         <is>
-          <t>ANTY</t>
+          <t>MAMAN </t>
         </is>
       </c>
       <c r="B293" s="0" t="inlineStr">
         <is>
-          <t>NAS</t>
+          <t>NABILA</t>
         </is>
       </c>
       <c r="R293" s="0" t="inlineStr">
@@ -10119,7 +10114,7 @@
       </c>
       <c r="X293" s="0" t="inlineStr">
         <is>
-          <t>1579000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z293" s="0" t="inlineStr">
@@ -10134,19 +10129,19 @@
       </c>
       <c r="AC293" s="0" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>87</t>
         </is>
       </c>
     </row>
     <row r="294" spans="1:29">
       <c r="A294" s="0" t="inlineStr">
         <is>
-          <t>RUKAYYA</t>
+          <t>ANTY</t>
         </is>
       </c>
       <c r="B294" s="0" t="inlineStr">
         <is>
-          <t>NASIR</t>
+          <t>NAS</t>
         </is>
       </c>
       <c r="R294" s="0" t="inlineStr">
@@ -10156,7 +10151,7 @@
       </c>
       <c r="X294" s="0" t="inlineStr">
         <is>
-          <t>516000.00</t>
+          <t>1979000.00</t>
         </is>
       </c>
       <c r="Z294" s="0" t="inlineStr">
@@ -10171,14 +10166,14 @@
       </c>
       <c r="AC294" s="0" t="inlineStr">
         <is>
-          <t>188</t>
+          <t>78</t>
         </is>
       </c>
     </row>
     <row r="295" spans="1:29">
       <c r="A295" s="0" t="inlineStr">
         <is>
-          <t>HAFSAT</t>
+          <t>RUKAYYA</t>
         </is>
       </c>
       <c r="B295" s="0" t="inlineStr">
@@ -10193,7 +10188,7 @@
       </c>
       <c r="X295" s="0" t="inlineStr">
         <is>
-          <t>22000.00</t>
+          <t>534000.00</t>
         </is>
       </c>
       <c r="Z295" s="0" t="inlineStr">
@@ -10208,19 +10203,19 @@
       </c>
       <c r="AC295" s="0" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>188</t>
         </is>
       </c>
     </row>
     <row r="296" spans="1:29">
       <c r="A296" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>HAFSAT</t>
         </is>
       </c>
       <c r="B296" s="0" t="inlineStr">
         <is>
-          <t>NATA'ALA</t>
+          <t>NASIR</t>
         </is>
       </c>
       <c r="R296" s="0" t="inlineStr">
@@ -10230,7 +10225,7 @@
       </c>
       <c r="X296" s="0" t="inlineStr">
         <is>
-          <t>33000.00</t>
+          <t>22000.00</t>
         </is>
       </c>
       <c r="Z296" s="0" t="inlineStr">
@@ -10245,19 +10240,19 @@
       </c>
       <c r="AC296" s="0" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>228</t>
         </is>
       </c>
     </row>
     <row r="297" spans="1:29">
       <c r="A297" s="0" t="inlineStr">
         <is>
-          <t>AMINA</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B297" s="0" t="inlineStr">
         <is>
-          <t>NINGI</t>
+          <t>NATA'ALA</t>
         </is>
       </c>
       <c r="R297" s="0" t="inlineStr">
@@ -10267,7 +10262,7 @@
       </c>
       <c r="X297" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>33000.00</t>
         </is>
       </c>
       <c r="Z297" s="0" t="inlineStr">
@@ -10282,19 +10277,19 @@
       </c>
       <c r="AC297" s="0" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>74</t>
         </is>
       </c>
     </row>
     <row r="298" spans="1:29">
       <c r="A298" s="0" t="inlineStr">
         <is>
-          <t>BILKIS</t>
+          <t>AMINA</t>
         </is>
       </c>
       <c r="B298" s="0" t="inlineStr">
         <is>
-          <t>ONLINE</t>
+          <t>NINGI</t>
         </is>
       </c>
       <c r="R298" s="0" t="inlineStr">
@@ -10319,19 +10314,19 @@
       </c>
       <c r="AC298" s="0" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>132</t>
         </is>
       </c>
     </row>
     <row r="299" spans="1:29">
       <c r="A299" s="0" t="inlineStr">
         <is>
-          <t>MADAM</t>
+          <t>BILKIS</t>
         </is>
       </c>
       <c r="B299" s="0" t="inlineStr">
         <is>
-          <t>RONKE</t>
+          <t>ONLINE</t>
         </is>
       </c>
       <c r="R299" s="0" t="inlineStr">
@@ -10356,19 +10351,19 @@
       </c>
       <c r="AC299" s="0" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>170</t>
         </is>
       </c>
     </row>
     <row r="300" spans="1:29">
       <c r="A300" s="0" t="inlineStr">
         <is>
-          <t>ASH</t>
+          <t>MADAM</t>
         </is>
       </c>
       <c r="B300" s="0" t="inlineStr">
         <is>
-          <t>RUKY</t>
+          <t>RONKE</t>
         </is>
       </c>
       <c r="R300" s="0" t="inlineStr">
@@ -10393,19 +10388,19 @@
       </c>
       <c r="AC300" s="0" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>226</t>
         </is>
       </c>
     </row>
     <row r="301" spans="1:29">
       <c r="A301" s="0" t="inlineStr">
         <is>
-          <t>IKILIMA</t>
+          <t>ASH</t>
         </is>
       </c>
       <c r="B301" s="0" t="inlineStr">
         <is>
-          <t>RUWAN DORAWA</t>
+          <t>RUKY</t>
         </is>
       </c>
       <c r="R301" s="0" t="inlineStr">
@@ -10430,19 +10425,19 @@
       </c>
       <c r="AC301" s="0" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>76</t>
         </is>
       </c>
     </row>
     <row r="302" spans="1:29">
       <c r="A302" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>IKILIMA</t>
         </is>
       </c>
       <c r="B302" s="0" t="inlineStr">
         <is>
-          <t>SAFWAN</t>
+          <t>RUWAN DORAWA</t>
         </is>
       </c>
       <c r="R302" s="0" t="inlineStr">
@@ -10452,7 +10447,7 @@
       </c>
       <c r="X302" s="0" t="inlineStr">
         <is>
-          <t>32000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z302" s="0" t="inlineStr">
@@ -10467,19 +10462,19 @@
       </c>
       <c r="AC302" s="0" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>139</t>
         </is>
       </c>
     </row>
     <row r="303" spans="1:29">
       <c r="A303" s="0" t="inlineStr">
         <is>
-          <t>SALMA</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B303" s="0" t="inlineStr">
         <is>
-          <t>SALMUR</t>
+          <t>SAFWAN</t>
         </is>
       </c>
       <c r="R303" s="0" t="inlineStr">
@@ -10489,7 +10484,7 @@
       </c>
       <c r="X303" s="0" t="inlineStr">
         <is>
-          <t>47500.00</t>
+          <t>32000.00</t>
         </is>
       </c>
       <c r="Z303" s="0" t="inlineStr">
@@ -10504,19 +10499,19 @@
       </c>
       <c r="AC303" s="0" t="inlineStr">
         <is>
-          <t>254</t>
+          <t>105</t>
         </is>
       </c>
     </row>
     <row r="304" spans="1:29">
       <c r="A304" s="0" t="inlineStr">
         <is>
-          <t>ASMI</t>
+          <t>SALMA</t>
         </is>
       </c>
       <c r="B304" s="0" t="inlineStr">
         <is>
-          <t>SAMBO</t>
+          <t>SALMUR</t>
         </is>
       </c>
       <c r="R304" s="0" t="inlineStr">
@@ -10526,7 +10521,7 @@
       </c>
       <c r="X304" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>47500.00</t>
         </is>
       </c>
       <c r="Z304" s="0" t="inlineStr">
@@ -10541,19 +10536,19 @@
       </c>
       <c r="AC304" s="0" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>254</t>
         </is>
       </c>
     </row>
     <row r="305" spans="1:29">
       <c r="A305" s="0" t="inlineStr">
         <is>
-          <t>SAMIHA</t>
+          <t>ASMI</t>
         </is>
       </c>
       <c r="B305" s="0" t="inlineStr">
         <is>
-          <t>SANI</t>
+          <t>SAMBO</t>
         </is>
       </c>
       <c r="R305" s="0" t="inlineStr">
@@ -10578,19 +10573,19 @@
       </c>
       <c r="AC305" s="0" t="inlineStr">
         <is>
-          <t>285</t>
+          <t>243</t>
         </is>
       </c>
     </row>
     <row r="306" spans="1:29">
       <c r="A306" s="0" t="inlineStr">
         <is>
-          <t>JAMILA</t>
+          <t>SAMIHA</t>
         </is>
       </c>
       <c r="B306" s="0" t="inlineStr">
         <is>
-          <t>SHANONO</t>
+          <t>SANI</t>
         </is>
       </c>
       <c r="R306" s="0" t="inlineStr">
@@ -10600,7 +10595,7 @@
       </c>
       <c r="X306" s="0" t="inlineStr">
         <is>
-          <t>443000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z306" s="0" t="inlineStr">
@@ -10615,19 +10610,19 @@
       </c>
       <c r="AC306" s="0" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>285</t>
         </is>
       </c>
     </row>
     <row r="307" spans="1:29">
       <c r="A307" s="0" t="inlineStr">
         <is>
-          <t>FARIDA</t>
+          <t>JAMILA</t>
         </is>
       </c>
       <c r="B307" s="0" t="inlineStr">
         <is>
-          <t>SHARADA</t>
+          <t>SHANONO</t>
         </is>
       </c>
       <c r="R307" s="0" t="inlineStr">
@@ -10637,7 +10632,7 @@
       </c>
       <c r="X307" s="0" t="inlineStr">
         <is>
-          <t>95000.00</t>
+          <t>443000.00</t>
         </is>
       </c>
       <c r="Z307" s="0" t="inlineStr">
@@ -10652,19 +10647,19 @@
       </c>
       <c r="AC307" s="0" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>83</t>
         </is>
       </c>
     </row>
     <row r="308" spans="1:29">
       <c r="A308" s="0" t="inlineStr">
         <is>
-          <t>FANNE</t>
+          <t>FARIDA</t>
         </is>
       </c>
       <c r="B308" s="0" t="inlineStr">
         <is>
-          <t>SHARIF</t>
+          <t>SHARADA</t>
         </is>
       </c>
       <c r="R308" s="0" t="inlineStr">
@@ -10674,7 +10669,7 @@
       </c>
       <c r="X308" s="0" t="inlineStr">
         <is>
-          <t>350000.00</t>
+          <t>95000.00</t>
         </is>
       </c>
       <c r="Z308" s="0" t="inlineStr">
@@ -10689,19 +10684,19 @@
       </c>
       <c r="AC308" s="0" t="inlineStr">
         <is>
-          <t>179</t>
+          <t>115</t>
         </is>
       </c>
     </row>
     <row r="309" spans="1:29">
       <c r="A309" s="0" t="inlineStr">
         <is>
-          <t>SAMIRA</t>
+          <t>FANNE</t>
         </is>
       </c>
       <c r="B309" s="0" t="inlineStr">
         <is>
-          <t>SHIRA</t>
+          <t>SHARIF</t>
         </is>
       </c>
       <c r="R309" s="0" t="inlineStr">
@@ -10711,7 +10706,7 @@
       </c>
       <c r="X309" s="0" t="inlineStr">
         <is>
-          <t>156000.00</t>
+          <t>350000.00</t>
         </is>
       </c>
       <c r="Z309" s="0" t="inlineStr">
@@ -10726,19 +10721,19 @@
       </c>
       <c r="AC309" s="0" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>179</t>
         </is>
       </c>
     </row>
     <row r="310" spans="1:29">
       <c r="A310" s="0" t="inlineStr">
         <is>
-          <t>FATIMA </t>
+          <t>SAMIRA</t>
         </is>
       </c>
       <c r="B310" s="0" t="inlineStr">
         <is>
-          <t>SIDI</t>
+          <t>SHIRA</t>
         </is>
       </c>
       <c r="R310" s="0" t="inlineStr">
@@ -10748,7 +10743,7 @@
       </c>
       <c r="X310" s="0" t="inlineStr">
         <is>
-          <t>40000.00</t>
+          <t>156000.00</t>
         </is>
       </c>
       <c r="Z310" s="0" t="inlineStr">
@@ -10763,19 +10758,19 @@
       </c>
       <c r="AC310" s="0" t="inlineStr">
         <is>
-          <t>313</t>
+          <t>98</t>
         </is>
       </c>
     </row>
     <row r="311" spans="1:29">
       <c r="A311" s="0" t="inlineStr">
         <is>
-          <t>HADIZA</t>
+          <t>FATIMA </t>
         </is>
       </c>
       <c r="B311" s="0" t="inlineStr">
         <is>
-          <t>SOKOTO</t>
+          <t>SIDI</t>
         </is>
       </c>
       <c r="R311" s="0" t="inlineStr">
@@ -10785,7 +10780,7 @@
       </c>
       <c r="X311" s="0" t="inlineStr">
         <is>
-          <t>852500.00</t>
+          <t>40000.00</t>
         </is>
       </c>
       <c r="Z311" s="0" t="inlineStr">
@@ -10800,19 +10795,19 @@
       </c>
       <c r="AC311" s="0" t="inlineStr">
         <is>
-          <t>118</t>
+          <t>313</t>
         </is>
       </c>
     </row>
     <row r="312" spans="1:29">
       <c r="A312" s="0" t="inlineStr">
         <is>
-          <t>FARIDA</t>
+          <t>HADIZA</t>
         </is>
       </c>
       <c r="B312" s="0" t="inlineStr">
         <is>
-          <t>SULAIMAN</t>
+          <t>SOKOTO</t>
         </is>
       </c>
       <c r="R312" s="0" t="inlineStr">
@@ -10822,7 +10817,7 @@
       </c>
       <c r="X312" s="0" t="inlineStr">
         <is>
-          <t>99500.00</t>
+          <t>852500.00</t>
         </is>
       </c>
       <c r="Z312" s="0" t="inlineStr">
@@ -10837,19 +10832,19 @@
       </c>
       <c r="AC312" s="0" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>118</t>
         </is>
       </c>
     </row>
     <row r="313" spans="1:29">
       <c r="A313" s="0" t="inlineStr">
         <is>
-          <t>MARYAM</t>
+          <t>FARIDA</t>
         </is>
       </c>
       <c r="B313" s="0" t="inlineStr">
         <is>
-          <t>TRENDY</t>
+          <t>SULAIMAN</t>
         </is>
       </c>
       <c r="R313" s="0" t="inlineStr">
@@ -10859,7 +10854,7 @@
       </c>
       <c r="X313" s="0" t="inlineStr">
         <is>
-          <t>110500.00</t>
+          <t>99500.00</t>
         </is>
       </c>
       <c r="Z313" s="0" t="inlineStr">
@@ -10874,19 +10869,19 @@
       </c>
       <c r="AC313" s="0" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>246</t>
         </is>
       </c>
     </row>
     <row r="314" spans="1:29">
       <c r="A314" s="0" t="inlineStr">
         <is>
-          <t>JAMILA</t>
+          <t>MARYAM</t>
         </is>
       </c>
       <c r="B314" s="0" t="inlineStr">
         <is>
-          <t>TUKUR</t>
+          <t>TRENDY</t>
         </is>
       </c>
       <c r="R314" s="0" t="inlineStr">
@@ -10896,7 +10891,7 @@
       </c>
       <c r="X314" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>110500.00</t>
         </is>
       </c>
       <c r="Z314" s="0" t="inlineStr">
@@ -10911,19 +10906,19 @@
       </c>
       <c r="AC314" s="0" t="inlineStr">
         <is>
-          <t>251</t>
+          <t>180</t>
         </is>
       </c>
     </row>
     <row r="315" spans="1:29">
       <c r="A315" s="0" t="inlineStr">
         <is>
-          <t>FATIMA</t>
+          <t>JAMILA</t>
         </is>
       </c>
       <c r="B315" s="0" t="inlineStr">
         <is>
-          <t>TURARE</t>
+          <t>TUKUR</t>
         </is>
       </c>
       <c r="R315" s="0" t="inlineStr">
@@ -10933,7 +10928,7 @@
       </c>
       <c r="X315" s="0" t="inlineStr">
         <is>
-          <t>21000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z315" s="0" t="inlineStr">
@@ -10948,19 +10943,19 @@
       </c>
       <c r="AC315" s="0" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>251</t>
         </is>
       </c>
     </row>
     <row r="316" spans="1:29">
       <c r="A316" s="0" t="inlineStr">
         <is>
-          <t>ZAINAB</t>
+          <t>FATIMA</t>
         </is>
       </c>
       <c r="B316" s="0" t="inlineStr">
         <is>
-          <t>UMAR</t>
+          <t>TURARE</t>
         </is>
       </c>
       <c r="R316" s="0" t="inlineStr">
@@ -10970,7 +10965,7 @@
       </c>
       <c r="X316" s="0" t="inlineStr">
         <is>
-          <t>65000.00</t>
+          <t>21000.00</t>
         </is>
       </c>
       <c r="Z316" s="0" t="inlineStr">
@@ -10985,7 +10980,7 @@
       </c>
       <c r="AC316" s="0" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>153</t>
         </is>
       </c>
     </row>
@@ -10997,7 +10992,7 @@
       </c>
       <c r="B317" s="0" t="inlineStr">
         <is>
-          <t>USMAN</t>
+          <t>UMAR</t>
         </is>
       </c>
       <c r="R317" s="0" t="inlineStr">
@@ -11007,7 +11002,7 @@
       </c>
       <c r="X317" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>65000.00</t>
         </is>
       </c>
       <c r="Z317" s="0" t="inlineStr">
@@ -11022,19 +11017,19 @@
       </c>
       <c r="AC317" s="0" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>203</t>
         </is>
       </c>
     </row>
     <row r="318" spans="1:29">
       <c r="A318" s="0" t="inlineStr">
         <is>
-          <t>HAJ SADIYA</t>
+          <t>ZAINAB</t>
         </is>
       </c>
       <c r="B318" s="0" t="inlineStr">
         <is>
-          <t>WAILO</t>
+          <t>USMAN</t>
         </is>
       </c>
       <c r="R318" s="0" t="inlineStr">
@@ -11059,19 +11054,19 @@
       </c>
       <c r="AC318" s="0" t="inlineStr">
         <is>
-          <t>259</t>
+          <t>152</t>
         </is>
       </c>
     </row>
     <row r="319" spans="1:29">
       <c r="A319" s="0" t="inlineStr">
         <is>
-          <t>SALIHU</t>
+          <t>HAJ SADIYA</t>
         </is>
       </c>
       <c r="B319" s="0" t="inlineStr">
         <is>
-          <t>YABATEX</t>
+          <t>WAILO</t>
         </is>
       </c>
       <c r="R319" s="0" t="inlineStr">
@@ -11081,7 +11076,7 @@
       </c>
       <c r="X319" s="0" t="inlineStr">
         <is>
-          <t>681000.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z319" s="0" t="inlineStr">
@@ -11096,19 +11091,19 @@
       </c>
       <c r="AC319" s="0" t="inlineStr">
         <is>
-          <t>258</t>
+          <t>259</t>
         </is>
       </c>
     </row>
     <row r="320" spans="1:29">
       <c r="A320" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>SALIHU</t>
         </is>
       </c>
       <c r="B320" s="0" t="inlineStr">
         <is>
-          <t>YAN BIYU</t>
+          <t>YABATEX</t>
         </is>
       </c>
       <c r="R320" s="0" t="inlineStr">
@@ -11118,7 +11113,7 @@
       </c>
       <c r="X320" s="0" t="inlineStr">
         <is>
-          <t>2501200.00</t>
+          <t>681000.00</t>
         </is>
       </c>
       <c r="Z320" s="0" t="inlineStr">
@@ -11133,19 +11128,19 @@
       </c>
       <c r="AC320" s="0" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>258</t>
         </is>
       </c>
     </row>
     <row r="321" spans="1:29">
       <c r="A321" s="0" t="inlineStr">
         <is>
-          <t>ZULAIHA</t>
+          <t>MAMAN</t>
         </is>
       </c>
       <c r="B321" s="0" t="inlineStr">
         <is>
-          <t>YOLA</t>
+          <t>YAN BIYU</t>
         </is>
       </c>
       <c r="R321" s="0" t="inlineStr">
@@ -11155,7 +11150,7 @@
       </c>
       <c r="X321" s="0" t="inlineStr">
         <is>
-          <t>392000.00</t>
+          <t>2501200.00</t>
         </is>
       </c>
       <c r="Z321" s="0" t="inlineStr">
@@ -11170,14 +11165,14 @@
       </c>
       <c r="AC321" s="0" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>121</t>
         </is>
       </c>
     </row>
     <row r="322" spans="1:29">
       <c r="A322" s="0" t="inlineStr">
         <is>
-          <t>FAUZIYYA</t>
+          <t>ZULAIHA</t>
         </is>
       </c>
       <c r="B322" s="0" t="inlineStr">
@@ -11192,7 +11187,7 @@
       </c>
       <c r="X322" s="0" t="inlineStr">
         <is>
-          <t>17000.00</t>
+          <t>392000.00</t>
         </is>
       </c>
       <c r="Z322" s="0" t="inlineStr">
@@ -11207,19 +11202,19 @@
       </c>
       <c r="AC322" s="0" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>110</t>
         </is>
       </c>
     </row>
     <row r="323" spans="1:29">
       <c r="A323" s="0" t="inlineStr">
         <is>
-          <t>HAJ RUKAYYA</t>
+          <t>FAUZIYYA</t>
         </is>
       </c>
       <c r="B323" s="0" t="inlineStr">
         <is>
-          <t>YUSUF</t>
+          <t>YOLA</t>
         </is>
       </c>
       <c r="R323" s="0" t="inlineStr">
@@ -11229,7 +11224,7 @@
       </c>
       <c r="X323" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>17000.00</t>
         </is>
       </c>
       <c r="Z323" s="0" t="inlineStr">
@@ -11244,19 +11239,19 @@
       </c>
       <c r="AC323" s="0" t="inlineStr">
         <is>
-          <t>248</t>
+          <t>229</t>
         </is>
       </c>
     </row>
     <row r="324" spans="1:29">
       <c r="A324" s="0" t="inlineStr">
         <is>
-          <t>MAMAN</t>
+          <t>HAJ RUKAYYA</t>
         </is>
       </c>
       <c r="B324" s="0" t="inlineStr">
         <is>
-          <t>ZAHRA ONLINE</t>
+          <t>YUSUF</t>
         </is>
       </c>
       <c r="R324" s="0" t="inlineStr">
@@ -11266,7 +11261,7 @@
       </c>
       <c r="X324" s="0" t="inlineStr">
         <is>
-          <t>406500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z324" s="0" t="inlineStr">
@@ -11281,42 +11276,79 @@
       </c>
       <c r="AC324" s="0" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>248</t>
         </is>
       </c>
     </row>
     <row r="325" spans="1:29">
       <c r="A325" s="0" t="inlineStr">
         <is>
+          <t>MAMAN</t>
+        </is>
+      </c>
+      <c r="B325" s="0" t="inlineStr">
+        <is>
+          <t>ZAHRA ONLINE</t>
+        </is>
+      </c>
+      <c r="R325" s="0" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="X325" s="0" t="inlineStr">
+        <is>
+          <t>406500.00</t>
+        </is>
+      </c>
+      <c r="Z325" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA325" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AC325" s="0" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+    </row>
+    <row r="326" spans="1:29">
+      <c r="A326" s="0" t="inlineStr">
+        <is>
           <t>FATIMA</t>
         </is>
       </c>
-      <c r="B325" s="0" t="inlineStr">
+      <c r="B326" s="0" t="inlineStr">
         <is>
           <t>ZARAMI</t>
         </is>
       </c>
-      <c r="R325" s="0" t="inlineStr">
-        <is>
-          <t>y</t>
-        </is>
-      </c>
-      <c r="X325" s="0" t="inlineStr">
+      <c r="R326" s="0" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="X326" s="0" t="inlineStr">
         <is>
           <t>768300.00</t>
         </is>
       </c>
-      <c r="Z325" s="0" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="AA325" s="0" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="AC325" s="0" t="inlineStr">
+      <c r="Z326" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AA326" s="0" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="AC326" s="0" t="inlineStr">
         <is>
           <t>97</t>
         </is>

</xml_diff>